<commit_message>
BOM workbook: store formula results so totals show in any viewer; tools in tools/bom/
The workbook saved by openpyxl held formulas without cached results, so
previews and viewers that do not recalculate showed empty totals.
tools/bom/book.py now writes each formula's value next to it (line totals,
group totals, the Summary), and --check fails if the stored values are stale.
The BOM tools move to tools/bom/ (book.py, summary.py).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bom/bom.xlsx
+++ b/bom/bom.xlsx
@@ -42,8 +42,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
   <fonts count="5">
@@ -103,24 +103,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -507,7 +511,7 @@
     <row r="2" ht="48" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>This workbook is the BOM's source of truth; copy it to track your own build. Set each line's status to to buy, ordered or owned and the totals follow. After editing, run python tools/bom_book.py to tidy it. Prices are indicative: see each line's price basis and the Sourcing sheet.</t>
+          <t>This workbook is the BOM's source of truth; copy it to track your own build. Set each line's status to to buy, ordered or owned and the totals follow. After editing, run python tools/bom/book.py to tidy it. Prices are indicative: see each line's price basis and the Sourcing sheet.</t>
         </is>
       </c>
     </row>
@@ -551,23 +555,23 @@
       </c>
       <c r="B5">
         <f>COUNTA('Actuators'!A2:A14)</f>
-        <v/>
-      </c>
-      <c r="C5" s="4">
+        <v>13</v>
+      </c>
+      <c r="C5" s="13">
         <f>'Actuators'!I16</f>
-        <v/>
-      </c>
-      <c r="D5" s="4">
+        <v>6200.98</v>
+      </c>
+      <c r="D5" s="13">
         <f>SUMIFS('Actuators'!$I$2:$I$14,'Actuators'!$E$2:$E$14,"owned")</f>
-        <v/>
-      </c>
-      <c r="E5" s="4">
+        <v>0</v>
+      </c>
+      <c r="E5" s="13">
         <f>SUMIFS('Actuators'!$I$2:$I$14,'Actuators'!$E$2:$E$14,"ordered")</f>
-        <v/>
-      </c>
-      <c r="F5" s="4">
+        <v>0</v>
+      </c>
+      <c r="F5" s="13">
         <f>SUMIFS('Actuators'!$I$2:$I$14,'Actuators'!$E$2:$E$14,"to buy")</f>
-        <v/>
+        <v>6200.98</v>
       </c>
     </row>
     <row r="6">
@@ -578,23 +582,23 @@
       </c>
       <c r="B6">
         <f>COUNTA('Hands'!A2:A4)</f>
-        <v/>
-      </c>
-      <c r="C6" s="4">
+        <v>3</v>
+      </c>
+      <c r="C6" s="13">
         <f>'Hands'!I6</f>
-        <v/>
-      </c>
-      <c r="D6" s="4">
+        <v>224</v>
+      </c>
+      <c r="D6" s="13">
         <f>SUMIFS('Hands'!$I$2:$I$4,'Hands'!$E$2:$E$4,"owned")</f>
-        <v/>
-      </c>
-      <c r="E6" s="4">
+        <v>198</v>
+      </c>
+      <c r="E6" s="13">
         <f>SUMIFS('Hands'!$I$2:$I$4,'Hands'!$E$2:$E$4,"ordered")</f>
-        <v/>
-      </c>
-      <c r="F6" s="4">
+        <v>0</v>
+      </c>
+      <c r="F6" s="13">
         <f>SUMIFS('Hands'!$I$2:$I$4,'Hands'!$E$2:$E$4,"to buy")</f>
-        <v/>
+        <v>26</v>
       </c>
     </row>
     <row r="7">
@@ -605,23 +609,23 @@
       </c>
       <c r="B7">
         <f>COUNTA('Compute &amp; sensors'!A2:A6)</f>
-        <v/>
-      </c>
-      <c r="C7" s="4">
+        <v>5</v>
+      </c>
+      <c r="C7" s="13">
         <f>'Compute &amp; sensors'!I8</f>
-        <v/>
-      </c>
-      <c r="D7" s="4">
+        <v>4723</v>
+      </c>
+      <c r="D7" s="13">
         <f>SUMIFS('Compute &amp; sensors'!$I$2:$I$6,'Compute &amp; sensors'!$E$2:$E$6,"owned")</f>
-        <v/>
-      </c>
-      <c r="E7" s="4">
+        <v>3534</v>
+      </c>
+      <c r="E7" s="13">
         <f>SUMIFS('Compute &amp; sensors'!$I$2:$I$6,'Compute &amp; sensors'!$E$2:$E$6,"ordered")</f>
-        <v/>
-      </c>
-      <c r="F7" s="4">
+        <v>0</v>
+      </c>
+      <c r="F7" s="13">
         <f>SUMIFS('Compute &amp; sensors'!$I$2:$I$6,'Compute &amp; sensors'!$E$2:$E$6,"to buy")</f>
-        <v/>
+        <v>1189</v>
       </c>
     </row>
     <row r="8">
@@ -632,23 +636,23 @@
       </c>
       <c r="B8">
         <f>COUNTA('Power'!A2:A15)</f>
-        <v/>
-      </c>
-      <c r="C8" s="4">
+        <v>14</v>
+      </c>
+      <c r="C8" s="13">
         <f>'Power'!I17</f>
-        <v/>
-      </c>
-      <c r="D8" s="4">
+        <v>1633.05</v>
+      </c>
+      <c r="D8" s="13">
         <f>SUMIFS('Power'!$I$2:$I$15,'Power'!$E$2:$E$15,"owned")</f>
-        <v/>
-      </c>
-      <c r="E8" s="4">
+        <v>0</v>
+      </c>
+      <c r="E8" s="13">
         <f>SUMIFS('Power'!$I$2:$I$15,'Power'!$E$2:$E$15,"ordered")</f>
-        <v/>
-      </c>
-      <c r="F8" s="4">
+        <v>0</v>
+      </c>
+      <c r="F8" s="13">
         <f>SUMIFS('Power'!$I$2:$I$15,'Power'!$E$2:$E$15,"to buy")</f>
-        <v/>
+        <v>1633.05</v>
       </c>
     </row>
     <row r="9">
@@ -659,23 +663,23 @@
       </c>
       <c r="B9">
         <f>COUNTA('Electronics &amp; wiring'!A2:A12)</f>
-        <v/>
-      </c>
-      <c r="C9" s="4">
+        <v>11</v>
+      </c>
+      <c r="C9" s="13">
         <f>'Electronics &amp; wiring'!I14</f>
-        <v/>
-      </c>
-      <c r="D9" s="4">
+        <v>808</v>
+      </c>
+      <c r="D9" s="13">
         <f>SUMIFS('Electronics &amp; wiring'!$I$2:$I$12,'Electronics &amp; wiring'!$E$2:$E$12,"owned")</f>
-        <v/>
-      </c>
-      <c r="E9" s="4">
+        <v>0</v>
+      </c>
+      <c r="E9" s="13">
         <f>SUMIFS('Electronics &amp; wiring'!$I$2:$I$12,'Electronics &amp; wiring'!$E$2:$E$12,"ordered")</f>
-        <v/>
-      </c>
-      <c r="F9" s="4">
+        <v>0</v>
+      </c>
+      <c r="F9" s="13">
         <f>SUMIFS('Electronics &amp; wiring'!$I$2:$I$12,'Electronics &amp; wiring'!$E$2:$E$12,"to buy")</f>
-        <v/>
+        <v>808</v>
       </c>
     </row>
     <row r="10">
@@ -686,23 +690,23 @@
       </c>
       <c r="B10">
         <f>COUNTA('Structure &amp; materials'!A2:A14)</f>
-        <v/>
-      </c>
-      <c r="C10" s="4">
+        <v>13</v>
+      </c>
+      <c r="C10" s="13">
         <f>'Structure &amp; materials'!I16</f>
-        <v/>
-      </c>
-      <c r="D10" s="4">
+        <v>2582</v>
+      </c>
+      <c r="D10" s="13">
         <f>SUMIFS('Structure &amp; materials'!$I$2:$I$14,'Structure &amp; materials'!$E$2:$E$14,"owned")</f>
-        <v/>
-      </c>
-      <c r="E10" s="4">
+        <v>0</v>
+      </c>
+      <c r="E10" s="13">
         <f>SUMIFS('Structure &amp; materials'!$I$2:$I$14,'Structure &amp; materials'!$E$2:$E$14,"ordered")</f>
-        <v/>
-      </c>
-      <c r="F10" s="4">
+        <v>0</v>
+      </c>
+      <c r="F10" s="13">
         <f>SUMIFS('Structure &amp; materials'!$I$2:$I$14,'Structure &amp; materials'!$E$2:$E$14,"to buy")</f>
-        <v/>
+        <v>2582</v>
       </c>
     </row>
     <row r="11">
@@ -713,23 +717,23 @@
       </c>
       <c r="B11">
         <f>COUNTA('Fasteners'!A2:A2)</f>
-        <v/>
-      </c>
-      <c r="C11" s="4">
+        <v>1</v>
+      </c>
+      <c r="C11" s="13">
         <f>'Fasteners'!I4</f>
-        <v/>
-      </c>
-      <c r="D11" s="4">
+        <v>180</v>
+      </c>
+      <c r="D11" s="13">
         <f>SUMIFS('Fasteners'!$I$2:$I$2,'Fasteners'!$E$2:$E$2,"owned")</f>
-        <v/>
-      </c>
-      <c r="E11" s="4">
+        <v>0</v>
+      </c>
+      <c r="E11" s="13">
         <f>SUMIFS('Fasteners'!$I$2:$I$2,'Fasteners'!$E$2:$E$2,"ordered")</f>
-        <v/>
-      </c>
-      <c r="F11" s="4">
+        <v>0</v>
+      </c>
+      <c r="F11" s="13">
         <f>SUMIFS('Fasteners'!$I$2:$I$2,'Fasteners'!$E$2:$E$2,"to buy")</f>
-        <v/>
+        <v>180</v>
       </c>
     </row>
     <row r="12">
@@ -740,23 +744,23 @@
       </c>
       <c r="B12">
         <f>COUNTA('Tooling'!A2:A6)</f>
-        <v/>
-      </c>
-      <c r="C12" s="4">
+        <v>5</v>
+      </c>
+      <c r="C12" s="13">
         <f>'Tooling'!I8</f>
-        <v/>
-      </c>
-      <c r="D12" s="4">
+        <v>710</v>
+      </c>
+      <c r="D12" s="13">
         <f>SUMIFS('Tooling'!$I$2:$I$6,'Tooling'!$E$2:$E$6,"owned")</f>
-        <v/>
-      </c>
-      <c r="E12" s="4">
+        <v>0</v>
+      </c>
+      <c r="E12" s="13">
         <f>SUMIFS('Tooling'!$I$2:$I$6,'Tooling'!$E$2:$E$6,"ordered")</f>
-        <v/>
-      </c>
-      <c r="F12" s="4">
+        <v>0</v>
+      </c>
+      <c r="F12" s="13">
         <f>SUMIFS('Tooling'!$I$2:$I$6,'Tooling'!$E$2:$E$6,"to buy")</f>
-        <v/>
+        <v>710</v>
       </c>
     </row>
     <row r="13">
@@ -767,23 +771,23 @@
       </c>
       <c r="B13">
         <f>COUNTA('Safety'!A2:A5)</f>
-        <v/>
-      </c>
-      <c r="C13" s="4">
+        <v>4</v>
+      </c>
+      <c r="C13" s="13">
         <f>'Safety'!I7</f>
-        <v/>
-      </c>
-      <c r="D13" s="4">
+        <v>470</v>
+      </c>
+      <c r="D13" s="13">
         <f>SUMIFS('Safety'!$I$2:$I$5,'Safety'!$E$2:$E$5,"owned")</f>
-        <v/>
-      </c>
-      <c r="E13" s="4">
+        <v>0</v>
+      </c>
+      <c r="E13" s="13">
         <f>SUMIFS('Safety'!$I$2:$I$5,'Safety'!$E$2:$E$5,"ordered")</f>
-        <v/>
-      </c>
-      <c r="F13" s="4">
+        <v>0</v>
+      </c>
+      <c r="F13" s="13">
         <f>SUMIFS('Safety'!$I$2:$I$5,'Safety'!$E$2:$E$5,"to buy")</f>
-        <v/>
+        <v>470</v>
       </c>
     </row>
     <row r="14">
@@ -794,30 +798,30 @@
       </c>
       <c r="B14" s="5">
         <f>SUM(B5:B13)</f>
-        <v/>
-      </c>
-      <c r="C14" s="6">
+        <v>69</v>
+      </c>
+      <c r="C14" s="14">
         <f>SUM(C5:C13)</f>
-        <v/>
-      </c>
-      <c r="D14" s="6">
+        <v>17531.03</v>
+      </c>
+      <c r="D14" s="14">
         <f>SUM(D5:D13)</f>
-        <v/>
-      </c>
-      <c r="E14" s="6">
+        <v>3732</v>
+      </c>
+      <c r="E14" s="14">
         <f>SUM(E5:E13)</f>
-        <v/>
-      </c>
-      <c r="F14" s="6">
+        <v>0</v>
+      </c>
+      <c r="F14" s="14">
         <f>SUM(F5:F13)</f>
-        <v/>
+        <v>13799.03</v>
       </c>
     </row>
     <row r="15">
-      <c r="C15" s="4" t="n"/>
-      <c r="D15" s="4" t="n"/>
-      <c r="E15" s="4" t="n"/>
-      <c r="F15" s="4" t="n"/>
+      <c r="C15" s="13" t="n"/>
+      <c r="D15" s="13" t="n"/>
+      <c r="E15" s="13" t="n"/>
+      <c r="F15" s="13" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -826,22 +830,22 @@
         </is>
       </c>
       <c r="B16" s="3" t="n"/>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C16" s="15" t="inlineStr">
         <is>
           <t>Total USD</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D16" s="15" t="inlineStr">
         <is>
           <t>Owned USD</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E16" s="15" t="inlineStr">
         <is>
           <t>Ordered USD</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
+      <c r="F16" s="15" t="inlineStr">
         <is>
           <t>To buy USD</t>
         </is>
@@ -853,21 +857,21 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="C17" s="4">
+      <c r="C17" s="13">
         <f>SUMIFS('Actuators'!$I$2:$I$14,'Actuators'!$D$2:$D$14,"P2")+SUMIFS('Hands'!$I$2:$I$4,'Hands'!$D$2:$D$4,"P2")+SUMIFS('Compute &amp; sensors'!$I$2:$I$6,'Compute &amp; sensors'!$D$2:$D$6,"P2")+SUMIFS('Power'!$I$2:$I$15,'Power'!$D$2:$D$15,"P2")+SUMIFS('Electronics &amp; wiring'!$I$2:$I$12,'Electronics &amp; wiring'!$D$2:$D$12,"P2")+SUMIFS('Structure &amp; materials'!$I$2:$I$14,'Structure &amp; materials'!$D$2:$D$14,"P2")+SUMIFS('Fasteners'!$I$2:$I$2,'Fasteners'!$D$2:$D$2,"P2")+SUMIFS('Tooling'!$I$2:$I$6,'Tooling'!$D$2:$D$6,"P2")+SUMIFS('Safety'!$I$2:$I$5,'Safety'!$D$2:$D$5,"P2")</f>
-        <v/>
-      </c>
-      <c r="D17" s="4">
+        <v>1030</v>
+      </c>
+      <c r="D17" s="13">
         <f>SUMIFS('Actuators'!$I$2:$I$14,'Actuators'!$D$2:$D$14,"P2",'Actuators'!$E$2:$E$14,"owned")+SUMIFS('Hands'!$I$2:$I$4,'Hands'!$D$2:$D$4,"P2",'Hands'!$E$2:$E$4,"owned")+SUMIFS('Compute &amp; sensors'!$I$2:$I$6,'Compute &amp; sensors'!$D$2:$D$6,"P2",'Compute &amp; sensors'!$E$2:$E$6,"owned")+SUMIFS('Power'!$I$2:$I$15,'Power'!$D$2:$D$15,"P2",'Power'!$E$2:$E$15,"owned")+SUMIFS('Electronics &amp; wiring'!$I$2:$I$12,'Electronics &amp; wiring'!$D$2:$D$12,"P2",'Electronics &amp; wiring'!$E$2:$E$12,"owned")+SUMIFS('Structure &amp; materials'!$I$2:$I$14,'Structure &amp; materials'!$D$2:$D$14,"P2",'Structure &amp; materials'!$E$2:$E$14,"owned")+SUMIFS('Fasteners'!$I$2:$I$2,'Fasteners'!$D$2:$D$2,"P2",'Fasteners'!$E$2:$E$2,"owned")+SUMIFS('Tooling'!$I$2:$I$6,'Tooling'!$D$2:$D$6,"P2",'Tooling'!$E$2:$E$6,"owned")+SUMIFS('Safety'!$I$2:$I$5,'Safety'!$D$2:$D$5,"P2",'Safety'!$E$2:$E$5,"owned")</f>
-        <v/>
-      </c>
-      <c r="E17" s="4">
+        <v>35</v>
+      </c>
+      <c r="E17" s="13">
         <f>SUMIFS('Actuators'!$I$2:$I$14,'Actuators'!$D$2:$D$14,"P2",'Actuators'!$E$2:$E$14,"ordered")+SUMIFS('Hands'!$I$2:$I$4,'Hands'!$D$2:$D$4,"P2",'Hands'!$E$2:$E$4,"ordered")+SUMIFS('Compute &amp; sensors'!$I$2:$I$6,'Compute &amp; sensors'!$D$2:$D$6,"P2",'Compute &amp; sensors'!$E$2:$E$6,"ordered")+SUMIFS('Power'!$I$2:$I$15,'Power'!$D$2:$D$15,"P2",'Power'!$E$2:$E$15,"ordered")+SUMIFS('Electronics &amp; wiring'!$I$2:$I$12,'Electronics &amp; wiring'!$D$2:$D$12,"P2",'Electronics &amp; wiring'!$E$2:$E$12,"ordered")+SUMIFS('Structure &amp; materials'!$I$2:$I$14,'Structure &amp; materials'!$D$2:$D$14,"P2",'Structure &amp; materials'!$E$2:$E$14,"ordered")+SUMIFS('Fasteners'!$I$2:$I$2,'Fasteners'!$D$2:$D$2,"P2",'Fasteners'!$E$2:$E$2,"ordered")+SUMIFS('Tooling'!$I$2:$I$6,'Tooling'!$D$2:$D$6,"P2",'Tooling'!$E$2:$E$6,"ordered")+SUMIFS('Safety'!$I$2:$I$5,'Safety'!$D$2:$D$5,"P2",'Safety'!$E$2:$E$5,"ordered")</f>
-        <v/>
-      </c>
-      <c r="F17" s="4">
+        <v>0</v>
+      </c>
+      <c r="F17" s="13">
         <f>SUMIFS('Actuators'!$I$2:$I$14,'Actuators'!$D$2:$D$14,"P2",'Actuators'!$E$2:$E$14,"to buy")+SUMIFS('Hands'!$I$2:$I$4,'Hands'!$D$2:$D$4,"P2",'Hands'!$E$2:$E$4,"to buy")+SUMIFS('Compute &amp; sensors'!$I$2:$I$6,'Compute &amp; sensors'!$D$2:$D$6,"P2",'Compute &amp; sensors'!$E$2:$E$6,"to buy")+SUMIFS('Power'!$I$2:$I$15,'Power'!$D$2:$D$15,"P2",'Power'!$E$2:$E$15,"to buy")+SUMIFS('Electronics &amp; wiring'!$I$2:$I$12,'Electronics &amp; wiring'!$D$2:$D$12,"P2",'Electronics &amp; wiring'!$E$2:$E$12,"to buy")+SUMIFS('Structure &amp; materials'!$I$2:$I$14,'Structure &amp; materials'!$D$2:$D$14,"P2",'Structure &amp; materials'!$E$2:$E$14,"to buy")+SUMIFS('Fasteners'!$I$2:$I$2,'Fasteners'!$D$2:$D$2,"P2",'Fasteners'!$E$2:$E$2,"to buy")+SUMIFS('Tooling'!$I$2:$I$6,'Tooling'!$D$2:$D$6,"P2",'Tooling'!$E$2:$E$6,"to buy")+SUMIFS('Safety'!$I$2:$I$5,'Safety'!$D$2:$D$5,"P2",'Safety'!$E$2:$E$5,"to buy")</f>
-        <v/>
+        <v>995</v>
       </c>
     </row>
     <row r="18">
@@ -876,21 +880,21 @@
           <t>P3</t>
         </is>
       </c>
-      <c r="C18" s="4">
+      <c r="C18" s="13">
         <f>SUMIFS('Actuators'!$I$2:$I$14,'Actuators'!$D$2:$D$14,"P3")+SUMIFS('Hands'!$I$2:$I$4,'Hands'!$D$2:$D$4,"P3")+SUMIFS('Compute &amp; sensors'!$I$2:$I$6,'Compute &amp; sensors'!$D$2:$D$6,"P3")+SUMIFS('Power'!$I$2:$I$15,'Power'!$D$2:$D$15,"P3")+SUMIFS('Electronics &amp; wiring'!$I$2:$I$12,'Electronics &amp; wiring'!$D$2:$D$12,"P3")+SUMIFS('Structure &amp; materials'!$I$2:$I$14,'Structure &amp; materials'!$D$2:$D$14,"P3")+SUMIFS('Fasteners'!$I$2:$I$2,'Fasteners'!$D$2:$D$2,"P3")+SUMIFS('Tooling'!$I$2:$I$6,'Tooling'!$D$2:$D$6,"P3")+SUMIFS('Safety'!$I$2:$I$5,'Safety'!$D$2:$D$5,"P3")</f>
-        <v/>
-      </c>
-      <c r="D18" s="4">
+        <v>3202</v>
+      </c>
+      <c r="D18" s="13">
         <f>SUMIFS('Actuators'!$I$2:$I$14,'Actuators'!$D$2:$D$14,"P3",'Actuators'!$E$2:$E$14,"owned")+SUMIFS('Hands'!$I$2:$I$4,'Hands'!$D$2:$D$4,"P3",'Hands'!$E$2:$E$4,"owned")+SUMIFS('Compute &amp; sensors'!$I$2:$I$6,'Compute &amp; sensors'!$D$2:$D$6,"P3",'Compute &amp; sensors'!$E$2:$E$6,"owned")+SUMIFS('Power'!$I$2:$I$15,'Power'!$D$2:$D$15,"P3",'Power'!$E$2:$E$15,"owned")+SUMIFS('Electronics &amp; wiring'!$I$2:$I$12,'Electronics &amp; wiring'!$D$2:$D$12,"P3",'Electronics &amp; wiring'!$E$2:$E$12,"owned")+SUMIFS('Structure &amp; materials'!$I$2:$I$14,'Structure &amp; materials'!$D$2:$D$14,"P3",'Structure &amp; materials'!$E$2:$E$14,"owned")+SUMIFS('Fasteners'!$I$2:$I$2,'Fasteners'!$D$2:$D$2,"P3",'Fasteners'!$E$2:$E$2,"owned")+SUMIFS('Tooling'!$I$2:$I$6,'Tooling'!$D$2:$D$6,"P3",'Tooling'!$E$2:$E$6,"owned")+SUMIFS('Safety'!$I$2:$I$5,'Safety'!$D$2:$D$5,"P3",'Safety'!$E$2:$E$5,"owned")</f>
-        <v/>
-      </c>
-      <c r="E18" s="4">
+        <v>0</v>
+      </c>
+      <c r="E18" s="13">
         <f>SUMIFS('Actuators'!$I$2:$I$14,'Actuators'!$D$2:$D$14,"P3",'Actuators'!$E$2:$E$14,"ordered")+SUMIFS('Hands'!$I$2:$I$4,'Hands'!$D$2:$D$4,"P3",'Hands'!$E$2:$E$4,"ordered")+SUMIFS('Compute &amp; sensors'!$I$2:$I$6,'Compute &amp; sensors'!$D$2:$D$6,"P3",'Compute &amp; sensors'!$E$2:$E$6,"ordered")+SUMIFS('Power'!$I$2:$I$15,'Power'!$D$2:$D$15,"P3",'Power'!$E$2:$E$15,"ordered")+SUMIFS('Electronics &amp; wiring'!$I$2:$I$12,'Electronics &amp; wiring'!$D$2:$D$12,"P3",'Electronics &amp; wiring'!$E$2:$E$12,"ordered")+SUMIFS('Structure &amp; materials'!$I$2:$I$14,'Structure &amp; materials'!$D$2:$D$14,"P3",'Structure &amp; materials'!$E$2:$E$14,"ordered")+SUMIFS('Fasteners'!$I$2:$I$2,'Fasteners'!$D$2:$D$2,"P3",'Fasteners'!$E$2:$E$2,"ordered")+SUMIFS('Tooling'!$I$2:$I$6,'Tooling'!$D$2:$D$6,"P3",'Tooling'!$E$2:$E$6,"ordered")+SUMIFS('Safety'!$I$2:$I$5,'Safety'!$D$2:$D$5,"P3",'Safety'!$E$2:$E$5,"ordered")</f>
-        <v/>
-      </c>
-      <c r="F18" s="4">
+        <v>0</v>
+      </c>
+      <c r="F18" s="13">
         <f>SUMIFS('Actuators'!$I$2:$I$14,'Actuators'!$D$2:$D$14,"P3",'Actuators'!$E$2:$E$14,"to buy")+SUMIFS('Hands'!$I$2:$I$4,'Hands'!$D$2:$D$4,"P3",'Hands'!$E$2:$E$4,"to buy")+SUMIFS('Compute &amp; sensors'!$I$2:$I$6,'Compute &amp; sensors'!$D$2:$D$6,"P3",'Compute &amp; sensors'!$E$2:$E$6,"to buy")+SUMIFS('Power'!$I$2:$I$15,'Power'!$D$2:$D$15,"P3",'Power'!$E$2:$E$15,"to buy")+SUMIFS('Electronics &amp; wiring'!$I$2:$I$12,'Electronics &amp; wiring'!$D$2:$D$12,"P3",'Electronics &amp; wiring'!$E$2:$E$12,"to buy")+SUMIFS('Structure &amp; materials'!$I$2:$I$14,'Structure &amp; materials'!$D$2:$D$14,"P3",'Structure &amp; materials'!$E$2:$E$14,"to buy")+SUMIFS('Fasteners'!$I$2:$I$2,'Fasteners'!$D$2:$D$2,"P3",'Fasteners'!$E$2:$E$2,"to buy")+SUMIFS('Tooling'!$I$2:$I$6,'Tooling'!$D$2:$D$6,"P3",'Tooling'!$E$2:$E$6,"to buy")+SUMIFS('Safety'!$I$2:$I$5,'Safety'!$D$2:$D$5,"P3",'Safety'!$E$2:$E$5,"to buy")</f>
-        <v/>
+        <v>3202</v>
       </c>
     </row>
     <row r="19">
@@ -899,21 +903,21 @@
           <t>P4</t>
         </is>
       </c>
-      <c r="C19" s="4">
+      <c r="C19" s="13">
         <f>SUMIFS('Actuators'!$I$2:$I$14,'Actuators'!$D$2:$D$14,"P4")+SUMIFS('Hands'!$I$2:$I$4,'Hands'!$D$2:$D$4,"P4")+SUMIFS('Compute &amp; sensors'!$I$2:$I$6,'Compute &amp; sensors'!$D$2:$D$6,"P4")+SUMIFS('Power'!$I$2:$I$15,'Power'!$D$2:$D$15,"P4")+SUMIFS('Electronics &amp; wiring'!$I$2:$I$12,'Electronics &amp; wiring'!$D$2:$D$12,"P4")+SUMIFS('Structure &amp; materials'!$I$2:$I$14,'Structure &amp; materials'!$D$2:$D$14,"P4")+SUMIFS('Fasteners'!$I$2:$I$2,'Fasteners'!$D$2:$D$2,"P4")+SUMIFS('Tooling'!$I$2:$I$6,'Tooling'!$D$2:$D$6,"P4")+SUMIFS('Safety'!$I$2:$I$5,'Safety'!$D$2:$D$5,"P4")</f>
-        <v/>
-      </c>
-      <c r="D19" s="4">
+        <v>9130.05</v>
+      </c>
+      <c r="D19" s="13">
         <f>SUMIFS('Actuators'!$I$2:$I$14,'Actuators'!$D$2:$D$14,"P4",'Actuators'!$E$2:$E$14,"owned")+SUMIFS('Hands'!$I$2:$I$4,'Hands'!$D$2:$D$4,"P4",'Hands'!$E$2:$E$4,"owned")+SUMIFS('Compute &amp; sensors'!$I$2:$I$6,'Compute &amp; sensors'!$D$2:$D$6,"P4",'Compute &amp; sensors'!$E$2:$E$6,"owned")+SUMIFS('Power'!$I$2:$I$15,'Power'!$D$2:$D$15,"P4",'Power'!$E$2:$E$15,"owned")+SUMIFS('Electronics &amp; wiring'!$I$2:$I$12,'Electronics &amp; wiring'!$D$2:$D$12,"P4",'Electronics &amp; wiring'!$E$2:$E$12,"owned")+SUMIFS('Structure &amp; materials'!$I$2:$I$14,'Structure &amp; materials'!$D$2:$D$14,"P4",'Structure &amp; materials'!$E$2:$E$14,"owned")+SUMIFS('Fasteners'!$I$2:$I$2,'Fasteners'!$D$2:$D$2,"P4",'Fasteners'!$E$2:$E$2,"owned")+SUMIFS('Tooling'!$I$2:$I$6,'Tooling'!$D$2:$D$6,"P4",'Tooling'!$E$2:$E$6,"owned")+SUMIFS('Safety'!$I$2:$I$5,'Safety'!$D$2:$D$5,"P4",'Safety'!$E$2:$E$5,"owned")</f>
-        <v/>
-      </c>
-      <c r="E19" s="4">
+        <v>3499</v>
+      </c>
+      <c r="E19" s="13">
         <f>SUMIFS('Actuators'!$I$2:$I$14,'Actuators'!$D$2:$D$14,"P4",'Actuators'!$E$2:$E$14,"ordered")+SUMIFS('Hands'!$I$2:$I$4,'Hands'!$D$2:$D$4,"P4",'Hands'!$E$2:$E$4,"ordered")+SUMIFS('Compute &amp; sensors'!$I$2:$I$6,'Compute &amp; sensors'!$D$2:$D$6,"P4",'Compute &amp; sensors'!$E$2:$E$6,"ordered")+SUMIFS('Power'!$I$2:$I$15,'Power'!$D$2:$D$15,"P4",'Power'!$E$2:$E$15,"ordered")+SUMIFS('Electronics &amp; wiring'!$I$2:$I$12,'Electronics &amp; wiring'!$D$2:$D$12,"P4",'Electronics &amp; wiring'!$E$2:$E$12,"ordered")+SUMIFS('Structure &amp; materials'!$I$2:$I$14,'Structure &amp; materials'!$D$2:$D$14,"P4",'Structure &amp; materials'!$E$2:$E$14,"ordered")+SUMIFS('Fasteners'!$I$2:$I$2,'Fasteners'!$D$2:$D$2,"P4",'Fasteners'!$E$2:$E$2,"ordered")+SUMIFS('Tooling'!$I$2:$I$6,'Tooling'!$D$2:$D$6,"P4",'Tooling'!$E$2:$E$6,"ordered")+SUMIFS('Safety'!$I$2:$I$5,'Safety'!$D$2:$D$5,"P4",'Safety'!$E$2:$E$5,"ordered")</f>
-        <v/>
-      </c>
-      <c r="F19" s="4">
+        <v>0</v>
+      </c>
+      <c r="F19" s="13">
         <f>SUMIFS('Actuators'!$I$2:$I$14,'Actuators'!$D$2:$D$14,"P4",'Actuators'!$E$2:$E$14,"to buy")+SUMIFS('Hands'!$I$2:$I$4,'Hands'!$D$2:$D$4,"P4",'Hands'!$E$2:$E$4,"to buy")+SUMIFS('Compute &amp; sensors'!$I$2:$I$6,'Compute &amp; sensors'!$D$2:$D$6,"P4",'Compute &amp; sensors'!$E$2:$E$6,"to buy")+SUMIFS('Power'!$I$2:$I$15,'Power'!$D$2:$D$15,"P4",'Power'!$E$2:$E$15,"to buy")+SUMIFS('Electronics &amp; wiring'!$I$2:$I$12,'Electronics &amp; wiring'!$D$2:$D$12,"P4",'Electronics &amp; wiring'!$E$2:$E$12,"to buy")+SUMIFS('Structure &amp; materials'!$I$2:$I$14,'Structure &amp; materials'!$D$2:$D$14,"P4",'Structure &amp; materials'!$E$2:$E$14,"to buy")+SUMIFS('Fasteners'!$I$2:$I$2,'Fasteners'!$D$2:$D$2,"P4",'Fasteners'!$E$2:$E$2,"to buy")+SUMIFS('Tooling'!$I$2:$I$6,'Tooling'!$D$2:$D$6,"P4",'Tooling'!$E$2:$E$6,"to buy")+SUMIFS('Safety'!$I$2:$I$5,'Safety'!$D$2:$D$5,"P4",'Safety'!$E$2:$E$5,"to buy")</f>
-        <v/>
+        <v>5631.05</v>
       </c>
     </row>
     <row r="20">
@@ -922,21 +926,21 @@
           <t>P5</t>
         </is>
       </c>
-      <c r="C20" s="4">
+      <c r="C20" s="13">
         <f>SUMIFS('Actuators'!$I$2:$I$14,'Actuators'!$D$2:$D$14,"P5")+SUMIFS('Hands'!$I$2:$I$4,'Hands'!$D$2:$D$4,"P5")+SUMIFS('Compute &amp; sensors'!$I$2:$I$6,'Compute &amp; sensors'!$D$2:$D$6,"P5")+SUMIFS('Power'!$I$2:$I$15,'Power'!$D$2:$D$15,"P5")+SUMIFS('Electronics &amp; wiring'!$I$2:$I$12,'Electronics &amp; wiring'!$D$2:$D$12,"P5")+SUMIFS('Structure &amp; materials'!$I$2:$I$14,'Structure &amp; materials'!$D$2:$D$14,"P5")+SUMIFS('Fasteners'!$I$2:$I$2,'Fasteners'!$D$2:$D$2,"P5")+SUMIFS('Tooling'!$I$2:$I$6,'Tooling'!$D$2:$D$6,"P5")+SUMIFS('Safety'!$I$2:$I$5,'Safety'!$D$2:$D$5,"P5")</f>
-        <v/>
-      </c>
-      <c r="D20" s="4">
+        <v>3809.98</v>
+      </c>
+      <c r="D20" s="13">
         <f>SUMIFS('Actuators'!$I$2:$I$14,'Actuators'!$D$2:$D$14,"P5",'Actuators'!$E$2:$E$14,"owned")+SUMIFS('Hands'!$I$2:$I$4,'Hands'!$D$2:$D$4,"P5",'Hands'!$E$2:$E$4,"owned")+SUMIFS('Compute &amp; sensors'!$I$2:$I$6,'Compute &amp; sensors'!$D$2:$D$6,"P5",'Compute &amp; sensors'!$E$2:$E$6,"owned")+SUMIFS('Power'!$I$2:$I$15,'Power'!$D$2:$D$15,"P5",'Power'!$E$2:$E$15,"owned")+SUMIFS('Electronics &amp; wiring'!$I$2:$I$12,'Electronics &amp; wiring'!$D$2:$D$12,"P5",'Electronics &amp; wiring'!$E$2:$E$12,"owned")+SUMIFS('Structure &amp; materials'!$I$2:$I$14,'Structure &amp; materials'!$D$2:$D$14,"P5",'Structure &amp; materials'!$E$2:$E$14,"owned")+SUMIFS('Fasteners'!$I$2:$I$2,'Fasteners'!$D$2:$D$2,"P5",'Fasteners'!$E$2:$E$2,"owned")+SUMIFS('Tooling'!$I$2:$I$6,'Tooling'!$D$2:$D$6,"P5",'Tooling'!$E$2:$E$6,"owned")+SUMIFS('Safety'!$I$2:$I$5,'Safety'!$D$2:$D$5,"P5",'Safety'!$E$2:$E$5,"owned")</f>
-        <v/>
-      </c>
-      <c r="E20" s="4">
+        <v>198</v>
+      </c>
+      <c r="E20" s="13">
         <f>SUMIFS('Actuators'!$I$2:$I$14,'Actuators'!$D$2:$D$14,"P5",'Actuators'!$E$2:$E$14,"ordered")+SUMIFS('Hands'!$I$2:$I$4,'Hands'!$D$2:$D$4,"P5",'Hands'!$E$2:$E$4,"ordered")+SUMIFS('Compute &amp; sensors'!$I$2:$I$6,'Compute &amp; sensors'!$D$2:$D$6,"P5",'Compute &amp; sensors'!$E$2:$E$6,"ordered")+SUMIFS('Power'!$I$2:$I$15,'Power'!$D$2:$D$15,"P5",'Power'!$E$2:$E$15,"ordered")+SUMIFS('Electronics &amp; wiring'!$I$2:$I$12,'Electronics &amp; wiring'!$D$2:$D$12,"P5",'Electronics &amp; wiring'!$E$2:$E$12,"ordered")+SUMIFS('Structure &amp; materials'!$I$2:$I$14,'Structure &amp; materials'!$D$2:$D$14,"P5",'Structure &amp; materials'!$E$2:$E$14,"ordered")+SUMIFS('Fasteners'!$I$2:$I$2,'Fasteners'!$D$2:$D$2,"P5",'Fasteners'!$E$2:$E$2,"ordered")+SUMIFS('Tooling'!$I$2:$I$6,'Tooling'!$D$2:$D$6,"P5",'Tooling'!$E$2:$E$6,"ordered")+SUMIFS('Safety'!$I$2:$I$5,'Safety'!$D$2:$D$5,"P5",'Safety'!$E$2:$E$5,"ordered")</f>
-        <v/>
-      </c>
-      <c r="F20" s="4">
+        <v>0</v>
+      </c>
+      <c r="F20" s="13">
         <f>SUMIFS('Actuators'!$I$2:$I$14,'Actuators'!$D$2:$D$14,"P5",'Actuators'!$E$2:$E$14,"to buy")+SUMIFS('Hands'!$I$2:$I$4,'Hands'!$D$2:$D$4,"P5",'Hands'!$E$2:$E$4,"to buy")+SUMIFS('Compute &amp; sensors'!$I$2:$I$6,'Compute &amp; sensors'!$D$2:$D$6,"P5",'Compute &amp; sensors'!$E$2:$E$6,"to buy")+SUMIFS('Power'!$I$2:$I$15,'Power'!$D$2:$D$15,"P5",'Power'!$E$2:$E$15,"to buy")+SUMIFS('Electronics &amp; wiring'!$I$2:$I$12,'Electronics &amp; wiring'!$D$2:$D$12,"P5",'Electronics &amp; wiring'!$E$2:$E$12,"to buy")+SUMIFS('Structure &amp; materials'!$I$2:$I$14,'Structure &amp; materials'!$D$2:$D$14,"P5",'Structure &amp; materials'!$E$2:$E$14,"to buy")+SUMIFS('Fasteners'!$I$2:$I$2,'Fasteners'!$D$2:$D$2,"P5",'Fasteners'!$E$2:$E$2,"to buy")+SUMIFS('Tooling'!$I$2:$I$6,'Tooling'!$D$2:$D$6,"P5",'Tooling'!$E$2:$E$6,"to buy")+SUMIFS('Safety'!$I$2:$I$5,'Safety'!$D$2:$D$5,"P5",'Safety'!$E$2:$E$5,"to buy")</f>
-        <v/>
+        <v>3611.98</v>
       </c>
     </row>
     <row r="21">
@@ -945,21 +949,21 @@
           <t>P6</t>
         </is>
       </c>
-      <c r="C21" s="4">
+      <c r="C21" s="13">
         <f>SUMIFS('Actuators'!$I$2:$I$14,'Actuators'!$D$2:$D$14,"P6")+SUMIFS('Hands'!$I$2:$I$4,'Hands'!$D$2:$D$4,"P6")+SUMIFS('Compute &amp; sensors'!$I$2:$I$6,'Compute &amp; sensors'!$D$2:$D$6,"P6")+SUMIFS('Power'!$I$2:$I$15,'Power'!$D$2:$D$15,"P6")+SUMIFS('Electronics &amp; wiring'!$I$2:$I$12,'Electronics &amp; wiring'!$D$2:$D$12,"P6")+SUMIFS('Structure &amp; materials'!$I$2:$I$14,'Structure &amp; materials'!$D$2:$D$14,"P6")+SUMIFS('Fasteners'!$I$2:$I$2,'Fasteners'!$D$2:$D$2,"P6")+SUMIFS('Tooling'!$I$2:$I$6,'Tooling'!$D$2:$D$6,"P6")+SUMIFS('Safety'!$I$2:$I$5,'Safety'!$D$2:$D$5,"P6")</f>
-        <v/>
-      </c>
-      <c r="D21" s="4">
+        <v>359</v>
+      </c>
+      <c r="D21" s="13">
         <f>SUMIFS('Actuators'!$I$2:$I$14,'Actuators'!$D$2:$D$14,"P6",'Actuators'!$E$2:$E$14,"owned")+SUMIFS('Hands'!$I$2:$I$4,'Hands'!$D$2:$D$4,"P6",'Hands'!$E$2:$E$4,"owned")+SUMIFS('Compute &amp; sensors'!$I$2:$I$6,'Compute &amp; sensors'!$D$2:$D$6,"P6",'Compute &amp; sensors'!$E$2:$E$6,"owned")+SUMIFS('Power'!$I$2:$I$15,'Power'!$D$2:$D$15,"P6",'Power'!$E$2:$E$15,"owned")+SUMIFS('Electronics &amp; wiring'!$I$2:$I$12,'Electronics &amp; wiring'!$D$2:$D$12,"P6",'Electronics &amp; wiring'!$E$2:$E$12,"owned")+SUMIFS('Structure &amp; materials'!$I$2:$I$14,'Structure &amp; materials'!$D$2:$D$14,"P6",'Structure &amp; materials'!$E$2:$E$14,"owned")+SUMIFS('Fasteners'!$I$2:$I$2,'Fasteners'!$D$2:$D$2,"P6",'Fasteners'!$E$2:$E$2,"owned")+SUMIFS('Tooling'!$I$2:$I$6,'Tooling'!$D$2:$D$6,"P6",'Tooling'!$E$2:$E$6,"owned")+SUMIFS('Safety'!$I$2:$I$5,'Safety'!$D$2:$D$5,"P6",'Safety'!$E$2:$E$5,"owned")</f>
-        <v/>
-      </c>
-      <c r="E21" s="4">
+        <v>0</v>
+      </c>
+      <c r="E21" s="13">
         <f>SUMIFS('Actuators'!$I$2:$I$14,'Actuators'!$D$2:$D$14,"P6",'Actuators'!$E$2:$E$14,"ordered")+SUMIFS('Hands'!$I$2:$I$4,'Hands'!$D$2:$D$4,"P6",'Hands'!$E$2:$E$4,"ordered")+SUMIFS('Compute &amp; sensors'!$I$2:$I$6,'Compute &amp; sensors'!$D$2:$D$6,"P6",'Compute &amp; sensors'!$E$2:$E$6,"ordered")+SUMIFS('Power'!$I$2:$I$15,'Power'!$D$2:$D$15,"P6",'Power'!$E$2:$E$15,"ordered")+SUMIFS('Electronics &amp; wiring'!$I$2:$I$12,'Electronics &amp; wiring'!$D$2:$D$12,"P6",'Electronics &amp; wiring'!$E$2:$E$12,"ordered")+SUMIFS('Structure &amp; materials'!$I$2:$I$14,'Structure &amp; materials'!$D$2:$D$14,"P6",'Structure &amp; materials'!$E$2:$E$14,"ordered")+SUMIFS('Fasteners'!$I$2:$I$2,'Fasteners'!$D$2:$D$2,"P6",'Fasteners'!$E$2:$E$2,"ordered")+SUMIFS('Tooling'!$I$2:$I$6,'Tooling'!$D$2:$D$6,"P6",'Tooling'!$E$2:$E$6,"ordered")+SUMIFS('Safety'!$I$2:$I$5,'Safety'!$D$2:$D$5,"P6",'Safety'!$E$2:$E$5,"ordered")</f>
-        <v/>
-      </c>
-      <c r="F21" s="4">
+        <v>0</v>
+      </c>
+      <c r="F21" s="13">
         <f>SUMIFS('Actuators'!$I$2:$I$14,'Actuators'!$D$2:$D$14,"P6",'Actuators'!$E$2:$E$14,"to buy")+SUMIFS('Hands'!$I$2:$I$4,'Hands'!$D$2:$D$4,"P6",'Hands'!$E$2:$E$4,"to buy")+SUMIFS('Compute &amp; sensors'!$I$2:$I$6,'Compute &amp; sensors'!$D$2:$D$6,"P6",'Compute &amp; sensors'!$E$2:$E$6,"to buy")+SUMIFS('Power'!$I$2:$I$15,'Power'!$D$2:$D$15,"P6",'Power'!$E$2:$E$15,"to buy")+SUMIFS('Electronics &amp; wiring'!$I$2:$I$12,'Electronics &amp; wiring'!$D$2:$D$12,"P6",'Electronics &amp; wiring'!$E$2:$E$12,"to buy")+SUMIFS('Structure &amp; materials'!$I$2:$I$14,'Structure &amp; materials'!$D$2:$D$14,"P6",'Structure &amp; materials'!$E$2:$E$14,"to buy")+SUMIFS('Fasteners'!$I$2:$I$2,'Fasteners'!$D$2:$D$2,"P6",'Fasteners'!$E$2:$E$2,"to buy")+SUMIFS('Tooling'!$I$2:$I$6,'Tooling'!$D$2:$D$6,"P6",'Tooling'!$E$2:$E$6,"to buy")+SUMIFS('Safety'!$I$2:$I$5,'Safety'!$D$2:$D$5,"P6",'Safety'!$E$2:$E$5,"to buy")</f>
-        <v/>
+        <v>359</v>
       </c>
     </row>
     <row r="22">
@@ -969,21 +973,21 @@
         </is>
       </c>
       <c r="B22" s="5" t="n"/>
-      <c r="C22" s="6">
+      <c r="C22" s="14">
         <f>SUM(C17:C21)</f>
-        <v/>
-      </c>
-      <c r="D22" s="6">
+        <v>17531.03</v>
+      </c>
+      <c r="D22" s="14">
         <f>SUM(D17:D21)</f>
-        <v/>
-      </c>
-      <c r="E22" s="6">
+        <v>3732</v>
+      </c>
+      <c r="E22" s="14">
         <f>SUM(E17:E21)</f>
-        <v/>
-      </c>
-      <c r="F22" s="6">
+        <v>0</v>
+      </c>
+      <c r="F22" s="14">
         <f>SUM(F17:F21)</f>
-        <v/>
+        <v>13799.03</v>
       </c>
     </row>
     <row r="23">
@@ -992,9 +996,9 @@
           <t>Check: phases add up to the group total</t>
         </is>
       </c>
-      <c r="C23">
+      <c r="C23" t="str">
         <f>IF(ROUND(C22-C14,2)=0,"OK","MISMATCH")</f>
-        <v/>
+        <v>OK</v>
       </c>
     </row>
     <row r="25" ht="48" customHeight="1">
@@ -1127,12 +1131,12 @@
       <c r="G2" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H2" s="10" t="n">
+      <c r="H2" s="16" t="n">
         <v>40</v>
       </c>
-      <c r="I2" s="10">
+      <c r="I2" s="16">
         <f>G2*H2</f>
-        <v/>
+        <v>40</v>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
@@ -1170,12 +1174,12 @@
       <c r="G3" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H3" s="10" t="n">
+      <c r="H3" s="16" t="n">
         <v>50</v>
       </c>
-      <c r="I3" s="10">
+      <c r="I3" s="16">
         <f>G3*H3</f>
-        <v/>
+        <v>50</v>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
@@ -1213,12 +1217,12 @@
       <c r="G4" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H4" s="10" t="n">
+      <c r="H4" s="16" t="n">
         <v>300</v>
       </c>
-      <c r="I4" s="10">
+      <c r="I4" s="16">
         <f>G4*H4</f>
-        <v/>
+        <v>300</v>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
@@ -1256,12 +1260,12 @@
       <c r="G5" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H5" s="10" t="n">
+      <c r="H5" s="16" t="n">
         <v>80</v>
       </c>
-      <c r="I5" s="10">
+      <c r="I5" s="16">
         <f>G5*H5</f>
-        <v/>
+        <v>80</v>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
@@ -1287,9 +1291,9 @@
       <c r="F7" s="5" t="n"/>
       <c r="G7" s="5" t="n"/>
       <c r="H7" s="5" t="n"/>
-      <c r="I7" s="6">
+      <c r="I7" s="14">
         <f>SUM(I2:I5)</f>
-        <v/>
+        <v>470</v>
       </c>
       <c r="J7" s="5" t="n"/>
       <c r="K7" s="5" t="n"/>
@@ -1406,7 +1410,7 @@
           <t>https://www.seeedstudio.com/Robostride-00-Actuator-p-6664.html</t>
         </is>
       </c>
-      <c r="E2" s="10" t="n">
+      <c r="E2" s="16" t="n">
         <v>138.99</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1456,7 +1460,7 @@
           <t>https://www.seeedstudio.com/Robostride-03-Actuator-p-6774.html</t>
         </is>
       </c>
-      <c r="E3" s="10" t="n">
+      <c r="E3" s="16" t="n">
         <v>225</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1502,7 +1506,7 @@
           <t>https://www.seeedstudio.com/Robostride-04-Actuator-p-6775.html</t>
         </is>
       </c>
-      <c r="E4" s="10" t="n">
+      <c r="E4" s="16" t="n">
         <v>255</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1552,7 +1556,7 @@
           <t>https://www.seeedstudio.com/Robostride-06-Actuator-p-6668.html</t>
         </is>
       </c>
-      <c r="E5" s="10" t="n">
+      <c r="E5" s="16" t="n">
         <v>210</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -1598,7 +1602,7 @@
           <t>https://simplybearings.co.uk/shop/p170125/68062RS-Budget-Rubber-Sealed-Thin-Section-Deep-Groove-Ball-Bearing-30x42x7mm/product_info.html</t>
         </is>
       </c>
-      <c r="E6" s="10" t="n"/>
+      <c r="E6" s="16" t="n"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
           <t>£6.33 ex VAT; £5.64 at 4+</t>
@@ -1642,7 +1646,7 @@
           <t>https://www.zoro.com/ezo-deep-groove-30mm-bore-42mm-od-sealed-6806-2rsc0srl/i/G2080051</t>
         </is>
       </c>
-      <c r="E7" s="10" t="n"/>
+      <c r="E7" s="16" t="n"/>
       <c r="F7" s="2" t="n"/>
       <c r="G7" s="2" t="n"/>
       <c r="H7" t="inlineStr">
@@ -1682,7 +1686,7 @@
           <t>https://www.18650batterystore.com/products/jk-b2a24s15p-bms</t>
         </is>
       </c>
-      <c r="E8" s="10" t="n">
+      <c r="E8" s="16" t="n">
         <v>145</v>
       </c>
       <c r="F8" s="2" t="n"/>
@@ -1728,7 +1732,7 @@
           <t>https://store.orbbec.com/products/gemini-335l</t>
         </is>
       </c>
-      <c r="E9" s="10" t="n">
+      <c r="E9" s="16" t="n">
         <v>359</v>
       </c>
       <c r="F9" s="2" t="n"/>
@@ -1770,7 +1774,7 @@
           <t>https://www.robotshop.com/products/orbbec-gemini-335l-camera</t>
         </is>
       </c>
-      <c r="E10" s="10" t="n">
+      <c r="E10" s="16" t="n">
         <v>413</v>
       </c>
       <c r="F10" s="2" t="n"/>
@@ -1816,7 +1820,7 @@
           <t>https://www.seeedstudio.com/Robostride-CAN-USB-Driver-Board-p-6708.html</t>
         </is>
       </c>
-      <c r="E11" s="10" t="n">
+      <c r="E11" s="16" t="n">
         <v>15</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1862,7 +1866,7 @@
           <t>https://reach.dog/shop/openlight-labs/products/canable-pro-isolated-usb-to-can-adapter</t>
         </is>
       </c>
-      <c r="E12" s="10" t="n">
+      <c r="E12" s="16" t="n">
         <v>60</v>
       </c>
       <c r="F12" s="2" t="n"/>
@@ -1904,7 +1908,7 @@
           <t>https://robotshop.com/products/eyou-robotics-can-usb-adapter-canable-pro</t>
         </is>
       </c>
-      <c r="E13" s="10" t="n">
+      <c r="E13" s="16" t="n">
         <v>42</v>
       </c>
       <c r="F13" s="2" t="n"/>
@@ -1946,7 +1950,7 @@
           <t>https://www.carrefouruae.com/mafuae/en/miscellaneous/innomaker-dual-channels-usb-to-can-converter-for-raspberry-pi5-4-pi3b-pi3-pi-zero-w-jetson-nano-tinker-board-any-sbcs-desktop-laptop-support-windows-linux-mac-os-android-venus-os-/p/1881649107638</t>
         </is>
       </c>
-      <c r="E14" s="10" t="n">
+      <c r="E14" s="16" t="n">
         <v>126</v>
       </c>
       <c r="F14" s="2" t="n"/>
@@ -1988,7 +1992,7 @@
           <t>https://github.com/INNO-MAKER/usb2can</t>
         </is>
       </c>
-      <c r="E15" s="10" t="n"/>
+      <c r="E15" s="16" t="n"/>
       <c r="F15" s="2" t="n"/>
       <c r="G15" s="2" t="n"/>
       <c r="H15" t="inlineStr">
@@ -2028,7 +2032,7 @@
           <t>https://www.18650batterystore.com/products/molicel-p45b</t>
         </is>
       </c>
-      <c r="E16" s="10" t="n">
+      <c r="E16" s="16" t="n">
         <v>9.99</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -2078,7 +2082,7 @@
           <t>https://www.batteriesinaflash.com/regular-rechargeable-batteries/molicel-inr-21700-p45b-3-6-volt-4500mah-45a-lithium-ion-cell</t>
         </is>
       </c>
-      <c r="E17" s="10" t="n">
+      <c r="E17" s="16" t="n">
         <v>9.949999999999999</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -2124,7 +2128,7 @@
           <t>https://www.cnx-software.com/2026/07/22/nvidia-increases-the-price-of-jetson-modules-and-devkits-by-up-to-101/</t>
         </is>
       </c>
-      <c r="E18" s="10" t="n">
+      <c r="E18" s="16" t="n">
         <v>3499</v>
       </c>
       <c r="F18" s="2" t="n"/>
@@ -2166,7 +2170,7 @@
           <t>https://marketplace.nvidia.com/en-us/enterprise/robotics-edge/jetson-agx-orin-developer-kit/</t>
         </is>
       </c>
-      <c r="E19" s="10" t="n">
+      <c r="E19" s="16" t="n">
         <v>3499</v>
       </c>
       <c r="F19" s="2" t="n"/>
@@ -2212,7 +2216,7 @@
           <t>https://www.sparkfun.com/nvidia-jetson-agx-orin-64gb-developer-kit.html</t>
         </is>
       </c>
-      <c r="E20" s="10" t="n">
+      <c r="E20" s="16" t="n">
         <v>3499</v>
       </c>
       <c r="F20" s="2" t="n"/>
@@ -2258,7 +2262,7 @@
           <t>https://www.bravoelectro.com/ddr-120c-12.html</t>
         </is>
       </c>
-      <c r="E21" s="10" t="n">
+      <c r="E21" s="16" t="n">
         <v>67.26000000000001</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -2304,7 +2308,7 @@
           <t>https://github.com/pollen-robotics/AmazingHand</t>
         </is>
       </c>
-      <c r="E22" s="10" t="n"/>
+      <c r="E22" s="16" t="n"/>
       <c r="F22" s="2" t="n"/>
       <c r="G22" s="2" t="n"/>
       <c r="H22" t="inlineStr">
@@ -2344,7 +2348,7 @@
           <t>https://www.seeedstudio.com/Amazing-Hand-Open-Source-3D-Printable-Robotic-Hand-Kit.html</t>
         </is>
       </c>
-      <c r="E23" s="10" t="n">
+      <c r="E23" s="16" t="n">
         <v>99</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -2394,7 +2398,7 @@
           <t>https://www.seeedstudio.com/Amazing-Hand-Right-Hand-The-Open-Source-Robotic-Hand-Developer-Kit.html</t>
         </is>
       </c>
-      <c r="E24" s="10" t="n">
+      <c r="E24" s="16" t="n">
         <v>99</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -2444,7 +2448,7 @@
           <t>https://uk.robotshop.com/products/fe-urt-1-usb-to-ttl-485-bus-programmer</t>
         </is>
       </c>
-      <c r="E25" s="10" t="n"/>
+      <c r="E25" s="16" t="n"/>
       <c r="F25" s="2" t="inlineStr">
         <is>
           <t>£13.67</t>
@@ -2492,7 +2496,7 @@
           <t>https://www.waveshare.com/bus-servo-adapter-a.htm</t>
         </is>
       </c>
-      <c r="E26" s="10" t="n">
+      <c r="E26" s="16" t="n">
         <v>4.99</v>
       </c>
       <c r="F26" s="2" t="n"/>
@@ -2534,7 +2538,7 @@
           <t>https://aifitlab.com/products/feetech-sts3250-servo-motor</t>
         </is>
       </c>
-      <c r="E27" s="10" t="n">
+      <c r="E27" s="16" t="n">
         <v>97</v>
       </c>
       <c r="F27" s="2" t="n"/>
@@ -2580,7 +2584,7 @@
           <t>https://openelab.io/products/feetech-sts3250-c002-servo-12v</t>
         </is>
       </c>
-      <c r="E28" s="10" t="n"/>
+      <c r="E28" s="16" t="n"/>
       <c r="F28" s="2" t="inlineStr">
         <is>
           <t>€75.85</t>
@@ -2624,7 +2628,7 @@
           <t>https://rcdrone.top/products/feetech-sts3250-servo-motor</t>
         </is>
       </c>
-      <c r="E29" s="10" t="n">
+      <c r="E29" s="16" t="n">
         <v>125</v>
       </c>
       <c r="F29" s="2" t="n"/>
@@ -7871,12 +7875,12 @@
       <c r="G2" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H2" s="10" t="n">
+      <c r="H2" s="16" t="n">
         <v>225</v>
       </c>
-      <c r="I2" s="10">
+      <c r="I2" s="16">
         <f>G2*H2</f>
-        <v/>
+        <v>225</v>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
@@ -7928,12 +7932,12 @@
       <c r="G3" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H3" s="10" t="n">
+      <c r="H3" s="16" t="n">
         <v>255</v>
       </c>
-      <c r="I3" s="10">
+      <c r="I3" s="16">
         <f>G3*H3</f>
-        <v/>
+        <v>255</v>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
@@ -7985,12 +7989,12 @@
       <c r="G4" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="H4" s="10" t="n">
+      <c r="H4" s="16" t="n">
         <v>225</v>
       </c>
-      <c r="I4" s="10">
+      <c r="I4" s="16">
         <f>G4*H4</f>
-        <v/>
+        <v>450</v>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
@@ -8042,12 +8046,12 @@
       <c r="G5" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="H5" s="10" t="n">
+      <c r="H5" s="16" t="n">
         <v>255</v>
       </c>
-      <c r="I5" s="10">
+      <c r="I5" s="16">
         <f>G5*H5</f>
-        <v/>
+        <v>510</v>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
@@ -8099,12 +8103,12 @@
       <c r="G6" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="H6" s="10" t="n">
+      <c r="H6" s="16" t="n">
         <v>225</v>
       </c>
-      <c r="I6" s="10">
+      <c r="I6" s="16">
         <f>G6*H6</f>
-        <v/>
+        <v>675</v>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
@@ -8156,12 +8160,12 @@
       <c r="G7" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="H7" s="10" t="n">
+      <c r="H7" s="16" t="n">
         <v>255</v>
       </c>
-      <c r="I7" s="10">
+      <c r="I7" s="16">
         <f>G7*H7</f>
-        <v/>
+        <v>765</v>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
@@ -8213,12 +8217,12 @@
       <c r="G8" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H8" s="10" t="n">
+      <c r="H8" s="16" t="n">
         <v>225</v>
       </c>
-      <c r="I8" s="10">
+      <c r="I8" s="16">
         <f>G8*H8</f>
-        <v/>
+        <v>225</v>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
@@ -8266,12 +8270,12 @@
       <c r="G9" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H9" s="10" t="n">
+      <c r="H9" s="16" t="n">
         <v>255</v>
       </c>
-      <c r="I9" s="10">
+      <c r="I9" s="16">
         <f>G9*H9</f>
-        <v/>
+        <v>255</v>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
@@ -8319,12 +8323,12 @@
       <c r="G10" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="H10" s="10" t="n">
+      <c r="H10" s="16" t="n">
         <v>97</v>
       </c>
-      <c r="I10" s="10">
+      <c r="I10" s="16">
         <f>G10*H10</f>
-        <v/>
+        <v>388</v>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
@@ -8376,12 +8380,12 @@
       <c r="G11" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="H11" s="10" t="n">
+      <c r="H11" s="16" t="n">
         <v>138.99</v>
       </c>
-      <c r="I11" s="10">
+      <c r="I11" s="16">
         <f>G11*H11</f>
-        <v/>
+        <v>277.98</v>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
@@ -8433,12 +8437,12 @@
       <c r="G12" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="H12" s="10" t="n">
+      <c r="H12" s="16" t="n">
         <v>225</v>
       </c>
-      <c r="I12" s="10">
+      <c r="I12" s="16">
         <f>G12*H12</f>
-        <v/>
+        <v>1125</v>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
@@ -8490,12 +8494,12 @@
       <c r="G13" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="H13" s="10" t="n">
+      <c r="H13" s="16" t="n">
         <v>210</v>
       </c>
-      <c r="I13" s="10">
+      <c r="I13" s="16">
         <f>G13*H13</f>
-        <v/>
+        <v>840</v>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
@@ -8547,12 +8551,12 @@
       <c r="G14" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H14" s="10" t="n">
+      <c r="H14" s="16" t="n">
         <v>210</v>
       </c>
-      <c r="I14" s="10">
+      <c r="I14" s="16">
         <f>G14*H14</f>
-        <v/>
+        <v>210</v>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
@@ -8579,9 +8583,9 @@
       <c r="F16" s="5" t="n"/>
       <c r="G16" s="5" t="n"/>
       <c r="H16" s="5" t="n"/>
-      <c r="I16" s="6">
+      <c r="I16" s="14">
         <f>SUM(I2:I14)</f>
-        <v/>
+        <v>6200.98</v>
       </c>
       <c r="J16" s="5" t="n"/>
       <c r="K16" s="5" t="n"/>
@@ -8733,12 +8737,12 @@
       <c r="G2" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="H2" s="10" t="n">
+      <c r="H2" s="16" t="n">
         <v>99</v>
       </c>
-      <c r="I2" s="10">
+      <c r="I2" s="16">
         <f>G2*H2</f>
-        <v/>
+        <v>198</v>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
@@ -8785,12 +8789,12 @@
       <c r="G3" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="H3" s="10" t="n">
+      <c r="H3" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="I3" s="10">
+      <c r="I3" s="16">
         <f>G3*H3</f>
-        <v/>
+        <v>16</v>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
@@ -8832,12 +8836,12 @@
       <c r="G4" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="H4" s="10" t="n">
+      <c r="H4" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="I4" s="10">
+      <c r="I4" s="16">
         <f>G4*H4</f>
-        <v/>
+        <v>10</v>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
@@ -8868,9 +8872,9 @@
       <c r="F6" s="5" t="n"/>
       <c r="G6" s="5" t="n"/>
       <c r="H6" s="5" t="n"/>
-      <c r="I6" s="6">
+      <c r="I6" s="14">
         <f>SUM(I2:I4)</f>
-        <v/>
+        <v>224</v>
       </c>
       <c r="J6" s="5" t="n"/>
       <c r="K6" s="5" t="n"/>
@@ -9011,12 +9015,12 @@
       <c r="G2" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H2" s="10" t="n">
+      <c r="H2" s="16" t="n">
         <v>35</v>
       </c>
-      <c r="I2" s="10">
+      <c r="I2" s="16">
         <f>G2*H2</f>
-        <v/>
+        <v>35</v>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
@@ -9058,12 +9062,12 @@
       <c r="G3" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H3" s="10" t="n">
+      <c r="H3" s="16" t="n">
         <v>3499</v>
       </c>
-      <c r="I3" s="10">
+      <c r="I3" s="16">
         <f>G3*H3</f>
-        <v/>
+        <v>3499</v>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
@@ -9110,12 +9114,12 @@
       <c r="G4" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H4" s="10" t="n">
+      <c r="H4" s="16" t="n">
         <v>100</v>
       </c>
-      <c r="I4" s="10">
+      <c r="I4" s="16">
         <f>G4*H4</f>
-        <v/>
+        <v>100</v>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
@@ -9157,12 +9161,12 @@
       <c r="G5" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H5" s="10" t="n">
+      <c r="H5" s="16" t="n">
         <v>730</v>
       </c>
-      <c r="I5" s="10">
+      <c r="I5" s="16">
         <f>G5*H5</f>
-        <v/>
+        <v>730</v>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
@@ -9204,12 +9208,12 @@
       <c r="G6" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H6" s="10" t="n">
+      <c r="H6" s="16" t="n">
         <v>359</v>
       </c>
-      <c r="I6" s="10">
+      <c r="I6" s="16">
         <f>G6*H6</f>
-        <v/>
+        <v>359</v>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
@@ -9240,9 +9244,9 @@
       <c r="F8" s="5" t="n"/>
       <c r="G8" s="5" t="n"/>
       <c r="H8" s="5" t="n"/>
-      <c r="I8" s="6">
+      <c r="I8" s="14">
         <f>SUM(I2:I6)</f>
-        <v/>
+        <v>4723</v>
       </c>
       <c r="J8" s="5" t="n"/>
       <c r="K8" s="5" t="n"/>
@@ -9383,12 +9387,12 @@
       <c r="G2" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H2" s="10" t="n">
+      <c r="H2" s="16" t="n">
         <v>250</v>
       </c>
-      <c r="I2" s="10">
+      <c r="I2" s="16">
         <f>G2*H2</f>
-        <v/>
+        <v>250</v>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
@@ -9430,12 +9434,12 @@
       <c r="G3" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H3" s="10" t="n">
+      <c r="H3" s="16" t="n">
         <v>60</v>
       </c>
-      <c r="I3" s="10">
+      <c r="I3" s="16">
         <f>G3*H3</f>
-        <v/>
+        <v>60</v>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
@@ -9477,12 +9481,12 @@
       <c r="G4" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H4" s="10" t="n">
+      <c r="H4" s="16" t="n">
         <v>40</v>
       </c>
-      <c r="I4" s="10">
+      <c r="I4" s="16">
         <f>G4*H4</f>
-        <v/>
+        <v>40</v>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
@@ -9524,12 +9528,12 @@
       <c r="G5" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H5" s="10" t="n">
+      <c r="H5" s="16" t="n">
         <v>300</v>
       </c>
-      <c r="I5" s="10">
+      <c r="I5" s="16">
         <f>G5*H5</f>
-        <v/>
+        <v>300</v>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
@@ -9571,12 +9575,12 @@
       <c r="G6" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H6" s="10" t="n">
+      <c r="H6" s="16" t="n">
         <v>145</v>
       </c>
-      <c r="I6" s="10">
+      <c r="I6" s="16">
         <f>G6*H6</f>
-        <v/>
+        <v>145</v>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
@@ -9623,12 +9627,12 @@
       <c r="G7" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="H7" s="10" t="n">
+      <c r="H7" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="I7" s="10">
+      <c r="I7" s="16">
         <f>G7*H7</f>
-        <v/>
+        <v>30</v>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
@@ -9670,12 +9674,12 @@
       <c r="G8" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H8" s="10" t="n">
+      <c r="H8" s="16" t="n">
         <v>60</v>
       </c>
-      <c r="I8" s="10">
+      <c r="I8" s="16">
         <f>G8*H8</f>
-        <v/>
+        <v>60</v>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
@@ -9713,12 +9717,12 @@
       <c r="G9" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H9" s="10" t="n">
+      <c r="H9" s="16" t="n">
         <v>80</v>
       </c>
-      <c r="I9" s="10">
+      <c r="I9" s="16">
         <f>G9*H9</f>
-        <v/>
+        <v>80</v>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
@@ -9760,12 +9764,12 @@
       <c r="G10" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H10" s="10" t="n">
+      <c r="H10" s="16" t="n">
         <v>40</v>
       </c>
-      <c r="I10" s="10">
+      <c r="I10" s="16">
         <f>G10*H10</f>
-        <v/>
+        <v>40</v>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
@@ -9803,12 +9807,12 @@
       <c r="G11" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H11" s="10" t="n">
+      <c r="H11" s="16" t="n">
         <v>80</v>
       </c>
-      <c r="I11" s="10">
+      <c r="I11" s="16">
         <f>G11*H11</f>
-        <v/>
+        <v>80</v>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
@@ -9850,12 +9854,12 @@
       <c r="G12" s="9" t="n">
         <v>39</v>
       </c>
-      <c r="H12" s="10" t="n">
+      <c r="H12" s="16" t="n">
         <v>9.949999999999999</v>
       </c>
-      <c r="I12" s="10">
+      <c r="I12" s="16">
         <f>G12*H12</f>
-        <v/>
+        <v>388.05</v>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
@@ -9902,12 +9906,12 @@
       <c r="G13" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H13" s="10" t="n">
+      <c r="H13" s="16" t="n">
         <v>80</v>
       </c>
-      <c r="I13" s="10">
+      <c r="I13" s="16">
         <f>G13*H13</f>
-        <v/>
+        <v>80</v>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
@@ -9945,12 +9949,12 @@
       <c r="G14" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H14" s="10" t="n">
+      <c r="H14" s="16" t="n">
         <v>20</v>
       </c>
-      <c r="I14" s="10">
+      <c r="I14" s="16">
         <f>G14*H14</f>
-        <v/>
+        <v>20</v>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
@@ -9988,12 +9992,12 @@
       <c r="G15" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H15" s="10" t="n">
+      <c r="H15" s="16" t="n">
         <v>60</v>
       </c>
-      <c r="I15" s="10">
+      <c r="I15" s="16">
         <f>G15*H15</f>
-        <v/>
+        <v>60</v>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
@@ -10019,9 +10023,9 @@
       <c r="F17" s="5" t="n"/>
       <c r="G17" s="5" t="n"/>
       <c r="H17" s="5" t="n"/>
-      <c r="I17" s="6">
+      <c r="I17" s="14">
         <f>SUM(I2:I15)</f>
-        <v/>
+        <v>1633.05</v>
       </c>
       <c r="J17" s="5" t="n"/>
       <c r="K17" s="5" t="n"/>
@@ -10162,12 +10166,12 @@
       <c r="G2" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H2" s="10" t="n">
+      <c r="H2" s="16" t="n">
         <v>60</v>
       </c>
-      <c r="I2" s="10">
+      <c r="I2" s="16">
         <f>G2*H2</f>
-        <v/>
+        <v>60</v>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
@@ -10214,12 +10218,12 @@
       <c r="G3" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H3" s="10" t="n">
+      <c r="H3" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="I3" s="10">
+      <c r="I3" s="16">
         <f>G3*H3</f>
-        <v/>
+        <v>15</v>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
@@ -10266,12 +10270,12 @@
       <c r="G4" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H4" s="10" t="n">
+      <c r="H4" s="16" t="n">
         <v>50</v>
       </c>
-      <c r="I4" s="10">
+      <c r="I4" s="16">
         <f>G4*H4</f>
-        <v/>
+        <v>50</v>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
@@ -10309,12 +10313,12 @@
       <c r="G5" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="H5" s="10" t="n">
+      <c r="H5" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="I5" s="10">
+      <c r="I5" s="16">
         <f>G5*H5</f>
-        <v/>
+        <v>20</v>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
@@ -10356,12 +10360,12 @@
       <c r="G6" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H6" s="10" t="n">
+      <c r="H6" s="16" t="n">
         <v>30</v>
       </c>
-      <c r="I6" s="10">
+      <c r="I6" s="16">
         <f>G6*H6</f>
-        <v/>
+        <v>30</v>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
@@ -10403,12 +10407,12 @@
       <c r="G7" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="H7" s="10" t="n">
+      <c r="H7" s="16" t="n">
         <v>130</v>
       </c>
-      <c r="I7" s="10">
+      <c r="I7" s="16">
         <f>G7*H7</f>
-        <v/>
+        <v>260</v>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
@@ -10455,12 +10459,12 @@
       <c r="G8" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H8" s="10" t="n">
+      <c r="H8" s="16" t="n">
         <v>60</v>
       </c>
-      <c r="I8" s="10">
+      <c r="I8" s="16">
         <f>G8*H8</f>
-        <v/>
+        <v>60</v>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
@@ -10507,12 +10511,12 @@
       <c r="G9" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="H9" s="10" t="n">
+      <c r="H9" s="16" t="n">
         <v>12</v>
       </c>
-      <c r="I9" s="10">
+      <c r="I9" s="16">
         <f>G9*H9</f>
-        <v/>
+        <v>48</v>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
@@ -10554,12 +10558,12 @@
       <c r="G10" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H10" s="10" t="n">
+      <c r="H10" s="16" t="n">
         <v>200</v>
       </c>
-      <c r="I10" s="10">
+      <c r="I10" s="16">
         <f>G10*H10</f>
-        <v/>
+        <v>200</v>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
@@ -10597,12 +10601,12 @@
       <c r="G11" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H11" s="10" t="n">
+      <c r="H11" s="16" t="n">
         <v>60</v>
       </c>
-      <c r="I11" s="10">
+      <c r="I11" s="16">
         <f>G11*H11</f>
-        <v/>
+        <v>60</v>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
@@ -10640,12 +10644,12 @@
       <c r="G12" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H12" s="10" t="n">
+      <c r="H12" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="I12" s="10">
+      <c r="I12" s="16">
         <f>G12*H12</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
@@ -10676,9 +10680,9 @@
       <c r="F14" s="5" t="n"/>
       <c r="G14" s="5" t="n"/>
       <c r="H14" s="5" t="n"/>
-      <c r="I14" s="6">
+      <c r="I14" s="14">
         <f>SUM(I2:I12)</f>
-        <v/>
+        <v>808</v>
       </c>
       <c r="J14" s="5" t="n"/>
       <c r="K14" s="5" t="n"/>
@@ -10822,12 +10826,12 @@
       <c r="G2" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H2" s="10" t="n">
+      <c r="H2" s="16" t="n">
         <v>300</v>
       </c>
-      <c r="I2" s="10">
+      <c r="I2" s="16">
         <f>G2*H2</f>
-        <v/>
+        <v>300</v>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
@@ -10869,12 +10873,12 @@
       <c r="G3" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="H3" s="10" t="n">
+      <c r="H3" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="I3" s="10">
+      <c r="I3" s="16">
         <f>G3*H3</f>
-        <v/>
+        <v>60</v>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
@@ -10921,12 +10925,12 @@
       <c r="G4" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H4" s="10" t="n">
+      <c r="H4" s="16" t="n">
         <v>100</v>
       </c>
-      <c r="I4" s="10">
+      <c r="I4" s="16">
         <f>G4*H4</f>
-        <v/>
+        <v>100</v>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
@@ -10964,12 +10968,12 @@
       <c r="G5" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="H5" s="10" t="n">
+      <c r="H5" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="I5" s="10">
+      <c r="I5" s="16">
         <f>G5*H5</f>
-        <v/>
+        <v>40</v>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
@@ -11011,12 +11015,12 @@
       <c r="G6" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="H6" s="10" t="n">
+      <c r="H6" s="16" t="n">
         <v>95</v>
       </c>
-      <c r="I6" s="10">
+      <c r="I6" s="16">
         <f>G6*H6</f>
-        <v/>
+        <v>380</v>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
@@ -11058,12 +11062,12 @@
       <c r="G7" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="H7" s="10" t="n">
+      <c r="H7" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="I7" s="10">
+      <c r="I7" s="16">
         <f>G7*H7</f>
-        <v/>
+        <v>64</v>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
@@ -11105,12 +11109,12 @@
       <c r="G8" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H8" s="10" t="n">
+      <c r="H8" s="16" t="n">
         <v>450</v>
       </c>
-      <c r="I8" s="10">
+      <c r="I8" s="16">
         <f>G8*H8</f>
-        <v/>
+        <v>450</v>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
@@ -11152,12 +11156,12 @@
       <c r="G9" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="H9" s="10" t="n">
+      <c r="H9" s="16" t="n">
         <v>33</v>
       </c>
-      <c r="I9" s="10">
+      <c r="I9" s="16">
         <f>G9*H9</f>
-        <v/>
+        <v>66</v>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
@@ -11199,12 +11203,12 @@
       <c r="G10" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H10" s="10" t="n">
+      <c r="H10" s="16" t="n">
         <v>42</v>
       </c>
-      <c r="I10" s="10">
+      <c r="I10" s="16">
         <f>G10*H10</f>
-        <v/>
+        <v>42</v>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
@@ -11246,12 +11250,12 @@
       <c r="G11" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H11" s="10" t="n">
+      <c r="H11" s="16" t="n">
         <v>400</v>
       </c>
-      <c r="I11" s="10">
+      <c r="I11" s="16">
         <f>G11*H11</f>
-        <v/>
+        <v>400</v>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
@@ -11293,12 +11297,12 @@
       <c r="G12" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H12" s="10" t="n">
+      <c r="H12" s="16" t="n">
         <v>250</v>
       </c>
-      <c r="I12" s="10">
+      <c r="I12" s="16">
         <f>G12*H12</f>
-        <v/>
+        <v>250</v>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
@@ -11336,12 +11340,12 @@
       <c r="G13" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H13" s="10" t="n">
+      <c r="H13" s="16" t="n">
         <v>80</v>
       </c>
-      <c r="I13" s="10">
+      <c r="I13" s="16">
         <f>G13*H13</f>
-        <v/>
+        <v>80</v>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
@@ -11379,12 +11383,12 @@
       <c r="G14" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H14" s="10" t="n">
+      <c r="H14" s="16" t="n">
         <v>350</v>
       </c>
-      <c r="I14" s="10">
+      <c r="I14" s="16">
         <f>G14*H14</f>
-        <v/>
+        <v>350</v>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
@@ -11410,9 +11414,9 @@
       <c r="F16" s="5" t="n"/>
       <c r="G16" s="5" t="n"/>
       <c r="H16" s="5" t="n"/>
-      <c r="I16" s="6">
+      <c r="I16" s="14">
         <f>SUM(I2:I14)</f>
-        <v/>
+        <v>2582</v>
       </c>
       <c r="J16" s="5" t="n"/>
       <c r="K16" s="5" t="n"/>
@@ -11552,12 +11556,12 @@
       <c r="G2" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H2" s="10" t="n">
+      <c r="H2" s="16" t="n">
         <v>180</v>
       </c>
-      <c r="I2" s="10">
+      <c r="I2" s="16">
         <f>G2*H2</f>
-        <v/>
+        <v>180</v>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
@@ -11583,9 +11587,9 @@
       <c r="F4" s="5" t="n"/>
       <c r="G4" s="5" t="n"/>
       <c r="H4" s="5" t="n"/>
-      <c r="I4" s="6">
+      <c r="I4" s="14">
         <f>SUM(I2:I2)</f>
-        <v/>
+        <v>180</v>
       </c>
       <c r="J4" s="5" t="n"/>
       <c r="K4" s="5" t="n"/>
@@ -11722,12 +11726,12 @@
       <c r="G2" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="H2" s="10" t="n">
+      <c r="H2" s="16" t="n">
         <v>20</v>
       </c>
-      <c r="I2" s="10">
+      <c r="I2" s="16">
         <f>G2*H2</f>
-        <v/>
+        <v>160</v>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
@@ -11765,12 +11769,12 @@
       <c r="G3" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H3" s="10" t="n">
+      <c r="H3" s="16" t="n">
         <v>200</v>
       </c>
-      <c r="I3" s="10">
+      <c r="I3" s="16">
         <f>G3*H3</f>
-        <v/>
+        <v>200</v>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
@@ -11812,12 +11816,12 @@
       <c r="G4" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H4" s="10" t="n">
+      <c r="H4" s="16" t="n">
         <v>80</v>
       </c>
-      <c r="I4" s="10">
+      <c r="I4" s="16">
         <f>G4*H4</f>
-        <v/>
+        <v>80</v>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
@@ -11859,12 +11863,12 @@
       <c r="G5" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H5" s="10" t="n">
+      <c r="H5" s="16" t="n">
         <v>120</v>
       </c>
-      <c r="I5" s="10">
+      <c r="I5" s="16">
         <f>G5*H5</f>
-        <v/>
+        <v>120</v>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
@@ -11902,12 +11906,12 @@
       <c r="G6" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H6" s="10" t="n">
+      <c r="H6" s="16" t="n">
         <v>150</v>
       </c>
-      <c r="I6" s="10">
+      <c r="I6" s="16">
         <f>G6*H6</f>
-        <v/>
+        <v>150</v>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
@@ -11933,9 +11937,9 @@
       <c r="F8" s="5" t="n"/>
       <c r="G8" s="5" t="n"/>
       <c r="H8" s="5" t="n"/>
-      <c r="I8" s="6">
+      <c r="I8" s="14">
         <f>SUM(I2:I6)</f>
-        <v/>
+        <v>710</v>
       </c>
       <c r="J8" s="5" t="n"/>
       <c r="K8" s="5" t="n"/>

</xml_diff>

<commit_message>
BOM workbook ships with every status empty, as a template for builders
No line, made part or bolt is marked owned or ordered; an empty status
counts as to buy, and the Summary's to-buy column is the total less owned
and ordered. Docs no longer quote what this build owns.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bom/bom.xlsx
+++ b/bom/bom.xlsx
@@ -511,7 +511,7 @@
     <row r="2" ht="48" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>This workbook is the BOM's source of truth; copy it to track your own build. Set each line's status to to buy, ordered or owned and the totals follow. After editing, run python tools/bom/book.py to tidy it. Prices are indicative: see each line's price basis and the Sourcing sheet.</t>
+          <t>This workbook is the BOM's source of truth; copy it to track your own build. Set a line's status to owned or ordered as you go (empty counts as to buy) and the totals follow. After editing, run python tools/bom/book.py to tidy it. Prices are indicative: see each line's price basis and the Sourcing sheet.</t>
         </is>
       </c>
     </row>
@@ -570,7 +570,7 @@
         <v>0</v>
       </c>
       <c r="F5" s="13">
-        <f>SUMIFS('Actuators'!$H$2:$H$6,'Actuators'!$D$2:$D$6,"to buy")</f>
+        <f>C5-D5-E5</f>
         <v>6200.98</v>
       </c>
     </row>
@@ -590,15 +590,15 @@
       </c>
       <c r="D6" s="13">
         <f>SUMIFS('Hands'!$H$2:$H$4,'Hands'!$D$2:$D$4,"owned")</f>
-        <v>198</v>
+        <v>0</v>
       </c>
       <c r="E6" s="13">
         <f>SUMIFS('Hands'!$H$2:$H$4,'Hands'!$D$2:$D$4,"ordered")</f>
         <v>0</v>
       </c>
       <c r="F6" s="13">
-        <f>SUMIFS('Hands'!$H$2:$H$4,'Hands'!$D$2:$D$4,"to buy")</f>
-        <v>26</v>
+        <f>C6-D6-E6</f>
+        <v>224</v>
       </c>
     </row>
     <row r="7">
@@ -617,15 +617,15 @@
       </c>
       <c r="D7" s="13">
         <f>SUMIFS('Compute &amp; sensors'!$H$2:$H$6,'Compute &amp; sensors'!$D$2:$D$6,"owned")</f>
-        <v>3534</v>
+        <v>0</v>
       </c>
       <c r="E7" s="13">
         <f>SUMIFS('Compute &amp; sensors'!$H$2:$H$6,'Compute &amp; sensors'!$D$2:$D$6,"ordered")</f>
         <v>0</v>
       </c>
       <c r="F7" s="13">
-        <f>SUMIFS('Compute &amp; sensors'!$H$2:$H$6,'Compute &amp; sensors'!$D$2:$D$6,"to buy")</f>
-        <v>1189</v>
+        <f>C7-D7-E7</f>
+        <v>4723</v>
       </c>
     </row>
     <row r="8">
@@ -651,7 +651,7 @@
         <v>0</v>
       </c>
       <c r="F8" s="13">
-        <f>SUMIFS('Power'!$H$2:$H$15,'Power'!$D$2:$D$15,"to buy")</f>
+        <f>C8-D8-E8</f>
         <v>1633.05</v>
       </c>
     </row>
@@ -678,7 +678,7 @@
         <v>0</v>
       </c>
       <c r="F9" s="13">
-        <f>SUMIFS('Electronics &amp; wiring'!$H$2:$H$11,'Electronics &amp; wiring'!$D$2:$D$11,"to buy")</f>
+        <f>C9-D9-E9</f>
         <v>808</v>
       </c>
     </row>
@@ -705,7 +705,7 @@
         <v>0</v>
       </c>
       <c r="F10" s="13">
-        <f>SUMIFS('Structure &amp; materials'!$H$2:$H$14,'Structure &amp; materials'!$D$2:$D$14,"to buy")</f>
+        <f>C10-D10-E10</f>
         <v>2582</v>
       </c>
     </row>
@@ -732,7 +732,7 @@
         <v>0</v>
       </c>
       <c r="F11" s="13">
-        <f>SUMIFS('Fasteners'!$H$2:$H$2,'Fasteners'!$D$2:$D$2,"to buy")</f>
+        <f>C11-D11-E11</f>
         <v>180</v>
       </c>
     </row>
@@ -759,7 +759,7 @@
         <v>0</v>
       </c>
       <c r="F12" s="13">
-        <f>SUMIFS('Tooling'!$H$2:$H$6,'Tooling'!$D$2:$D$6,"to buy")</f>
+        <f>C12-D12-E12</f>
         <v>710</v>
       </c>
     </row>
@@ -786,7 +786,7 @@
         <v>0</v>
       </c>
       <c r="F13" s="13">
-        <f>SUMIFS('Safety'!$H$2:$H$5,'Safety'!$D$2:$D$5,"to buy")</f>
+        <f>C13-D13-E13</f>
         <v>470</v>
       </c>
     </row>
@@ -806,7 +806,7 @@
       </c>
       <c r="D14" s="14">
         <f>SUM(D5:D13)</f>
-        <v>3732</v>
+        <v>0</v>
       </c>
       <c r="E14" s="14">
         <f>SUM(E5:E13)</f>
@@ -814,7 +814,7 @@
       </c>
       <c r="F14" s="14">
         <f>SUM(F5:F13)</f>
-        <v>13799.03</v>
+        <v>17531.03</v>
       </c>
     </row>
     <row r="16" ht="48" customHeight="1">
@@ -923,11 +923,6 @@
           <t>Fall padding foam</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E2" s="9" t="n">
         <v>1</v>
       </c>
@@ -959,11 +954,6 @@
           <t>Gantry frame; harness and hoist</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E3" s="9" t="n">
         <v>1</v>
       </c>
@@ -995,11 +985,6 @@
           <t>Latching e-stop button and contactor driver</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E4" s="9" t="n">
         <v>1</v>
       </c>
@@ -1029,11 +1014,6 @@
       <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Wireless e-stop: handheld transmitter; receiver and watchdog relay</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>to buy</t>
         </is>
       </c>
       <c r="E5" s="9" t="n">
@@ -1083,7 +1063,7 @@
   </sheetData>
   <autoFilter ref="A1:K5"/>
   <dataValidations count="1">
-    <dataValidation sqref="D2:D5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="Choose one of: to buy, ordered, owned" type="list">
+    <dataValidation sqref="D2:D5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose one of: to buy, ordered, owned" type="list">
       <formula1>"to buy,ordered,owned"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2427,7 +2407,7 @@
   </sheetData>
   <autoFilter ref="A1:J29"/>
   <dataValidations count="1">
-    <dataValidation sqref="I2:I29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="Choose one of: yes, no" type="list">
+    <dataValidation sqref="I2:I29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose one of: yes, no" type="list">
       <formula1>"yes,no"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2576,11 +2556,6 @@
           <t>battery connector, cradle half (AS150 class), at the front of the battery bay</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K2" s="2" t="n"/>
     </row>
     <row r="3">
@@ -2615,11 +2590,6 @@
           <t>arm power and signal connectors</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K3" s="2" t="n"/>
     </row>
     <row r="4">
@@ -2654,11 +2624,6 @@
           <t>leg power (XT60 class) and signal connectors</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K4" s="2" t="n"/>
     </row>
     <row r="5">
@@ -2693,11 +2658,6 @@
           <t>isolated USB-CAN adapter</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K5" s="2" t="n"/>
     </row>
     <row r="6">
@@ -2732,11 +2692,6 @@
           <t>isolated USB-CAN adapter</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K6" s="2" t="n"/>
     </row>
     <row r="7">
@@ -2771,11 +2726,6 @@
           <t>isolated USB-CAN adapter</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K7" s="2" t="n"/>
     </row>
     <row r="8">
@@ -2810,11 +2760,6 @@
           <t>main contactor, 48 V DC, opened by the e-stop chain</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K8" s="2" t="n"/>
     </row>
     <row r="9">
@@ -2849,11 +2794,6 @@
           <t>DC-DC 48 V to 19-20 V, 120 W+, ahead of the contactor</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K9" s="2" t="n"/>
     </row>
     <row r="10">
@@ -2888,11 +2828,6 @@
           <t>DC-DC 48 V to 12 V, 10 A (servos)</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K10" s="2" t="n"/>
     </row>
     <row r="11">
@@ -2927,11 +2862,6 @@
           <t>wireless e-stop receiver and watchdog relay</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K11" s="2" t="n"/>
     </row>
     <row r="12">
@@ -2966,11 +2896,6 @@
           <t>harness allowance: pelvis (limb-root connectors on the bulkheads)</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K12" s="2" t="n"/>
     </row>
     <row r="13">
@@ -3005,11 +2930,6 @@
           <t>harness allowance: torso (limb-root connectors on the bulkheads)</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K13" s="2" t="n"/>
     </row>
     <row r="14">
@@ -3044,11 +2964,6 @@
           <t>IMU on the pelvis, near the hip axes</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K14" s="2" t="n"/>
     </row>
     <row r="15">
@@ -3083,11 +2998,6 @@
           <t>pelvis power board: leg branch fuses</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K15" s="2" t="n"/>
     </row>
     <row r="16">
@@ -3122,11 +3032,6 @@
           <t>torso power board: bus bars, arm branch fuses</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K16" s="2" t="n"/>
     </row>
     <row r="17">
@@ -3161,11 +3066,6 @@
           <t>precharge resistor and relay, across the contactor</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K17" s="2" t="n"/>
     </row>
     <row r="18">
@@ -3196,11 +3096,6 @@
         </is>
       </c>
       <c r="I18" s="2" t="n"/>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K18" s="2" t="n"/>
     </row>
     <row r="19">
@@ -3235,11 +3130,6 @@
           <t>steel tube with two M6 rod ends</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K19" s="2" t="n"/>
     </row>
     <row r="20">
@@ -3274,11 +3164,6 @@
           <t>steel tube with two M6 rod ends</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K20" s="2" t="n"/>
     </row>
     <row r="21">
@@ -3313,11 +3198,6 @@
           <t>AmazingHand by Pollen Robotics (CC-BY-4.0), description/third_party/amazing_hand</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K21" s="2" t="n"/>
     </row>
     <row r="22">
@@ -3352,11 +3232,6 @@
           <t>6806-2RS far-side bearing</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K22" s="2" t="n"/>
     </row>
     <row r="23">
@@ -3391,11 +3266,6 @@
           <t>6806-2RS far-side bearing</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K23" s="2" t="n"/>
     </row>
     <row r="24">
@@ -3430,11 +3300,6 @@
           <t>6806-2RS far-side bearing</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K24" s="2" t="n"/>
     </row>
     <row r="25">
@@ -3473,11 +3338,6 @@
         </is>
       </c>
       <c r="I25" s="2" t="n"/>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K25" s="2" t="n"/>
     </row>
     <row r="26">
@@ -3516,11 +3376,6 @@
         </is>
       </c>
       <c r="I26" s="2" t="n"/>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K26" s="2" t="n"/>
     </row>
     <row r="27">
@@ -3559,11 +3414,6 @@
         </is>
       </c>
       <c r="I27" s="2" t="n"/>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K27" s="2" t="n"/>
     </row>
     <row r="28">
@@ -3602,11 +3452,6 @@
         </is>
       </c>
       <c r="I28" s="2" t="n"/>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K28" s="2" t="n"/>
     </row>
     <row r="29">
@@ -3645,11 +3490,6 @@
         </is>
       </c>
       <c r="I29" s="2" t="n"/>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K29" s="2" t="n"/>
     </row>
     <row r="30">
@@ -3688,11 +3528,6 @@
         </is>
       </c>
       <c r="I30" s="2" t="n"/>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K30" s="2" t="n"/>
     </row>
     <row r="31">
@@ -3731,11 +3566,6 @@
         </is>
       </c>
       <c r="I31" s="2" t="n"/>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K31" s="2" t="n"/>
     </row>
     <row r="32">
@@ -3774,11 +3604,6 @@
         </is>
       </c>
       <c r="I32" s="2" t="n"/>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K32" s="2" t="n"/>
     </row>
     <row r="33">
@@ -3817,11 +3642,6 @@
         </is>
       </c>
       <c r="I33" s="2" t="n"/>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K33" s="2" t="n"/>
     </row>
     <row r="34">
@@ -3860,11 +3680,6 @@
         </is>
       </c>
       <c r="I34" s="2" t="n"/>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K34" s="2" t="n"/>
     </row>
     <row r="35">
@@ -3903,11 +3718,6 @@
         </is>
       </c>
       <c r="I35" s="2" t="n"/>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K35" s="2" t="n"/>
     </row>
     <row r="36">
@@ -3946,11 +3756,6 @@
         </is>
       </c>
       <c r="I36" s="2" t="n"/>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K36" s="2" t="n"/>
     </row>
     <row r="37">
@@ -3989,11 +3794,6 @@
         </is>
       </c>
       <c r="I37" s="2" t="n"/>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K37" s="2" t="n"/>
     </row>
     <row r="38">
@@ -4032,11 +3832,6 @@
         </is>
       </c>
       <c r="I38" s="2" t="n"/>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K38" s="2" t="n"/>
     </row>
     <row r="39">
@@ -4075,11 +3870,6 @@
         </is>
       </c>
       <c r="I39" s="2" t="n"/>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K39" s="2" t="n"/>
     </row>
     <row r="40">
@@ -4118,11 +3908,6 @@
         </is>
       </c>
       <c r="I40" s="2" t="n"/>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K40" s="2" t="n"/>
     </row>
     <row r="41">
@@ -4161,11 +3946,6 @@
         </is>
       </c>
       <c r="I41" s="2" t="n"/>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K41" s="2" t="n"/>
     </row>
     <row r="42">
@@ -4204,11 +3984,6 @@
         </is>
       </c>
       <c r="I42" s="2" t="n"/>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K42" s="2" t="n"/>
     </row>
     <row r="43">
@@ -4247,11 +4022,6 @@
         </is>
       </c>
       <c r="I43" s="2" t="n"/>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K43" s="2" t="n"/>
     </row>
     <row r="44">
@@ -4290,11 +4060,6 @@
         </is>
       </c>
       <c r="I44" s="2" t="n"/>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K44" s="2" t="n"/>
     </row>
     <row r="45">
@@ -4333,11 +4098,6 @@
         </is>
       </c>
       <c r="I45" s="2" t="n"/>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K45" s="2" t="n"/>
     </row>
     <row r="46">
@@ -4376,11 +4136,6 @@
         </is>
       </c>
       <c r="I46" s="2" t="n"/>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K46" s="2" t="n"/>
     </row>
     <row r="47">
@@ -4419,11 +4174,6 @@
         </is>
       </c>
       <c r="I47" s="2" t="n"/>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K47" s="2" t="n"/>
     </row>
     <row r="48">
@@ -4462,11 +4212,6 @@
         </is>
       </c>
       <c r="I48" s="2" t="n"/>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K48" s="2" t="n"/>
     </row>
     <row r="49">
@@ -4505,11 +4250,6 @@
         </is>
       </c>
       <c r="I49" s="2" t="n"/>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K49" s="2" t="n"/>
     </row>
     <row r="50">
@@ -4548,11 +4288,6 @@
         </is>
       </c>
       <c r="I50" s="2" t="n"/>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K50" s="2" t="n"/>
     </row>
     <row r="51">
@@ -4591,11 +4326,6 @@
         </is>
       </c>
       <c r="I51" s="2" t="n"/>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K51" s="2" t="n"/>
     </row>
     <row r="52">
@@ -4634,11 +4364,6 @@
         </is>
       </c>
       <c r="I52" s="2" t="n"/>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K52" s="2" t="n"/>
     </row>
     <row r="53">
@@ -4677,11 +4402,6 @@
         </is>
       </c>
       <c r="I53" s="2" t="n"/>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K53" s="2" t="n"/>
     </row>
     <row r="54">
@@ -4720,11 +4440,6 @@
         </is>
       </c>
       <c r="I54" s="2" t="n"/>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K54" s="2" t="n"/>
     </row>
     <row r="55">
@@ -4763,11 +4478,6 @@
         </is>
       </c>
       <c r="I55" s="2" t="n"/>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K55" s="2" t="n"/>
     </row>
     <row r="56">
@@ -4806,11 +4516,6 @@
         </is>
       </c>
       <c r="I56" s="2" t="n"/>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K56" s="2" t="n"/>
     </row>
     <row r="57">
@@ -4849,11 +4554,6 @@
         </is>
       </c>
       <c r="I57" s="2" t="n"/>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K57" s="2" t="n"/>
     </row>
     <row r="58">
@@ -4892,11 +4592,6 @@
         </is>
       </c>
       <c r="I58" s="2" t="n"/>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K58" s="2" t="n"/>
     </row>
     <row r="59">
@@ -4935,11 +4630,6 @@
         </is>
       </c>
       <c r="I59" s="2" t="n"/>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K59" s="2" t="n"/>
     </row>
     <row r="60">
@@ -4978,11 +4668,6 @@
         </is>
       </c>
       <c r="I60" s="2" t="n"/>
-      <c r="J60" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K60" s="2" t="n"/>
     </row>
     <row r="61">
@@ -5021,11 +4706,6 @@
         </is>
       </c>
       <c r="I61" s="2" t="n"/>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K61" s="2" t="n"/>
     </row>
     <row r="62">
@@ -5064,11 +4744,6 @@
         </is>
       </c>
       <c r="I62" s="2" t="n"/>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K62" s="2" t="n"/>
     </row>
     <row r="63">
@@ -5107,11 +4782,6 @@
         </is>
       </c>
       <c r="I63" s="2" t="n"/>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K63" s="2" t="n"/>
     </row>
     <row r="64">
@@ -5150,11 +4820,6 @@
         </is>
       </c>
       <c r="I64" s="2" t="n"/>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K64" s="2" t="n"/>
     </row>
     <row r="65">
@@ -5193,11 +4858,6 @@
         </is>
       </c>
       <c r="I65" s="2" t="n"/>
-      <c r="J65" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K65" s="2" t="n"/>
     </row>
     <row r="66">
@@ -5236,11 +4896,6 @@
         </is>
       </c>
       <c r="I66" s="2" t="n"/>
-      <c r="J66" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K66" s="2" t="n"/>
     </row>
     <row r="67">
@@ -5279,11 +4934,6 @@
         </is>
       </c>
       <c r="I67" s="2" t="n"/>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K67" s="2" t="n"/>
     </row>
     <row r="68">
@@ -5322,11 +4972,6 @@
         </is>
       </c>
       <c r="I68" s="2" t="n"/>
-      <c r="J68" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K68" s="2" t="n"/>
     </row>
     <row r="69">
@@ -5365,11 +5010,6 @@
         </is>
       </c>
       <c r="I69" s="2" t="n"/>
-      <c r="J69" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K69" s="2" t="n"/>
     </row>
     <row r="70">
@@ -5408,11 +5048,6 @@
         </is>
       </c>
       <c r="I70" s="2" t="n"/>
-      <c r="J70" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K70" s="2" t="n"/>
     </row>
     <row r="71">
@@ -5451,11 +5086,6 @@
         </is>
       </c>
       <c r="I71" s="2" t="n"/>
-      <c r="J71" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K71" s="2" t="n"/>
     </row>
     <row r="72">
@@ -5494,11 +5124,6 @@
         </is>
       </c>
       <c r="I72" s="2" t="n"/>
-      <c r="J72" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K72" s="2" t="n"/>
     </row>
     <row r="73">
@@ -5537,11 +5162,6 @@
         </is>
       </c>
       <c r="I73" s="2" t="n"/>
-      <c r="J73" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K73" s="2" t="n"/>
     </row>
     <row r="74">
@@ -5580,11 +5200,6 @@
         </is>
       </c>
       <c r="I74" s="2" t="n"/>
-      <c r="J74" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K74" s="2" t="n"/>
     </row>
     <row r="75">
@@ -5623,11 +5238,6 @@
         </is>
       </c>
       <c r="I75" s="2" t="n"/>
-      <c r="J75" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K75" s="2" t="n"/>
     </row>
     <row r="76">
@@ -5666,11 +5276,6 @@
         </is>
       </c>
       <c r="I76" s="2" t="n"/>
-      <c r="J76" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K76" s="2" t="n"/>
     </row>
     <row r="77">
@@ -5709,11 +5314,6 @@
         </is>
       </c>
       <c r="I77" s="2" t="n"/>
-      <c r="J77" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K77" s="2" t="n"/>
     </row>
     <row r="78">
@@ -5752,11 +5352,6 @@
         </is>
       </c>
       <c r="I78" s="2" t="n"/>
-      <c r="J78" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K78" s="2" t="n"/>
     </row>
     <row r="79">
@@ -5792,11 +5387,6 @@
         </is>
       </c>
       <c r="I79" s="2" t="n"/>
-      <c r="J79" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K79" s="2" t="n"/>
     </row>
     <row r="80">
@@ -5832,11 +5422,6 @@
         </is>
       </c>
       <c r="I80" s="2" t="n"/>
-      <c r="J80" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K80" s="2" t="n"/>
     </row>
     <row r="81">
@@ -5872,11 +5457,6 @@
         </is>
       </c>
       <c r="I81" s="2" t="n"/>
-      <c r="J81" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K81" s="2" t="n"/>
     </row>
     <row r="82">
@@ -5912,11 +5492,6 @@
         </is>
       </c>
       <c r="I82" s="2" t="n"/>
-      <c r="J82" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K82" s="2" t="n"/>
     </row>
     <row r="83">
@@ -5952,11 +5527,6 @@
         </is>
       </c>
       <c r="I83" s="2" t="n"/>
-      <c r="J83" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K83" s="2" t="n"/>
     </row>
     <row r="84">
@@ -5992,11 +5562,6 @@
         </is>
       </c>
       <c r="I84" s="2" t="n"/>
-      <c r="J84" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K84" s="2" t="n"/>
     </row>
     <row r="85">
@@ -6032,11 +5597,6 @@
         </is>
       </c>
       <c r="I85" s="2" t="n"/>
-      <c r="J85" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K85" s="2" t="n"/>
     </row>
     <row r="86">
@@ -6072,11 +5632,6 @@
         </is>
       </c>
       <c r="I86" s="2" t="n"/>
-      <c r="J86" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K86" s="2" t="n"/>
     </row>
     <row r="87">
@@ -6112,11 +5667,6 @@
         </is>
       </c>
       <c r="I87" s="2" t="n"/>
-      <c r="J87" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K87" s="2" t="n"/>
     </row>
     <row r="88">
@@ -6152,11 +5702,6 @@
         </is>
       </c>
       <c r="I88" s="2" t="n"/>
-      <c r="J88" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K88" s="2" t="n"/>
     </row>
     <row r="89">
@@ -6192,11 +5737,6 @@
         </is>
       </c>
       <c r="I89" s="2" t="n"/>
-      <c r="J89" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K89" s="2" t="n"/>
     </row>
     <row r="90">
@@ -6232,11 +5772,6 @@
         </is>
       </c>
       <c r="I90" s="2" t="n"/>
-      <c r="J90" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K90" s="2" t="n"/>
     </row>
     <row r="91">
@@ -6272,11 +5807,6 @@
         </is>
       </c>
       <c r="I91" s="2" t="n"/>
-      <c r="J91" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K91" s="2" t="n"/>
     </row>
     <row r="92">
@@ -6312,11 +5842,6 @@
         </is>
       </c>
       <c r="I92" s="2" t="n"/>
-      <c r="J92" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K92" s="2" t="n"/>
     </row>
     <row r="93">
@@ -6352,11 +5877,6 @@
         </is>
       </c>
       <c r="I93" s="2" t="n"/>
-      <c r="J93" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K93" s="2" t="n"/>
     </row>
     <row r="94">
@@ -6392,11 +5912,6 @@
         </is>
       </c>
       <c r="I94" s="2" t="n"/>
-      <c r="J94" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K94" s="2" t="n"/>
     </row>
     <row r="95">
@@ -6432,11 +5947,6 @@
         </is>
       </c>
       <c r="I95" s="2" t="n"/>
-      <c r="J95" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K95" s="2" t="n"/>
     </row>
     <row r="96">
@@ -6472,11 +5982,6 @@
         </is>
       </c>
       <c r="I96" s="2" t="n"/>
-      <c r="J96" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K96" s="2" t="n"/>
     </row>
     <row r="97">
@@ -6512,11 +6017,6 @@
         </is>
       </c>
       <c r="I97" s="2" t="n"/>
-      <c r="J97" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K97" s="2" t="n"/>
     </row>
     <row r="98">
@@ -6552,11 +6052,6 @@
         </is>
       </c>
       <c r="I98" s="2" t="n"/>
-      <c r="J98" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K98" s="2" t="n"/>
     </row>
     <row r="99">
@@ -6592,11 +6087,6 @@
         </is>
       </c>
       <c r="I99" s="2" t="n"/>
-      <c r="J99" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K99" s="2" t="n"/>
     </row>
     <row r="100">
@@ -6632,11 +6122,6 @@
         </is>
       </c>
       <c r="I100" s="2" t="n"/>
-      <c r="J100" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K100" s="2" t="n"/>
     </row>
     <row r="101">
@@ -6672,11 +6157,6 @@
         </is>
       </c>
       <c r="I101" s="2" t="n"/>
-      <c r="J101" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K101" s="2" t="n"/>
     </row>
     <row r="102">
@@ -6712,11 +6192,6 @@
         </is>
       </c>
       <c r="I102" s="2" t="n"/>
-      <c r="J102" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K102" s="2" t="n"/>
     </row>
     <row r="103">
@@ -6752,11 +6227,6 @@
         </is>
       </c>
       <c r="I103" s="2" t="n"/>
-      <c r="J103" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K103" s="2" t="n"/>
     </row>
     <row r="104">
@@ -6792,11 +6262,6 @@
         </is>
       </c>
       <c r="I104" s="2" t="n"/>
-      <c r="J104" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K104" s="2" t="n"/>
     </row>
     <row r="105">
@@ -6832,11 +6297,6 @@
         </is>
       </c>
       <c r="I105" s="2" t="n"/>
-      <c r="J105" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K105" s="2" t="n"/>
     </row>
     <row r="106">
@@ -6872,11 +6332,6 @@
         </is>
       </c>
       <c r="I106" s="2" t="n"/>
-      <c r="J106" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K106" s="2" t="n"/>
     </row>
     <row r="107">
@@ -6912,11 +6367,6 @@
         </is>
       </c>
       <c r="I107" s="2" t="n"/>
-      <c r="J107" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K107" s="2" t="n"/>
     </row>
     <row r="108">
@@ -6955,11 +6405,6 @@
         </is>
       </c>
       <c r="I108" s="2" t="n"/>
-      <c r="J108" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K108" s="2" t="n"/>
     </row>
     <row r="109">
@@ -6998,11 +6443,6 @@
         </is>
       </c>
       <c r="I109" s="2" t="n"/>
-      <c r="J109" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K109" s="2" t="n"/>
     </row>
     <row r="110">
@@ -7041,11 +6481,6 @@
         </is>
       </c>
       <c r="I110" s="2" t="n"/>
-      <c r="J110" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K110" s="2" t="n"/>
     </row>
     <row r="111">
@@ -7084,11 +6519,6 @@
         </is>
       </c>
       <c r="I111" s="2" t="n"/>
-      <c r="J111" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K111" s="2" t="n"/>
     </row>
     <row r="112">
@@ -7127,11 +6557,6 @@
         </is>
       </c>
       <c r="I112" s="2" t="n"/>
-      <c r="J112" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K112" s="2" t="n"/>
     </row>
     <row r="113">
@@ -7170,11 +6595,6 @@
         </is>
       </c>
       <c r="I113" s="2" t="n"/>
-      <c r="J113" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K113" s="2" t="n"/>
     </row>
     <row r="114">
@@ -7213,17 +6633,12 @@
         </is>
       </c>
       <c r="I114" s="2" t="n"/>
-      <c r="J114" t="inlineStr">
-        <is>
-          <t>to make</t>
-        </is>
-      </c>
       <c r="K114" s="2" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:K114"/>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J114" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="Choose one of: to make, ordered, made" type="list">
+    <dataValidation sqref="J2:J114" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose one of: to make, ordered, made" type="list">
       <formula1>"to make,ordered,made"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7304,11 +6719,6 @@
           <t>socket head, 12.9; length = plate + thread engagement, per part</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -7334,11 +6744,6 @@
           <t>socket head, 12.9; length = plate + thread engagement, per part</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -7364,11 +6769,6 @@
           <t>socket head, 12.9; length = plate + thread engagement, per part</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -7394,11 +6794,6 @@
           <t>socket head, 12.9; length = plate + thread engagement, per part</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -7424,11 +6819,6 @@
           <t>socket head, 12.9; length = plate + thread engagement, per part</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -7454,11 +6844,6 @@
           <t>socket head, 12.9; length = plate + thread engagement, per part</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -7484,11 +6869,6 @@
           <t>socket head, 12.9; length = plate + thread engagement, per part</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -7512,18 +6892,13 @@
       <c r="E9" s="2" t="inlineStr">
         <is>
           <t>socket head, 12.9; length = plate + thread engagement, per part</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>to buy</t>
         </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:F9"/>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="Choose one of: to buy, ordered, owned" type="list">
+    <dataValidation sqref="F2:F9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose one of: to buy, ordered, owned" type="list">
       <formula1>"to buy,ordered,owned"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7626,11 +7001,6 @@
           <t>STS3250</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E2" s="9" t="n">
         <v>4</v>
       </c>
@@ -7676,11 +7046,6 @@
           <t>RS00</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E3" s="9" t="n">
         <v>2</v>
       </c>
@@ -7726,11 +7091,6 @@
           <t>RS03</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E4" s="9" t="n">
         <v>11</v>
       </c>
@@ -7776,11 +7136,6 @@
           <t>RS04</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E5" s="9" t="n">
         <v>6</v>
       </c>
@@ -7824,11 +7179,6 @@
       <c r="C6" t="inlineStr">
         <is>
           <t>RS06</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>to buy</t>
         </is>
       </c>
       <c r="E6" s="9" t="n">
@@ -7883,7 +7233,7 @@
   </sheetData>
   <autoFilter ref="A1:K6"/>
   <dataValidations count="1">
-    <dataValidation sqref="D2:D6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="Choose one of: to buy, ordered, owned" type="list">
+    <dataValidation sqref="D2:D6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose one of: to buy, ordered, owned" type="list">
       <formula1>"to buy,ordered,owned"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7988,11 +7338,6 @@
           <t>AmazingHand open-source 8-DOF four-finger hand kit, left and right (8 Feetech SCS0009 servos each, 5 V)</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>owned</t>
-        </is>
-      </c>
       <c r="E2" s="9" t="n">
         <v>2</v>
       </c>
@@ -8018,7 +7363,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>owned by this build; the listing does not say what is in the box, so check that servos are included. 0.40 kg each as published (weigh); its design is CC-BY-4.0, see ACKNOWLEDGMENTS.md</t>
+          <t>the listing does not say what is in the box, so check that servos are included. 0.40 kg each as published (weigh); its design is CC-BY-4.0, see ACKNOWLEDGMENTS.md</t>
         </is>
       </c>
     </row>
@@ -8031,11 +7376,6 @@
       <c r="B3" s="2" t="inlineStr">
         <is>
           <t>DC-DC 12 V to 5 V, 3 A, small (in the wrist)</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>to buy</t>
         </is>
       </c>
       <c r="E3" s="9" t="n">
@@ -8071,11 +7411,6 @@
       <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Feetech serial-bus USB adapter (Waveshare Bus Servo Adapter (A) class)</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>to buy</t>
         </is>
       </c>
       <c r="E4" s="9" t="n">
@@ -8130,7 +7465,7 @@
   </sheetData>
   <autoFilter ref="A1:K4"/>
   <dataValidations count="1">
-    <dataValidation sqref="D2:D4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="Choose one of: to buy, ordered, owned" type="list">
+    <dataValidation sqref="D2:D4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose one of: to buy, ordered, owned" type="list">
       <formula1>"to buy,ordered,owned"</formula1>
     </dataValidation>
   </dataValidations>
@@ -8232,11 +7567,6 @@
           <t>Jetson AGX Orin 64 GB developer kit</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>owned</t>
-        </is>
-      </c>
       <c r="E2" s="9" t="n">
         <v>1</v>
       </c>
@@ -8260,11 +7590,7 @@
           <t>https://marketplace.nvidia.com/en-us/enterprise/robotics-edge/jetson-agx-orin-developer-kit/</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>owned by this build; a replicator buys it</t>
-        </is>
-      </c>
+      <c r="K2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -8275,11 +7601,6 @@
       <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Low-cost USB AHRS IMU</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>owned</t>
         </is>
       </c>
       <c r="E3" s="9" t="n">
@@ -8317,11 +7638,6 @@
           <t>NVMe SSD, 1 TB, M.2 2280</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E4" s="9" t="n">
         <v>1</v>
       </c>
@@ -8357,11 +7673,6 @@
           <t>Orbbec Gemini 335L depth camera</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E5" s="9" t="n">
         <v>1</v>
       </c>
@@ -8400,11 +7711,6 @@
       <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Primary IMU (industrial AHRS; or BMI088 on a microcontroller)</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>to buy</t>
         </is>
       </c>
       <c r="E6" s="9" t="n">
@@ -8454,7 +7760,7 @@
   </sheetData>
   <autoFilter ref="A1:K6"/>
   <dataValidations count="1">
-    <dataValidation sqref="D2:D6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="Choose one of: to buy, ordered, owned" type="list">
+    <dataValidation sqref="D2:D6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose one of: to buy, ordered, owned" type="list">
       <formula1>"to buy,ordered,owned"</formula1>
     </dataValidation>
   </dataValidations>
@@ -8556,11 +7862,6 @@
           <t>13S charger adjustable to 4.1 V per cell</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E2" s="9" t="n">
         <v>1</v>
       </c>
@@ -8596,11 +7897,6 @@
           <t>13S smart BMS 150 A with CAN telemetry</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E3" s="9" t="n">
         <v>1</v>
       </c>
@@ -8641,11 +7937,6 @@
           <t>48 V 20 A bench power supply</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E4" s="9" t="n">
         <v>1</v>
       </c>
@@ -8681,11 +7972,6 @@
           <t>Anti-spark blind-mate battery connector (AS150 class)</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E5" s="9" t="n">
         <v>2</v>
       </c>
@@ -8721,11 +8007,6 @@
           <t>Class-T fuse 100-125 A with holder; limb branch fuses</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E6" s="9" t="n">
         <v>1</v>
       </c>
@@ -8757,11 +8038,6 @@
           <t>DC-DC 48 V to 12 V, 10 A, compact (at most 60 x 34 x 25 mm)</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E7" s="9" t="n">
         <v>1</v>
       </c>
@@ -8797,11 +8073,6 @@
           <t>DC-DC 75 V-input to 19-20 V; at least 120 W (computer)</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E8" s="9" t="n">
         <v>1</v>
       </c>
@@ -8837,11 +8108,6 @@
           <t>Ideal-diode OR circuit (LTC4359 class) for the computer rail</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E9" s="9" t="n">
         <v>1</v>
       </c>
@@ -8873,11 +8139,6 @@
           <t>Keep-alive battery 50-100 Wh for the computer</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E10" s="9" t="n">
         <v>1</v>
       </c>
@@ -8913,11 +8174,6 @@
           <t>Main contactor (48 V DC rated)</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E11" s="9" t="n">
         <v>1</v>
       </c>
@@ -8953,11 +8209,6 @@
           <t>Molicel P45B 21700 cells</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E12" s="9" t="n">
         <v>39</v>
       </c>
@@ -8998,11 +8249,6 @@
           <t>Pack housing; nickel strip; quick-release cradle</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E13" s="9" t="n">
         <v>1</v>
       </c>
@@ -9034,11 +8280,6 @@
           <t>Precharge resistor and relay</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E14" s="9" t="n">
         <v>1</v>
       </c>
@@ -9068,11 +8309,6 @@
       <c r="B15" s="2" t="inlineStr">
         <is>
           <t>Regen clamp (brake resistor chopper or TVS ~56-58 V)</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>to buy</t>
         </is>
       </c>
       <c r="E15" s="9" t="n">
@@ -9122,7 +8358,7 @@
   </sheetData>
   <autoFilter ref="A1:K15"/>
   <dataValidations count="1">
-    <dataValidation sqref="D2:D15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="Choose one of: to buy, ordered, owned" type="list">
+    <dataValidation sqref="D2:D15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose one of: to buy, ordered, owned" type="list">
       <formula1>"to buy,ordered,owned"</formula1>
     </dataValidation>
   </dataValidations>
@@ -9224,11 +8460,6 @@
           <t>3.3 V CAN transceiver boards for the Orin's on-board CAN</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E2" s="9" t="n">
         <v>2</v>
       </c>
@@ -9264,11 +8495,6 @@
           <t>Compact USB 3 hub, 4-port</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E3" s="9" t="n">
         <v>1</v>
       </c>
@@ -9304,11 +8530,6 @@
           <t>Feetech serial-bus USB adapter (Waveshare Bus Servo Adapter (A) class)</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E4" s="9" t="n">
         <v>1</v>
       </c>
@@ -9349,11 +8570,6 @@
           <t>Isolated USB-CAN adapter, dual channel (InnoMaker USB2CAN-X2 class; SocketCAN)</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E5" s="9" t="n">
         <v>2</v>
       </c>
@@ -9394,11 +8610,6 @@
           <t>Isolated USB-CAN adapter, single channel (CANable Pro class; candleLight / gs_usb)</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E6" s="9" t="n">
         <v>2</v>
       </c>
@@ -9439,11 +8650,6 @@
           <t>Limb-root connectors: XT60-class power pair and latching signal pair, per limb</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E7" s="9" t="n">
         <v>4</v>
       </c>
@@ -9479,11 +8685,6 @@
           <t>RobStride USB-to-CAN debug adapter (official GUI tool)</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E8" s="9" t="n">
         <v>1</v>
       </c>
@@ -9524,11 +8725,6 @@
           <t>Silicone wire; connectors; strain relief; sleeving</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E9" s="9" t="n">
         <v>1</v>
       </c>
@@ -9560,11 +8756,6 @@
           <t>Twisted-pair CAN cable, connectors and 120 Ω terminations</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E10" s="9" t="n">
         <v>1</v>
       </c>
@@ -9594,11 +8785,6 @@
       <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Wireless gamepad</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>to buy</t>
         </is>
       </c>
       <c r="E11" s="9" t="n">
@@ -9644,7 +8830,7 @@
   </sheetData>
   <autoFilter ref="A1:K11"/>
   <dataValidations count="1">
-    <dataValidation sqref="D2:D11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="Choose one of: to buy, ordered, owned" type="list">
+    <dataValidation sqref="D2:D11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose one of: to buy, ordered, owned" type="list">
       <formula1>"to buy,ordered,owned"</formula1>
     </dataValidation>
   </dataValidations>
@@ -9748,11 +8934,6 @@
           <t>6061-T6 aluminium plate and bar stock</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E2" s="9" t="n">
         <v>1</v>
       </c>
@@ -9788,11 +8969,6 @@
           <t>6806-2RS thin-section ball bearing (30 x 42 x 7 mm) for far-side joint support</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E3" s="9" t="n">
         <v>6</v>
       </c>
@@ -9833,11 +9009,6 @@
           <t>7075-T6 bar for highly loaded flanges and ankle cranks</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E4" s="9" t="n">
         <v>1</v>
       </c>
@@ -9869,11 +9040,6 @@
           <t>Aluminium and filament for torso; arms; head</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E5" s="9" t="n">
         <v>1</v>
       </c>
@@ -9905,11 +9071,6 @@
           <t>Ankle push rods (steel tube with threaded inserts)</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E6" s="9" t="n">
         <v>4</v>
       </c>
@@ -9945,11 +9106,6 @@
           <t>Carbon-fibre nylon filament (kg)</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E7" s="9" t="n">
         <v>4</v>
       </c>
@@ -9985,11 +9141,6 @@
           <t>Crossed-roller bearing for the waist</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E8" s="9" t="n">
         <v>1</v>
       </c>
@@ -10021,11 +9172,6 @@
           <t>M6 steel-ball rod ends for ankle push rods</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E9" s="9" t="n">
         <v>8</v>
       </c>
@@ -10061,11 +9207,6 @@
           <t>Online machining: pelvis back (20 mm, 3D), pelvis top and two gussets (6 mm plates)</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E10" s="9" t="n">
         <v>1</v>
       </c>
@@ -10101,11 +9242,6 @@
           <t>Online machining: shin inner and outer plates, foot bases (6 pocketed 4-5 mm 6061 plates)</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E11" s="9" t="n">
         <v>1</v>
       </c>
@@ -10141,11 +9277,6 @@
           <t>Online machining: two torso uprights (25 mm 6061; 3D)</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E12" s="9" t="n">
         <v>1</v>
       </c>
@@ -10181,11 +9312,6 @@
           <t>PETG-CF filament (kg)</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E13" s="9" t="n">
         <v>2</v>
       </c>
@@ -10219,11 +9345,6 @@
       <c r="B14" s="2" t="inlineStr">
         <is>
           <t>TPU 95A filament (kg)</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>to buy</t>
         </is>
       </c>
       <c r="E14" s="9" t="n">
@@ -10273,7 +9394,7 @@
   </sheetData>
   <autoFilter ref="A1:K14"/>
   <dataValidations count="1">
-    <dataValidation sqref="D2:D14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="Choose one of: to buy, ordered, owned" type="list">
+    <dataValidation sqref="D2:D14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose one of: to buy, ordered, owned" type="list">
       <formula1>"to buy,ordered,owned"</formula1>
     </dataValidation>
   </dataValidations>
@@ -10374,11 +9495,6 @@
           <t>Metric fasteners; heat-set inserts; dowel pins; threadlocker</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E2" s="9" t="n">
         <v>1</v>
       </c>
@@ -10426,7 +9542,7 @@
   </sheetData>
   <autoFilter ref="A1:K2"/>
   <dataValidations count="1">
-    <dataValidation sqref="D2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="Choose one of: to buy, ordered, owned" type="list">
+    <dataValidation sqref="D2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose one of: to buy, ordered, owned" type="list">
       <formula1>"to buy,ordered,owned"</formula1>
     </dataValidation>
   </dataValidations>
@@ -10524,11 +9640,6 @@
           <t>Battery spot welder and pack supplies (fish paper, insulating rings, Kapton)</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E2" s="9" t="n">
         <v>1</v>
       </c>
@@ -10564,11 +9675,6 @@
           <t>Carbide 3-flute end mills for aluminium (1/8 and 1/4 in)</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E3" s="9" t="n">
         <v>8</v>
       </c>
@@ -10600,11 +9706,6 @@
           <t>Hand tools: torque screwdriver and hex bits, crimp tools, multimeter, digital scale (5 kg x 1 g)</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E4" s="9" t="n">
         <v>1</v>
       </c>
@@ -10640,11 +9741,6 @@
           <t>Hardened-steel nozzle and filament dryer</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>to buy</t>
-        </is>
-      </c>
       <c r="E5" s="9" t="n">
         <v>1</v>
       </c>
@@ -10678,11 +9774,6 @@
       <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Single-leg test jig (aluminium extrusion)</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>to buy</t>
         </is>
       </c>
       <c r="E6" s="9" t="n">
@@ -10728,7 +9819,7 @@
   </sheetData>
   <autoFilter ref="A1:K6"/>
   <dataValidations count="1">
-    <dataValidation sqref="D2:D6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="Choose one of: to buy, ordered, owned" type="list">
+    <dataValidation sqref="D2:D6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose one of: to buy, ordered, owned" type="list">
       <formula1>"to buy,ordered,owned"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
CAD: lightened to 41.95 kg with covers, every metal part at SF 2.3 or better
- the pelvis box and rear gussets out (10 mm back plate instead), plates at
  SF 4 and up thinned or pocketed, the printed shells under the covers gone
- covers 1.0 mm, head shell 1.8 mm, TPU soles 3 mm
- cad/mounts.py: output_windows; thin rings pocketed only inside their screw
  circle; cad/fea.py checks cage strips through FEA-only bonded solids
- 41.16 kg bare, 41.95 kg with covers: tools/check_all.sh passes

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bom/bom.xlsx
+++ b/bom/bom.xlsx
@@ -32,7 +32,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Tooling'!$A$1:$K$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Safety'!$A$1:$K$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Sourcing'!$A$1:$J$29</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Made parts (CAD)'!$A$1:$K$143</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Made parts (CAD)'!$A$1:$K$142</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Actuator bolts (CAD)'!$A$1:$F$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2451,7 +2451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K143"/>
+  <dimension ref="A1:K142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3463,14 +3463,14 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>flat 10.0 mm</t>
+          <t>flat 10.5 mm</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G29" s="12" t="n">
-        <v>7.7</v>
+        <v>8.1</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
@@ -3501,14 +3501,14 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>flat 10.0 mm</t>
+          <t>flat 10.5 mm</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G30" s="12" t="n">
-        <v>7.7</v>
+        <v>8.1</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
@@ -3539,14 +3539,14 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>flat 10.0 mm</t>
+          <t>flat 10.5 mm</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G31" s="12" t="n">
-        <v>7.7</v>
+        <v>8.1</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
@@ -3577,14 +3577,14 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>flat 10.0 mm</t>
+          <t>flat 10.5 mm</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G32" s="12" t="n">
-        <v>7.7</v>
+        <v>8.1</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
@@ -3660,11 +3660,11 @@
         <v>8</v>
       </c>
       <c r="G34" s="12" t="n">
-        <v>40.3</v>
+        <v>41.1</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>64 x 36 x 8</t>
+          <t>66 x 36 x 8</t>
         </is>
       </c>
       <c r="I34" s="2" t="n"/>
@@ -3698,7 +3698,7 @@
         <v>20</v>
       </c>
       <c r="G35" s="12" t="n">
-        <v>28.5</v>
+        <v>29.2</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
@@ -3736,7 +3736,7 @@
         <v>20</v>
       </c>
       <c r="G36" s="12" t="n">
-        <v>28.5</v>
+        <v>29.2</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -3863,7 +3863,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>{side}_hip_pitch_back</t>
+          <t>{side}_hip_pitch_flange</t>
         </is>
       </c>
       <c r="B40" s="9" t="n">
@@ -3881,18 +3881,18 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>flat 4.0 mm</t>
+          <t>3D</t>
         </is>
       </c>
       <c r="F40" t="n">
         <v>4</v>
       </c>
       <c r="G40" s="12" t="n">
-        <v>50.2</v>
+        <v>42.4</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>71 x 66 x 4</t>
+          <t>80 x 80 x 4</t>
         </is>
       </c>
       <c r="I40" s="2" t="n"/>
@@ -3901,7 +3901,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>{side}_hip_pitch_flange</t>
+          <t>{side}_hip_pitch_inner</t>
         </is>
       </c>
       <c r="B41" s="9" t="n">
@@ -3919,18 +3919,18 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>3D</t>
+          <t>flat 4.0 mm</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G41" s="12" t="n">
-        <v>68.40000000000001</v>
+        <v>81</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>80 x 80 x 6</t>
+          <t>170 x 80 x 4</t>
         </is>
       </c>
       <c r="I41" s="2" t="n"/>
@@ -3939,7 +3939,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>{side}_hip_pitch_front</t>
+          <t>{side}_hip_pitch_stub</t>
         </is>
       </c>
       <c r="B42" s="9" t="n">
@@ -3957,18 +3957,18 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>flat 4.0 mm</t>
+          <t>flat 12.0 mm</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="G42" s="12" t="n">
-        <v>50.2</v>
+        <v>21</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>71 x 66 x 4</t>
+          <t>30 x 30 x 12</t>
         </is>
       </c>
       <c r="I42" s="2" t="n"/>
@@ -3977,7 +3977,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>{side}_hip_pitch_inner</t>
+          <t>{side}_shin_bridge_spacer</t>
         </is>
       </c>
       <c r="B43" s="9" t="n">
@@ -3995,18 +3995,18 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>flat 4.0 mm</t>
+          <t>flat 2.0 mm</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G43" s="12" t="n">
-        <v>80.3</v>
+        <v>1.4</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>168 x 80 x 4</t>
+          <t>24 x 24 x 2</t>
         </is>
       </c>
       <c r="I43" s="2" t="n"/>
@@ -4015,7 +4015,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>{side}_hip_pitch_stub</t>
+          <t>{side}_shin_knee_outer</t>
         </is>
       </c>
       <c r="B44" s="9" t="n">
@@ -4033,18 +4033,18 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>flat 12.0 mm</t>
+          <t>3D</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G44" s="12" t="n">
-        <v>21</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>30 x 30 x 12</t>
+          <t>121 x 100 x 8</t>
         </is>
       </c>
       <c r="I44" s="2" t="n"/>
@@ -4053,7 +4053,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>{side}_shin_bridge_spacer</t>
+          <t>{side}_shin_spacer_0</t>
         </is>
       </c>
       <c r="B45" s="9" t="n">
@@ -4071,18 +4071,18 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>flat 2.0 mm</t>
+          <t>3D</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="G45" s="12" t="n">
-        <v>1.7</v>
+        <v>22.4</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>28 x 28 x 2</t>
+          <t>58 x 16 x 16</t>
         </is>
       </c>
       <c r="I45" s="2" t="n"/>
@@ -4091,7 +4091,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>{side}_shin_knee_outer</t>
+          <t>{side}_shin_spacer_1</t>
         </is>
       </c>
       <c r="B46" s="9" t="n">
@@ -4113,14 +4113,14 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="G46" s="12" t="n">
-        <v>97.90000000000001</v>
+        <v>22.4</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>121 x 100 x 8</t>
+          <t>58 x 16 x 16</t>
         </is>
       </c>
       <c r="I46" s="2" t="n"/>
@@ -4129,7 +4129,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>{side}_shin_spacer_0</t>
+          <t>{side}_thigh_knee_mount</t>
         </is>
       </c>
       <c r="B47" s="9" t="n">
@@ -4151,14 +4151,14 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G47" s="12" t="n">
-        <v>22.4</v>
+        <v>61.4</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>58 x 16 x 16</t>
+          <t>120 x 120 x 14</t>
         </is>
       </c>
       <c r="I47" s="2" t="n"/>
@@ -4167,7 +4167,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>{side}_shin_spacer_1</t>
+          <t>{side}_thigh_knee_stub</t>
         </is>
       </c>
       <c r="B48" s="9" t="n">
@@ -4185,18 +4185,18 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>3D</t>
+          <t>flat 12.0 mm</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="G48" s="12" t="n">
-        <v>22.4</v>
+        <v>21</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>58 x 16 x 16</t>
+          <t>30 x 30 x 12</t>
         </is>
       </c>
       <c r="I48" s="2" t="n"/>
@@ -4205,11 +4205,11 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>{side}_thigh_knee_mount</t>
+          <t>head_frame</t>
         </is>
       </c>
       <c r="B49" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -4218,23 +4218,23 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>al6061</t>
+          <t>al7075</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>3D</t>
+          <t>flat 6.0 mm</t>
         </is>
       </c>
       <c r="F49" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="G49" s="12" t="n">
-        <v>61.4</v>
+        <v>20.1</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>120 x 120 x 14</t>
+          <t>75 x 16 x 6</t>
         </is>
       </c>
       <c r="I49" s="2" t="n"/>
@@ -4243,11 +4243,11 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>{side}_thigh_knee_stub</t>
+          <t>head_frame_bridge</t>
         </is>
       </c>
       <c r="B50" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -4256,23 +4256,23 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>al6061</t>
+          <t>al7075</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>flat 12.0 mm</t>
+          <t>flat 4.0 mm</t>
         </is>
       </c>
       <c r="F50" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="G50" s="12" t="n">
-        <v>21</v>
+        <v>8.9</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>30 x 30 x 12</t>
+          <t>40 x 20 x 4</t>
         </is>
       </c>
       <c r="I50" s="2" t="n"/>
@@ -4281,7 +4281,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>head_frame</t>
+          <t>head_frame_side_horn</t>
         </is>
       </c>
       <c r="B51" s="9" t="n">
@@ -4299,18 +4299,18 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>flat 6.0 mm</t>
+          <t>flat 3.0 mm</t>
         </is>
       </c>
       <c r="F51" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G51" s="12" t="n">
-        <v>20.1</v>
+        <v>16.2</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>75 x 16 x 6</t>
+          <t>110 x 18 x 3</t>
         </is>
       </c>
       <c r="I51" s="2" t="n"/>
@@ -4319,7 +4319,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>head_frame_bridge</t>
+          <t>head_frame_side_idler</t>
         </is>
       </c>
       <c r="B52" s="9" t="n">
@@ -4337,18 +4337,18 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>flat 4.0 mm</t>
+          <t>flat 3.0 mm</t>
         </is>
       </c>
       <c r="F52" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G52" s="12" t="n">
-        <v>8.9</v>
+        <v>16.2</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>40 x 20 x 4</t>
+          <t>110 x 18 x 3</t>
         </is>
       </c>
       <c r="I52" s="2" t="n"/>
@@ -4357,7 +4357,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>head_frame_side_horn</t>
+          <t>head_frame_top</t>
         </is>
       </c>
       <c r="B53" s="9" t="n">
@@ -4375,18 +4375,18 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>flat 3.0 mm</t>
+          <t>flat 4.0 mm</t>
         </is>
       </c>
       <c r="F53" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G53" s="12" t="n">
-        <v>16.2</v>
+        <v>7.8</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>110 x 18 x 3</t>
+          <t>40 x 18 x 4</t>
         </is>
       </c>
       <c r="I53" s="2" t="n"/>
@@ -4395,7 +4395,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>head_frame_side_idler</t>
+          <t>neck_bracket</t>
         </is>
       </c>
       <c r="B54" s="9" t="n">
@@ -4413,18 +4413,18 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>flat 3.0 mm</t>
+          <t>flat 2.5 mm</t>
         </is>
       </c>
       <c r="F54" t="n">
         <v>3</v>
       </c>
       <c r="G54" s="12" t="n">
-        <v>16.2</v>
+        <v>14</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>110 x 18 x 3</t>
+          <t>50 x 40 x 2</t>
         </is>
       </c>
       <c r="I54" s="2" t="n"/>
@@ -4433,11 +4433,11 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>head_frame_top</t>
+          <t>neck_cheek_{side}</t>
         </is>
       </c>
       <c r="B55" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -4451,18 +4451,18 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>flat 4.0 mm</t>
+          <t>flat 2.5 mm</t>
         </is>
       </c>
       <c r="F55" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G55" s="12" t="n">
-        <v>7.8</v>
+        <v>15.2</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>40 x 18 x 4</t>
+          <t>53 x 42 x 2</t>
         </is>
       </c>
       <c r="I55" s="2" t="n"/>
@@ -4471,7 +4471,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>neck_bracket</t>
+          <t>neck_hub</t>
         </is>
       </c>
       <c r="B56" s="9" t="n">
@@ -4489,18 +4489,18 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>flat 3.0 mm</t>
+          <t>flat 7.0 mm</t>
         </is>
       </c>
       <c r="F56" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G56" s="12" t="n">
-        <v>16.8</v>
+        <v>6.2</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>50 x 40 x 3</t>
+          <t>20 x 20 x 7</t>
         </is>
       </c>
       <c r="I56" s="2" t="n"/>
@@ -4509,7 +4509,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>neck_cheek_{side}</t>
+          <t>pelvis_gusset_front_{side}</t>
         </is>
       </c>
       <c r="B57" s="9" t="n">
@@ -4527,18 +4527,18 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>flat 3.0 mm</t>
+          <t>flat 8.0 mm</t>
         </is>
       </c>
       <c r="F57" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G57" s="12" t="n">
-        <v>18.1</v>
+        <v>252.2</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>52 x 42 x 3</t>
+          <t>212 x 135 x 8</t>
         </is>
       </c>
       <c r="I57" s="2" t="n"/>
@@ -4547,7 +4547,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>neck_hub</t>
+          <t>pelvis_keel_floor</t>
         </is>
       </c>
       <c r="B58" s="9" t="n">
@@ -4565,18 +4565,18 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>flat 7.0 mm</t>
+          <t>flat 3.0 mm</t>
         </is>
       </c>
       <c r="F58" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G58" s="12" t="n">
-        <v>6.2</v>
+        <v>31</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>20 x 20 x 7</t>
+          <t>97 x 38 x 3</t>
         </is>
       </c>
       <c r="I58" s="2" t="n"/>
@@ -4585,7 +4585,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>pelvis_gusset_front_{side}</t>
+          <t>pelvis_roll_carrier_{side}</t>
         </is>
       </c>
       <c r="B59" s="9" t="n">
@@ -4603,18 +4603,18 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>flat 8.0 mm</t>
+          <t>3D</t>
         </is>
       </c>
       <c r="F59" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="G59" s="12" t="n">
-        <v>255.1</v>
+        <v>120</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>212 x 134 x 8</t>
+          <t>120 x 120 x 12</t>
         </is>
       </c>
       <c r="I59" s="2" t="n"/>
@@ -4623,7 +4623,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>pelvis_gusset_rear_{side}</t>
+          <t>pelvis_roll_mount_{side}</t>
         </is>
       </c>
       <c r="B60" s="9" t="n">
@@ -4641,18 +4641,18 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>flat 8.0 mm</t>
+          <t>3D</t>
         </is>
       </c>
       <c r="F60" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="G60" s="12" t="n">
-        <v>60.3</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>104 x 30 x 8</t>
+          <t>120 x 120 x 14</t>
         </is>
       </c>
       <c r="I60" s="2" t="n"/>
@@ -4661,7 +4661,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>pelvis_keel_floor</t>
+          <t>pelvis_top</t>
         </is>
       </c>
       <c r="B61" s="9" t="n">
@@ -4679,18 +4679,18 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>flat 5.0 mm</t>
+          <t>flat 4.0 mm</t>
         </is>
       </c>
       <c r="F61" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G61" s="12" t="n">
-        <v>51.7</v>
+        <v>197.5</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>97 x 38 x 5</t>
+          <t>234 x 124 x 4</t>
         </is>
       </c>
       <c r="I61" s="2" t="n"/>
@@ -4699,11 +4699,11 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>pelvis_roll_carrier_{side}</t>
+          <t>pelvis_waist_cage</t>
         </is>
       </c>
       <c r="B62" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -4717,18 +4717,18 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>3D</t>
+          <t>flat 55.1 mm</t>
         </is>
       </c>
       <c r="F62" t="n">
-        <v>15</v>
+        <v>60</v>
       </c>
       <c r="G62" s="12" t="n">
-        <v>130.9</v>
+        <v>111.5</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>120 x 120 x 12</t>
+          <t>107 x 107 x 55</t>
         </is>
       </c>
       <c r="I62" s="2" t="n"/>
@@ -4737,11 +4737,11 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>pelvis_roll_mount_{side}</t>
+          <t>pelvis_waist_ring</t>
         </is>
       </c>
       <c r="B63" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -4759,14 +4759,14 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="G63" s="12" t="n">
-        <v>78.90000000000001</v>
+        <v>122.3</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>120 x 120 x 14</t>
+          <t>112 x 112 x 12</t>
         </is>
       </c>
       <c r="I63" s="2" t="n"/>
@@ -4775,7 +4775,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>pelvis_top</t>
+          <t>torso_base</t>
         </is>
       </c>
       <c r="B64" s="9" t="n">
@@ -4793,18 +4793,18 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>flat 5.0 mm</t>
+          <t>flat 2.5 mm</t>
         </is>
       </c>
       <c r="F64" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G64" s="12" t="n">
-        <v>246.8</v>
+        <v>112.9</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>234 x 124 x 5</t>
+          <t>150 x 122 x 2</t>
         </is>
       </c>
       <c r="I64" s="2" t="n"/>
@@ -4813,7 +4813,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>pelvis_waist_cage</t>
+          <t>torso_battery_shelf</t>
         </is>
       </c>
       <c r="B65" s="9" t="n">
@@ -4831,18 +4831,18 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>flat 55.1 mm</t>
+          <t>flat 1.5 mm</t>
         </is>
       </c>
       <c r="F65" t="n">
-        <v>60</v>
+        <v>3</v>
       </c>
       <c r="G65" s="12" t="n">
-        <v>111.5</v>
+        <v>20.4</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>107 x 107 x 55</t>
+          <t>155 x 60 x 2</t>
         </is>
       </c>
       <c r="I65" s="2" t="n"/>
@@ -4851,7 +4851,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>pelvis_waist_ring</t>
+          <t>torso_bridge</t>
         </is>
       </c>
       <c r="B66" s="9" t="n">
@@ -4869,18 +4869,18 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>3D</t>
+          <t>flat 8.0 mm</t>
         </is>
       </c>
       <c r="F66" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G66" s="12" t="n">
-        <v>129.4</v>
+        <v>192</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>112 x 112 x 12</t>
+          <t>112 x 108 x 8</t>
         </is>
       </c>
       <c r="I66" s="2" t="n"/>
@@ -4889,7 +4889,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>torso_base</t>
+          <t>torso_compute_plate</t>
         </is>
       </c>
       <c r="B67" s="9" t="n">
@@ -4907,18 +4907,18 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>flat 3.0 mm</t>
+          <t>flat 1.5 mm</t>
         </is>
       </c>
       <c r="F67" t="n">
         <v>3</v>
       </c>
       <c r="G67" s="12" t="n">
-        <v>135.5</v>
+        <v>27.1</v>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>150 x 122 x 3</t>
+          <t>115 x 104 x 2</t>
         </is>
       </c>
       <c r="I67" s="2" t="n"/>
@@ -4927,11 +4927,11 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>torso_battery_shelf</t>
+          <t>torso_shoulder_cage_{side}</t>
         </is>
       </c>
       <c r="B68" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -4945,18 +4945,18 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>flat 3.0 mm</t>
+          <t>flat 41.6 mm</t>
         </is>
       </c>
       <c r="F68" t="n">
-        <v>3</v>
+        <v>50</v>
       </c>
       <c r="G68" s="12" t="n">
-        <v>40.5</v>
+        <v>46.8</v>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>154 x 60 x 3</t>
+          <t>119 x 119 x 42</t>
         </is>
       </c>
       <c r="I68" s="2" t="n"/>
@@ -4965,11 +4965,11 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>torso_bridge</t>
+          <t>torso_shoulder_plate_{side}</t>
         </is>
       </c>
       <c r="B69" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -4983,18 +4983,18 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>flat 8.0 mm</t>
+          <t>flat 6.0 mm</t>
         </is>
       </c>
       <c r="F69" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G69" s="12" t="n">
-        <v>192</v>
+        <v>107.7</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>112 x 108 x 8</t>
+          <t>146 x 134 x 6</t>
         </is>
       </c>
       <c r="I69" s="2" t="n"/>
@@ -5003,11 +5003,11 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>torso_compute_plate</t>
+          <t>torso_shoulder_ring_{side}</t>
         </is>
       </c>
       <c r="B70" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -5021,18 +5021,18 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>flat 3.0 mm</t>
+          <t>3D</t>
         </is>
       </c>
       <c r="F70" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G70" s="12" t="n">
-        <v>54</v>
+        <v>51.5</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>115 x 104 x 3</t>
+          <t>119 x 119 x 5</t>
         </is>
       </c>
       <c r="I70" s="2" t="n"/>
@@ -5041,11 +5041,11 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>torso_shoulder_cage_{side}</t>
+          <t>torso_spacer_l0</t>
         </is>
       </c>
       <c r="B71" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -5059,18 +5059,18 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>flat 41.6 mm</t>
+          <t>flat 17.3 mm</t>
         </is>
       </c>
       <c r="F71" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="G71" s="12" t="n">
-        <v>67.3</v>
+        <v>20.7</v>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>122 x 122 x 42</t>
+          <t>22 x 22 x 17</t>
         </is>
       </c>
       <c r="I71" s="2" t="n"/>
@@ -5079,11 +5079,11 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>torso_shoulder_plate_{side}</t>
+          <t>torso_spacer_l1</t>
         </is>
       </c>
       <c r="B72" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
@@ -5097,18 +5097,18 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>flat 6.0 mm</t>
+          <t>flat 17.3 mm</t>
         </is>
       </c>
       <c r="F72" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="G72" s="12" t="n">
-        <v>110.6</v>
+        <v>20.7</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>148 x 136 x 6</t>
+          <t>22 x 22 x 17</t>
         </is>
       </c>
       <c r="I72" s="2" t="n"/>
@@ -5117,11 +5117,11 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>torso_shoulder_ring_{side}</t>
+          <t>torso_spacer_r0</t>
         </is>
       </c>
       <c r="B73" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
@@ -5135,18 +5135,18 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>3D</t>
+          <t>flat 17.3 mm</t>
         </is>
       </c>
       <c r="F73" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="G73" s="12" t="n">
-        <v>65.2</v>
+        <v>20.7</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>122 x 122 x 6</t>
+          <t>22 x 22 x 17</t>
         </is>
       </c>
       <c r="I73" s="2" t="n"/>
@@ -5155,7 +5155,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>torso_spacer_l0</t>
+          <t>torso_spacer_r1</t>
         </is>
       </c>
       <c r="B74" s="9" t="n">
@@ -5173,14 +5173,14 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>flat 16.8 mm</t>
+          <t>flat 17.3 mm</t>
         </is>
       </c>
       <c r="F74" t="n">
         <v>20</v>
       </c>
       <c r="G74" s="12" t="n">
-        <v>20.1</v>
+        <v>20.7</v>
       </c>
       <c r="H74" t="inlineStr">
         <is>
@@ -5193,7 +5193,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>torso_spacer_l1</t>
+          <t>torso_waist_hub</t>
         </is>
       </c>
       <c r="B75" s="9" t="n">
@@ -5211,18 +5211,18 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>flat 16.8 mm</t>
+          <t>3D</t>
         </is>
       </c>
       <c r="F75" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="G75" s="12" t="n">
-        <v>20.1</v>
+        <v>38.2</v>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>22 x 22 x 17</t>
+          <t>66 x 66 x 9</t>
         </is>
       </c>
       <c r="I75" s="2" t="n"/>
@@ -5231,11 +5231,11 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>torso_spacer_r0</t>
+          <t>{side}_ankle_crank_a</t>
         </is>
       </c>
       <c r="B76" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
@@ -5249,18 +5249,18 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>flat 16.8 mm</t>
+          <t>3D</t>
         </is>
       </c>
       <c r="F76" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G76" s="12" t="n">
-        <v>20.1</v>
+        <v>43.9</v>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>22 x 22 x 17</t>
+          <t>86 x 36 x 13</t>
         </is>
       </c>
       <c r="I76" s="2" t="n"/>
@@ -5269,11 +5269,11 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>torso_spacer_r1</t>
+          <t>{side}_ankle_crank_b</t>
         </is>
       </c>
       <c r="B77" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
@@ -5287,18 +5287,18 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>flat 16.8 mm</t>
+          <t>3D</t>
         </is>
       </c>
       <c r="F77" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>20.1</v>
+        <v>43.9</v>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>22 x 22 x 17</t>
+          <t>86 x 36 x 13</t>
         </is>
       </c>
       <c r="I77" s="2" t="n"/>
@@ -5307,11 +5307,11 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>torso_waist_hub</t>
+          <t>{side}_ankle_cross</t>
         </is>
       </c>
       <c r="B78" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
@@ -5329,14 +5329,14 @@
         </is>
       </c>
       <c r="F78" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="G78" s="12" t="n">
-        <v>45.7</v>
+        <v>48.9</v>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>66 x 66 x 9</t>
+          <t>53 x 44 x 30</t>
         </is>
       </c>
       <c r="I78" s="2" t="n"/>
@@ -5345,7 +5345,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>{side}_ankle_crank_a</t>
+          <t>{side}_foot_lug_front</t>
         </is>
       </c>
       <c r="B79" s="9" t="n">
@@ -5363,18 +5363,18 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>3D</t>
+          <t>flat 8.0 mm</t>
         </is>
       </c>
       <c r="F79" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="G79" s="12" t="n">
-        <v>45.8</v>
+        <v>42.8</v>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>86 x 36 x 14</t>
+          <t>66 x 36 x 8</t>
         </is>
       </c>
       <c r="I79" s="2" t="n"/>
@@ -5383,7 +5383,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>{side}_ankle_crank_b</t>
+          <t>{side}_forearm_frame</t>
         </is>
       </c>
       <c r="B80" s="9" t="n">
@@ -5405,14 +5405,14 @@
         </is>
       </c>
       <c r="F80" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="G80" s="12" t="n">
-        <v>45.8</v>
+        <v>71.7</v>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>86 x 36 x 14</t>
+          <t>132 x 72 x 5</t>
         </is>
       </c>
       <c r="I80" s="2" t="n"/>
@@ -5421,7 +5421,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>{side}_ankle_cross</t>
+          <t>{side}_forearm_hub</t>
         </is>
       </c>
       <c r="B81" s="9" t="n">
@@ -5439,18 +5439,18 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>3D</t>
+          <t>flat 5.0 mm</t>
         </is>
       </c>
       <c r="F81" t="n">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G81" s="12" t="n">
-        <v>48.9</v>
+        <v>26.9</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>53 x 44 x 30</t>
+          <t>52 x 52 x 5</t>
         </is>
       </c>
       <c r="I81" s="2" t="n"/>
@@ -5459,7 +5459,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>{side}_foot_lug_front</t>
+          <t>{side}_hand_arm_horn</t>
         </is>
       </c>
       <c r="B82" s="9" t="n">
@@ -5477,18 +5477,18 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>flat 8.0 mm</t>
+          <t>flat 3.0 mm</t>
         </is>
       </c>
       <c r="F82" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G82" s="12" t="n">
-        <v>42</v>
+        <v>4.9</v>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>64 x 36 x 8</t>
+          <t>29 x 22 x 3</t>
         </is>
       </c>
       <c r="I82" s="2" t="n"/>
@@ -5497,7 +5497,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>{side}_forearm_frame</t>
+          <t>{side}_hand_arm_idler</t>
         </is>
       </c>
       <c r="B83" s="9" t="n">
@@ -5515,18 +5515,18 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>3D</t>
+          <t>flat 3.0 mm</t>
         </is>
       </c>
       <c r="F83" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G83" s="12" t="n">
-        <v>88.90000000000001</v>
+        <v>3.3</v>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>130 x 72 x 6</t>
+          <t>26 x 22 x 3</t>
         </is>
       </c>
       <c r="I83" s="2" t="n"/>
@@ -5535,7 +5535,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>{side}_forearm_hub</t>
+          <t>{side}_hand_mount</t>
         </is>
       </c>
       <c r="B84" s="9" t="n">
@@ -5553,18 +5553,18 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>flat 5.0 mm</t>
+          <t>flat 4.0 mm</t>
         </is>
       </c>
       <c r="F84" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G84" s="12" t="n">
-        <v>26.9</v>
+        <v>35.7</v>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>52 x 52 x 5</t>
+          <t>68 x 53 x 4</t>
         </is>
       </c>
       <c r="I84" s="2" t="n"/>
@@ -5573,7 +5573,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>{side}_hand_arm_horn</t>
+          <t>{side}_hip_pitch_back</t>
         </is>
       </c>
       <c r="B85" s="9" t="n">
@@ -5598,11 +5598,11 @@
         <v>3</v>
       </c>
       <c r="G85" s="12" t="n">
-        <v>4.9</v>
+        <v>27.3</v>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>29 x 22 x 3</t>
+          <t>69 x 68 x 3</t>
         </is>
       </c>
       <c r="I85" s="2" t="n"/>
@@ -5611,7 +5611,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>{side}_hand_arm_idler</t>
+          <t>{side}_hip_pitch_front</t>
         </is>
       </c>
       <c r="B86" s="9" t="n">
@@ -5636,11 +5636,11 @@
         <v>3</v>
       </c>
       <c r="G86" s="12" t="n">
-        <v>3.3</v>
+        <v>27.3</v>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>26 x 22 x 3</t>
+          <t>69 x 68 x 3</t>
         </is>
       </c>
       <c r="I86" s="2" t="n"/>
@@ -5649,7 +5649,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>{side}_hand_mount</t>
+          <t>{side}_hip_pitch_mount</t>
         </is>
       </c>
       <c r="B87" s="9" t="n">
@@ -5667,18 +5667,18 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>flat 4.0 mm</t>
+          <t>3D</t>
         </is>
       </c>
       <c r="F87" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="G87" s="12" t="n">
-        <v>35.7</v>
+        <v>67.7</v>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>68 x 53 x 4</t>
+          <t>120 x 120 x 14</t>
         </is>
       </c>
       <c r="I87" s="2" t="n"/>
@@ -5687,7 +5687,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>{side}_hip_pitch_mount</t>
+          <t>{side}_hip_pitch_outer</t>
         </is>
       </c>
       <c r="B88" s="9" t="n">
@@ -5709,14 +5709,14 @@
         </is>
       </c>
       <c r="F88" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="G88" s="12" t="n">
-        <v>67.7</v>
+        <v>129.5</v>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>120 x 120 x 14</t>
+          <t>168 x 76 x 8</t>
         </is>
       </c>
       <c r="I88" s="2" t="n"/>
@@ -5725,7 +5725,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>{side}_hip_pitch_outer</t>
+          <t>{side}_hip_pitch_top</t>
         </is>
       </c>
       <c r="B89" s="9" t="n">
@@ -5747,14 +5747,14 @@
         </is>
       </c>
       <c r="F89" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G89" s="12" t="n">
-        <v>133.8</v>
+        <v>52.2</v>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>166 x 76 x 8</t>
+          <t>109 x 96 x 3</t>
         </is>
       </c>
       <c r="I89" s="2" t="n"/>
@@ -5763,7 +5763,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>{side}_hip_pitch_top</t>
+          <t>{side}_hip_roll_front</t>
         </is>
       </c>
       <c r="B90" s="9" t="n">
@@ -5788,11 +5788,11 @@
         <v>5</v>
       </c>
       <c r="G90" s="12" t="n">
-        <v>97</v>
+        <v>105.8</v>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>111 x 96 x 5</t>
+          <t>141 x 98 x 5</t>
         </is>
       </c>
       <c r="I90" s="2" t="n"/>
@@ -5801,7 +5801,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>{side}_hip_roll_front</t>
+          <t>{side}_hip_roll_hub</t>
         </is>
       </c>
       <c r="B91" s="9" t="n">
@@ -5823,14 +5823,14 @@
         </is>
       </c>
       <c r="F91" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G91" s="12" t="n">
-        <v>130.6</v>
+        <v>37.3</v>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>141 x 98 x 6</t>
+          <t>66 x 66 x 9</t>
         </is>
       </c>
       <c r="I91" s="2" t="n"/>
@@ -5839,7 +5839,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>{side}_hip_roll_hub</t>
+          <t>{side}_hip_roll_web</t>
         </is>
       </c>
       <c r="B92" s="9" t="n">
@@ -5857,18 +5857,18 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>3D</t>
+          <t>flat 6.0 mm</t>
         </is>
       </c>
       <c r="F92" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G92" s="12" t="n">
-        <v>44.7</v>
+        <v>182</v>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>66 x 66 x 9</t>
+          <t>154 x 128 x 6</t>
         </is>
       </c>
       <c r="I92" s="2" t="n"/>
@@ -5877,7 +5877,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>{side}_hip_roll_web</t>
+          <t>{side}_hip_yaw_hub</t>
         </is>
       </c>
       <c r="B93" s="9" t="n">
@@ -5895,18 +5895,18 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>flat 6.0 mm</t>
+          <t>3D</t>
         </is>
       </c>
       <c r="F93" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G93" s="12" t="n">
-        <v>181.2</v>
+        <v>38.2</v>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>154 x 127 x 6</t>
+          <t>66 x 66 x 9</t>
         </is>
       </c>
       <c r="I93" s="2" t="n"/>
@@ -5915,7 +5915,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>{side}_hip_yaw_hub</t>
+          <t>{side}_shin_bridge</t>
         </is>
       </c>
       <c r="B94" s="9" t="n">
@@ -5937,14 +5937,14 @@
         </is>
       </c>
       <c r="F94" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="G94" s="12" t="n">
-        <v>45.7</v>
+        <v>40.8</v>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>66 x 66 x 9</t>
+          <t>58 x 24 x 24</t>
         </is>
       </c>
       <c r="I94" s="2" t="n"/>
@@ -5953,7 +5953,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>{side}_shin_bridge</t>
+          <t>{side}_shoulder_flange</t>
         </is>
       </c>
       <c r="B95" s="9" t="n">
@@ -5971,18 +5971,18 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>3D</t>
+          <t>flat 6.0 mm</t>
         </is>
       </c>
       <c r="F95" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="G95" s="12" t="n">
-        <v>48.6</v>
+        <v>65.5</v>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>58 x 28 x 28</t>
+          <t>101 x 92 x 6</t>
         </is>
       </c>
       <c r="I95" s="2" t="n"/>
@@ -5991,7 +5991,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>{side}_shoulder_flange</t>
+          <t>{side}_shoulder_hub</t>
         </is>
       </c>
       <c r="B96" s="9" t="n">
@@ -6009,18 +6009,18 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>flat 6.0 mm</t>
+          <t>flat 3.0 mm</t>
         </is>
       </c>
       <c r="F96" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G96" s="12" t="n">
-        <v>63.1</v>
+        <v>26.2</v>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>101 x 92 x 6</t>
+          <t>70 x 70 x 3</t>
         </is>
       </c>
       <c r="I96" s="2" t="n"/>
@@ -6029,7 +6029,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>{side}_shoulder_hub</t>
+          <t>{side}_shoulder_roll_front</t>
         </is>
       </c>
       <c r="B97" s="9" t="n">
@@ -6047,18 +6047,18 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>flat 4.0 mm</t>
+          <t>3D</t>
         </is>
       </c>
       <c r="F97" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G97" s="12" t="n">
-        <v>30.1</v>
+        <v>190</v>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>70 x 54 x 4</t>
+          <t>152 x 112 x 10</t>
         </is>
       </c>
       <c r="I97" s="2" t="n"/>
@@ -6067,7 +6067,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>{side}_shoulder_roll_front</t>
+          <t>{side}_shoulder_roll_hub</t>
         </is>
       </c>
       <c r="B98" s="9" t="n">
@@ -6085,18 +6085,18 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>3D</t>
+          <t>flat 4.0 mm</t>
         </is>
       </c>
       <c r="F98" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="G98" s="12" t="n">
-        <v>235.6</v>
+        <v>40.8</v>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>152 x 112 x 10</t>
+          <t>70 x 70 x 4</t>
         </is>
       </c>
       <c r="I98" s="2" t="n"/>
@@ -6105,7 +6105,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>{side}_shoulder_roll_hub</t>
+          <t>{side}_shoulder_roll_ring</t>
         </is>
       </c>
       <c r="B99" s="9" t="n">
@@ -6123,18 +6123,18 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>flat 4.0 mm</t>
+          <t>3D</t>
         </is>
       </c>
       <c r="F99" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G99" s="12" t="n">
-        <v>40.8</v>
+        <v>32.2</v>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>70 x 70 x 4</t>
+          <t>105 x 97 x 6</t>
         </is>
       </c>
       <c r="I99" s="2" t="n"/>
@@ -6143,7 +6143,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>{side}_shoulder_roll_ring</t>
+          <t>{side}_shoulder_roll_top</t>
         </is>
       </c>
       <c r="B100" s="9" t="n">
@@ -6161,18 +6161,18 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>3D</t>
+          <t>flat 2.5 mm</t>
         </is>
       </c>
       <c r="F100" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G100" s="12" t="n">
-        <v>31.9</v>
+        <v>42.2</v>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>105 x 96 x 6</t>
+          <t>93 x 79 x 2</t>
         </is>
       </c>
       <c r="I100" s="2" t="n"/>
@@ -6181,7 +6181,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>{side}_shoulder_roll_top</t>
+          <t>{side}_shoulder_yaw_cage</t>
         </is>
       </c>
       <c r="B101" s="9" t="n">
@@ -6199,18 +6199,18 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>flat 3.0 mm</t>
+          <t>3D</t>
         </is>
       </c>
       <c r="F101" t="n">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="G101" s="12" t="n">
-        <v>50.7</v>
+        <v>49.6</v>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>93 x 79 x 3</t>
+          <t>93 x 49 x 25</t>
         </is>
       </c>
       <c r="I101" s="2" t="n"/>
@@ -6219,7 +6219,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>{side}_shoulder_yaw_cage</t>
+          <t>{side}_shoulder_yaw_ring</t>
         </is>
       </c>
       <c r="B102" s="9" t="n">
@@ -6241,14 +6241,14 @@
         </is>
       </c>
       <c r="F102" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="G102" s="12" t="n">
-        <v>49.6</v>
+        <v>77.7</v>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>93 x 49 x 25</t>
+          <t>112 x 93 x 9</t>
         </is>
       </c>
       <c r="I102" s="2" t="n"/>
@@ -6257,7 +6257,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>{side}_shoulder_yaw_ring</t>
+          <t>{side}_thigh_cage</t>
         </is>
       </c>
       <c r="B103" s="9" t="n">
@@ -6275,18 +6275,18 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>3D</t>
+          <t>flat 55.1 mm</t>
         </is>
       </c>
       <c r="F103" t="n">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="G103" s="12" t="n">
-        <v>77.09999999999999</v>
+        <v>39.6</v>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>112 x 93 x 9</t>
+          <t>94 x 94 x 55</t>
         </is>
       </c>
       <c r="I103" s="2" t="n"/>
@@ -6295,7 +6295,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>{side}_thigh_cage</t>
+          <t>{side}_thigh_floor</t>
         </is>
       </c>
       <c r="B104" s="9" t="n">
@@ -6313,18 +6313,18 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>flat 55.1 mm</t>
+          <t>flat 6.0 mm</t>
         </is>
       </c>
       <c r="F104" t="n">
-        <v>60</v>
+        <v>6</v>
       </c>
       <c r="G104" s="12" t="n">
-        <v>61.9</v>
+        <v>127.2</v>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>98 x 98 x 55</t>
+          <t>124 x 124 x 6</t>
         </is>
       </c>
       <c r="I104" s="2" t="n"/>
@@ -6333,7 +6333,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>{side}_thigh_floor</t>
+          <t>{side}_thigh_plate</t>
         </is>
       </c>
       <c r="B105" s="9" t="n">
@@ -6351,18 +6351,18 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>flat 6.0 mm</t>
+          <t>flat 5.0 mm</t>
         </is>
       </c>
       <c r="F105" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G105" s="12" t="n">
-        <v>127.8</v>
+        <v>156.2</v>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>124 x 124 x 6</t>
+          <t>182 x 124 x 5</t>
         </is>
       </c>
       <c r="I105" s="2" t="n"/>
@@ -6371,7 +6371,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>{side}_thigh_plate</t>
+          <t>{side}_thigh_rib_back</t>
         </is>
       </c>
       <c r="B106" s="9" t="n">
@@ -6389,18 +6389,18 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>flat 5.0 mm</t>
+          <t>flat 6.0 mm</t>
         </is>
       </c>
       <c r="F106" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G106" s="12" t="n">
-        <v>156.2</v>
+        <v>17.2</v>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>182 x 124 x 5</t>
+          <t>61 x 17 x 6</t>
         </is>
       </c>
       <c r="I106" s="2" t="n"/>
@@ -6409,7 +6409,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>{side}_thigh_rib_back</t>
+          <t>{side}_thigh_rib_front</t>
         </is>
       </c>
       <c r="B107" s="9" t="n">
@@ -6447,7 +6447,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>{side}_thigh_rib_front</t>
+          <t>{side}_thigh_yaw_ring</t>
         </is>
       </c>
       <c r="B108" s="9" t="n">
@@ -6465,18 +6465,18 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>flat 6.0 mm</t>
+          <t>3D</t>
         </is>
       </c>
       <c r="F108" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="G108" s="12" t="n">
-        <v>17.2</v>
+        <v>107.9</v>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>61 x 17 x 6</t>
+          <t>112 x 112 x 12</t>
         </is>
       </c>
       <c r="I108" s="2" t="n"/>
@@ -6485,7 +6485,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>{side}_thigh_yaw_ring</t>
+          <t>{side}_upper_arm_hub</t>
         </is>
       </c>
       <c r="B109" s="9" t="n">
@@ -6503,18 +6503,18 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>3D</t>
+          <t>flat 4.0 mm</t>
         </is>
       </c>
       <c r="F109" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="G109" s="12" t="n">
-        <v>119.2</v>
+        <v>21.5</v>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>112 x 112 x 12</t>
+          <t>52 x 52 x 4</t>
         </is>
       </c>
       <c r="I109" s="2" t="n"/>
@@ -6523,7 +6523,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>{side}_upper_arm_hub</t>
+          <t>{side}_upper_arm_ring</t>
         </is>
       </c>
       <c r="B110" s="9" t="n">
@@ -6541,18 +6541,18 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>flat 4.0 mm</t>
+          <t>3D</t>
         </is>
       </c>
       <c r="F110" t="n">
         <v>4</v>
       </c>
       <c r="G110" s="12" t="n">
-        <v>21.5</v>
+        <v>46.4</v>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>52 x 52 x 4</t>
+          <t>84 x 84 x 4</t>
         </is>
       </c>
       <c r="I110" s="2" t="n"/>
@@ -6561,7 +6561,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>{side}_upper_arm_ring</t>
+          <t>{side}_upper_arm_strap</t>
         </is>
       </c>
       <c r="B111" s="9" t="n">
@@ -6579,18 +6579,18 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>3D</t>
+          <t>flat 6.0 mm</t>
         </is>
       </c>
       <c r="F111" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G111" s="12" t="n">
-        <v>46.4</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>84 x 84 x 4</t>
+          <t>130 x 96 x 6</t>
         </is>
       </c>
       <c r="I111" s="2" t="n"/>
@@ -6599,7 +6599,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>{side}_upper_arm_strap</t>
+          <t>{side}_wrist_bracket</t>
         </is>
       </c>
       <c r="B112" s="9" t="n">
@@ -6617,18 +6617,18 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>flat 6.0 mm</t>
+          <t>flat 3.5 mm</t>
         </is>
       </c>
       <c r="F112" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G112" s="12" t="n">
-        <v>95.59999999999999</v>
+        <v>30</v>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>130 x 96 x 6</t>
+          <t>67 x 63 x 4</t>
         </is>
       </c>
       <c r="I112" s="2" t="n"/>
@@ -6637,7 +6637,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>{side}_wrist_bracket</t>
+          <t>{side}_wrist_cradle</t>
         </is>
       </c>
       <c r="B113" s="9" t="n">
@@ -6655,18 +6655,18 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>flat 5.0 mm</t>
+          <t>3D</t>
         </is>
       </c>
       <c r="F113" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G113" s="12" t="n">
-        <v>43.5</v>
+        <v>15.9</v>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>68 x 63 x 5</t>
+          <t>55 x 55 x 3</t>
         </is>
       </c>
       <c r="I113" s="2" t="n"/>
@@ -6675,7 +6675,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>{side}_wrist_cradle</t>
+          <t>{side}_wrist_cradle_back</t>
         </is>
       </c>
       <c r="B114" s="9" t="n">
@@ -6693,18 +6693,18 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>3D</t>
+          <t>flat 3.0 mm</t>
         </is>
       </c>
       <c r="F114" t="n">
         <v>3</v>
       </c>
       <c r="G114" s="12" t="n">
-        <v>15.9</v>
+        <v>11.4</v>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>55 x 55 x 3</t>
+          <t>44 x 31 x 3</t>
         </is>
       </c>
       <c r="I114" s="2" t="n"/>
@@ -6713,11 +6713,11 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>{side}_wrist_cradle_back</t>
+          <t>{side}_wrist_cradle_side_{side}</t>
         </is>
       </c>
       <c r="B115" s="9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C115" t="inlineStr">
         <is>
@@ -6738,11 +6738,11 @@
         <v>3</v>
       </c>
       <c r="G115" s="12" t="n">
-        <v>11.4</v>
+        <v>6.6</v>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>44 x 31 x 3</t>
+          <t>30 x 26 x 3</t>
         </is>
       </c>
       <c r="I115" s="2" t="n"/>
@@ -6751,36 +6751,33 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>{side}_wrist_cradle_side_{side}</t>
+          <t>neck_cover</t>
         </is>
       </c>
       <c r="B116" s="9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>cnc</t>
+          <t>cover</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>al7075</t>
+          <t>pa_cf</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>flat 3.0 mm</t>
-        </is>
-      </c>
-      <c r="F116" t="n">
-        <v>3</v>
+          <t>3D</t>
+        </is>
       </c>
       <c r="G116" s="12" t="n">
-        <v>6.6</v>
+        <v>40.6</v>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>30 x 26 x 3</t>
+          <t>92 x 92 x 73</t>
         </is>
       </c>
       <c r="I116" s="2" t="n"/>
@@ -6789,7 +6786,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>neck_cover</t>
+          <t>pelvis_cover_back</t>
         </is>
       </c>
       <c r="B117" s="9" t="n">
@@ -6811,11 +6808,11 @@
         </is>
       </c>
       <c r="G117" s="12" t="n">
-        <v>40.6</v>
+        <v>17.6</v>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>92 x 92 x 73</t>
+          <t>200 x 90 x 56</t>
         </is>
       </c>
       <c r="I117" s="2" t="n"/>
@@ -6824,7 +6821,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>pelvis_cover_back</t>
+          <t>pelvis_cover_front</t>
         </is>
       </c>
       <c r="B118" s="9" t="n">
@@ -6846,11 +6843,11 @@
         </is>
       </c>
       <c r="G118" s="12" t="n">
-        <v>22.6</v>
+        <v>10.2</v>
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>200 x 120 x 56</t>
+          <t>143 x 68 x 56</t>
         </is>
       </c>
       <c r="I118" s="2" t="n"/>
@@ -6859,7 +6856,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>pelvis_cover_front</t>
+          <t>torso_cover_back_l_waist</t>
         </is>
       </c>
       <c r="B119" s="9" t="n">
@@ -6881,11 +6878,11 @@
         </is>
       </c>
       <c r="G119" s="12" t="n">
-        <v>12.2</v>
+        <v>41.5</v>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>143 x 68 x 56</t>
+          <t>174 x 93 x 87</t>
         </is>
       </c>
       <c r="I119" s="2" t="n"/>
@@ -6894,7 +6891,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>torso_cover_back_l_waist</t>
+          <t>torso_cover_back_r_waist</t>
         </is>
       </c>
       <c r="B120" s="9" t="n">
@@ -6916,7 +6913,7 @@
         </is>
       </c>
       <c r="G120" s="12" t="n">
-        <v>50</v>
+        <v>41.5</v>
       </c>
       <c r="H120" t="inlineStr">
         <is>
@@ -6929,11 +6926,11 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>torso_cover_back_r_waist</t>
+          <t>torso_cover_back_{side}</t>
         </is>
       </c>
       <c r="B121" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C121" t="inlineStr">
         <is>
@@ -6951,11 +6948,11 @@
         </is>
       </c>
       <c r="G121" s="12" t="n">
-        <v>50</v>
+        <v>49.7</v>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>174 x 93 x 87</t>
+          <t>215 x 98 x 84</t>
         </is>
       </c>
       <c r="I121" s="2" t="n"/>
@@ -6964,11 +6961,11 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>torso_cover_back_{side}</t>
+          <t>torso_cover_front_l_waist</t>
         </is>
       </c>
       <c r="B122" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C122" t="inlineStr">
         <is>
@@ -6986,11 +6983,11 @@
         </is>
       </c>
       <c r="G122" s="12" t="n">
-        <v>59.8</v>
+        <v>41.4</v>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>217 x 98 x 84</t>
+          <t>174 x 93 x 89</t>
         </is>
       </c>
       <c r="I122" s="2" t="n"/>
@@ -6999,7 +6996,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>torso_cover_front_l_waist</t>
+          <t>torso_cover_front_r_waist</t>
         </is>
       </c>
       <c r="B123" s="9" t="n">
@@ -7021,7 +7018,7 @@
         </is>
       </c>
       <c r="G123" s="12" t="n">
-        <v>49.9</v>
+        <v>41.4</v>
       </c>
       <c r="H123" t="inlineStr">
         <is>
@@ -7034,11 +7031,11 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>torso_cover_front_r_waist</t>
+          <t>torso_cover_front_{side}</t>
         </is>
       </c>
       <c r="B124" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C124" t="inlineStr">
         <is>
@@ -7056,11 +7053,11 @@
         </is>
       </c>
       <c r="G124" s="12" t="n">
-        <v>49.9</v>
+        <v>54.4</v>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>174 x 93 x 89</t>
+          <t>215 x 98 x 91</t>
         </is>
       </c>
       <c r="I124" s="2" t="n"/>
@@ -7069,7 +7066,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>torso_cover_front_{side}</t>
+          <t>{side}_forearm_cover</t>
         </is>
       </c>
       <c r="B125" s="9" t="n">
@@ -7091,11 +7088,11 @@
         </is>
       </c>
       <c r="G125" s="12" t="n">
-        <v>65.59999999999999</v>
+        <v>20.2</v>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>217 x 98 x 93</t>
+          <t>80 x 77 x 76</t>
         </is>
       </c>
       <c r="I125" s="2" t="n"/>
@@ -7104,7 +7101,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>{side}_forearm_cover</t>
+          <t>{side}_shin_cover</t>
         </is>
       </c>
       <c r="B126" s="9" t="n">
@@ -7126,11 +7123,11 @@
         </is>
       </c>
       <c r="G126" s="12" t="n">
-        <v>24.5</v>
+        <v>49.9</v>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>80 x 78 x 76</t>
+          <t>188 x 103 x 103</t>
         </is>
       </c>
       <c r="I126" s="2" t="n"/>
@@ -7139,7 +7136,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>{side}_shin_cover</t>
+          <t>{side}_shoulder_cover</t>
         </is>
       </c>
       <c r="B127" s="9" t="n">
@@ -7161,11 +7158,11 @@
         </is>
       </c>
       <c r="G127" s="12" t="n">
-        <v>60</v>
+        <v>6.6</v>
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>188 x 104 x 103</t>
+          <t>106 x 75 x 64</t>
         </is>
       </c>
       <c r="I127" s="2" t="n"/>
@@ -7174,7 +7171,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>{side}_shoulder_cover</t>
+          <t>{side}_thigh_cover</t>
         </is>
       </c>
       <c r="B128" s="9" t="n">
@@ -7196,11 +7193,11 @@
         </is>
       </c>
       <c r="G128" s="12" t="n">
-        <v>7.9</v>
+        <v>55.3</v>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>107 x 75 x 64</t>
+          <t>201 x 134 x 134</t>
         </is>
       </c>
       <c r="I128" s="2" t="n"/>
@@ -7209,7 +7206,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>{side}_thigh_cover</t>
+          <t>{side}_toe_cover</t>
         </is>
       </c>
       <c r="B129" s="9" t="n">
@@ -7231,11 +7228,11 @@
         </is>
       </c>
       <c r="G129" s="12" t="n">
-        <v>66.7</v>
+        <v>13.6</v>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>201 x 134 x 134</t>
+          <t>119 x 99 x 64</t>
         </is>
       </c>
       <c r="I129" s="2" t="n"/>
@@ -7244,7 +7241,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>{side}_toe_cover</t>
+          <t>{side}_upper_arm_cover</t>
         </is>
       </c>
       <c r="B130" s="9" t="n">
@@ -7266,11 +7263,11 @@
         </is>
       </c>
       <c r="G130" s="12" t="n">
-        <v>16.6</v>
+        <v>16.1</v>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>120 x 100 x 64</t>
+          <t>103 x 94 x 82</t>
         </is>
       </c>
       <c r="I130" s="2" t="n"/>
@@ -7279,7 +7276,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>{side}_upper_arm_cover</t>
+          <t>{side}_upper_thigh_cover</t>
         </is>
       </c>
       <c r="B131" s="9" t="n">
@@ -7301,11 +7298,11 @@
         </is>
       </c>
       <c r="G131" s="12" t="n">
-        <v>19.4</v>
+        <v>12.7</v>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>103 x 94 x 82</t>
+          <t>108 x 91 x 64</t>
         </is>
       </c>
       <c r="I131" s="2" t="n"/>
@@ -7314,15 +7311,15 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>{side}_upper_thigh_cover</t>
+          <t>head_camera_frame</t>
         </is>
       </c>
       <c r="B132" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>cover</t>
+          <t>print</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -7336,11 +7333,11 @@
         </is>
       </c>
       <c r="G132" s="12" t="n">
-        <v>15.1</v>
+        <v>20.4</v>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>108 x 91 x 64</t>
+          <t>131 x 56 x 36</t>
         </is>
       </c>
       <c r="I132" s="2" t="n"/>
@@ -7349,7 +7346,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>head_camera_frame</t>
+          <t>head_shell</t>
         </is>
       </c>
       <c r="B133" s="9" t="n">
@@ -7371,11 +7368,11 @@
         </is>
       </c>
       <c r="G133" s="12" t="n">
-        <v>21.5</v>
+        <v>72.3</v>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>131 x 58 x 36</t>
+          <t>167 x 142 x 136</t>
         </is>
       </c>
       <c r="I133" s="2" t="n"/>
@@ -7384,7 +7381,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>head_shell</t>
+          <t>head_visor</t>
         </is>
       </c>
       <c r="B134" s="9" t="n">
@@ -7406,11 +7403,11 @@
         </is>
       </c>
       <c r="G134" s="12" t="n">
-        <v>100</v>
+        <v>59.6</v>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>167 x 142 x 136</t>
+          <t>168 x 141 x 114</t>
         </is>
       </c>
       <c r="I134" s="2" t="n"/>
@@ -7419,7 +7416,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>head_visor</t>
+          <t>torso_battery_guides</t>
         </is>
       </c>
       <c r="B135" s="9" t="n">
@@ -7441,11 +7438,11 @@
         </is>
       </c>
       <c r="G135" s="12" t="n">
-        <v>81.8</v>
+        <v>7.9</v>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>168 x 141 x 114</t>
+          <t>147 x 60 x 20</t>
         </is>
       </c>
       <c r="I135" s="2" t="n"/>
@@ -7454,7 +7451,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>torso_battery_guides</t>
+          <t>torso_battery_latch</t>
         </is>
       </c>
       <c r="B136" s="9" t="n">
@@ -7476,11 +7473,11 @@
         </is>
       </c>
       <c r="G136" s="12" t="n">
-        <v>7.9</v>
+        <v>34.3</v>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>147 x 60 x 20</t>
+          <t>130 x 60 x 4</t>
         </is>
       </c>
       <c r="I136" s="2" t="n"/>
@@ -7489,11 +7486,11 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>torso_battery_latch</t>
+          <t>{side}_foot_sole</t>
         </is>
       </c>
       <c r="B137" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C137" t="inlineStr">
         <is>
@@ -7502,7 +7499,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>pa_cf</t>
+          <t>tpu</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
@@ -7511,11 +7508,11 @@
         </is>
       </c>
       <c r="G137" s="12" t="n">
-        <v>34.3</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>130 x 60 x 4</t>
+          <t>240 x 110 x 3</t>
         </is>
       </c>
       <c r="I137" s="2" t="n"/>
@@ -7524,33 +7521,36 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>{side}_foot_sole</t>
+          <t>pelvis_back</t>
         </is>
       </c>
       <c r="B138" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>print</t>
+          <t>service</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>tpu</t>
+          <t>al7075</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>3D</t>
-        </is>
+          <t>flat 10.0 mm</t>
+        </is>
+      </c>
+      <c r="F138" t="n">
+        <v>10</v>
       </c>
       <c r="G138" s="12" t="n">
-        <v>104.9</v>
+        <v>632.9</v>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>240 x 110 x 4</t>
+          <t>324 x 135 x 10</t>
         </is>
       </c>
       <c r="I138" s="2" t="n"/>
@@ -7559,11 +7559,11 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>pelvis_back</t>
+          <t>torso_upright_{side}</t>
         </is>
       </c>
       <c r="B139" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C139" t="inlineStr">
         <is>
@@ -7577,18 +7577,18 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>flat 10.0 mm</t>
+          <t>flat 3.0 mm</t>
         </is>
       </c>
       <c r="F139" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="G139" s="12" t="n">
-        <v>628.5</v>
+        <v>116.8</v>
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>324 x 134 x 10</t>
+          <t>314 x 149 x 3</t>
         </is>
       </c>
       <c r="I139" s="2" t="n"/>
@@ -7597,7 +7597,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>torso_upright_{side}</t>
+          <t>{side}_foot_base</t>
         </is>
       </c>
       <c r="B140" s="9" t="n">
@@ -7622,11 +7622,11 @@
         <v>4</v>
       </c>
       <c r="G140" s="12" t="n">
-        <v>155.6</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>314 x 149 x 4</t>
+          <t>230 x 100 x 4</t>
         </is>
       </c>
       <c r="I140" s="2" t="n"/>
@@ -7635,7 +7635,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>{side}_foot_base</t>
+          <t>{side}_shin_inner</t>
         </is>
       </c>
       <c r="B141" s="9" t="n">
@@ -7660,11 +7660,11 @@
         <v>4</v>
       </c>
       <c r="G141" s="12" t="n">
-        <v>96.90000000000001</v>
+        <v>194.8</v>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>230 x 100 x 4</t>
+          <t>379 x 140 x 4</t>
         </is>
       </c>
       <c r="I141" s="2" t="n"/>
@@ -7673,7 +7673,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>{side}_shin_inner</t>
+          <t>{side}_shin_outer</t>
         </is>
       </c>
       <c r="B142" s="9" t="n">
@@ -7691,65 +7691,27 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>flat 4.0 mm</t>
+          <t>flat 5.0 mm</t>
         </is>
       </c>
       <c r="F142" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G142" s="12" t="n">
-        <v>194.8</v>
+        <v>186.7</v>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>379 x 140 x 4</t>
+          <t>310 x 160 x 5</t>
         </is>
       </c>
       <c r="I142" s="2" t="n"/>
       <c r="K142" s="2" t="n"/>
     </row>
-    <row r="143">
-      <c r="A143" t="inlineStr">
-        <is>
-          <t>{side}_shin_outer</t>
-        </is>
-      </c>
-      <c r="B143" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="C143" t="inlineStr">
-        <is>
-          <t>service</t>
-        </is>
-      </c>
-      <c r="D143" t="inlineStr">
-        <is>
-          <t>al7075</t>
-        </is>
-      </c>
-      <c r="E143" t="inlineStr">
-        <is>
-          <t>flat 5.0 mm</t>
-        </is>
-      </c>
-      <c r="F143" t="n">
-        <v>5</v>
-      </c>
-      <c r="G143" s="12" t="n">
-        <v>186.7</v>
-      </c>
-      <c r="H143" t="inlineStr">
-        <is>
-          <t>310 x 160 x 5</t>
-        </is>
-      </c>
-      <c r="I143" s="2" t="n"/>
-      <c r="K143" s="2" t="n"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:K143"/>
+  <autoFilter ref="A1:K142"/>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J143" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose one of: to make, ordered, made" type="list">
+    <dataValidation sqref="J2:J142" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose one of: to make, ordered, made" type="list">
       <formula1>"to make,ordered,made"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Wiring paths for the front-ring layout; harness measured from the motors' caps
- tools/build_harness.py: run lengths from each RobStride's driver cap (its
  cable exit), and each service loop tied to a named plate either side
  (CLIPS, checked against description/cad_model.yaml)
- the pelvis power board and servo DC-DC back on the pelvis top plate (it
  dropped 9 mm with the waist motor)
- BOM: grommets for the motor cable holes; ties, P-clips and spiral wrap for
  the loops
- docs/design/assembly_wiring.md: the paths through the new frame, joint by
  joint

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bom/bom.xlsx
+++ b/bom/bom.xlsx
@@ -26,7 +26,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Hands'!$A$1:$K$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Compute &amp; sensors'!$A$1:$K$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Power'!$A$1:$K$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Electronics &amp; wiring'!$A$1:$K$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Electronics &amp; wiring'!$A$1:$K$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Structure &amp; materials'!$A$1:$K$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Fasteners'!$A$1:$K$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Tooling'!$A$1:$K$6</definedName>
@@ -662,24 +662,24 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTA('Electronics &amp; wiring'!A2:A11)</f>
-        <v>10</v>
+        <f>COUNTA('Electronics &amp; wiring'!A2:A13)</f>
+        <v>12</v>
       </c>
       <c r="C9" s="13">
-        <f>'Electronics &amp; wiring'!H13</f>
-        <v>808</v>
+        <f>'Electronics &amp; wiring'!H15</f>
+        <v>836</v>
       </c>
       <c r="D9" s="13">
-        <f>SUMIFS('Electronics &amp; wiring'!$H$2:$H$11,'Electronics &amp; wiring'!$D$2:$D$11,"owned")</f>
+        <f>SUMIFS('Electronics &amp; wiring'!$H$2:$H$13,'Electronics &amp; wiring'!$D$2:$D$13,"owned")</f>
         <v>0</v>
       </c>
       <c r="E9" s="13">
-        <f>SUMIFS('Electronics &amp; wiring'!$H$2:$H$11,'Electronics &amp; wiring'!$D$2:$D$11,"ordered")</f>
+        <f>SUMIFS('Electronics &amp; wiring'!$H$2:$H$13,'Electronics &amp; wiring'!$D$2:$D$13,"ordered")</f>
         <v>0</v>
       </c>
       <c r="F9" s="13">
         <f>C9-D9-E9</f>
-        <v>808</v>
+        <v>836</v>
       </c>
     </row>
     <row r="10">
@@ -798,11 +798,11 @@
       </c>
       <c r="B14" s="5">
         <f>SUM(B5:B13)</f>
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C14" s="14">
         <f>SUM(C5:C13)</f>
-        <v>17531.03</v>
+        <v>17559.03</v>
       </c>
       <c r="D14" s="14">
         <f>SUM(D5:D13)</f>
@@ -814,7 +814,7 @@
       </c>
       <c r="F14" s="14">
         <f>SUM(F5:F13)</f>
-        <v>17531.03</v>
+        <v>17559.03</v>
       </c>
     </row>
     <row r="16" ht="48" customHeight="1">
@@ -9449,7 +9449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -9560,12 +9560,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>usb-hub</t>
+          <t>loop-ties</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Compact USB 3 hub, 4-port</t>
+          <t>Cable ties, P-clips and spiral wrap for the service loops</t>
         </is>
       </c>
       <c r="E3" s="9" t="n">
@@ -9575,11 +9575,11 @@
         <v>0</v>
       </c>
       <c r="G3" s="16" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H3" s="16">
         <f>(E3+F3)*G3</f>
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -9588,19 +9588,19 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>the dev kit has 4 USB-A and 2 USB-C ports; the robot uses 3 CAN adapters, 3 servo adapters, the camera, the IMU and the gamepad receiver</t>
+          <t>each joint's service loop tied to a plate either side (electrical/harness.yaml lists the plates): ties through the plates' lightening pockets, P-clips under a screw where a plate has none; spiral wrap over each loop</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>servo-adapter</t>
+          <t>usb-hub</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Feetech serial-bus USB adapter (Waveshare Bus Servo Adapter (A) class)</t>
+          <t>Compact USB 3 hub, 4-port</t>
         </is>
       </c>
       <c r="E4" s="9" t="n">
@@ -9610,77 +9610,72 @@
         <v>0</v>
       </c>
       <c r="G4" s="16" t="n">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="H4" s="16">
         <f>(E4+F4)*G4</f>
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Waveshare 2026-10-29: $4.99 (SKU 25514)</t>
-        </is>
-      </c>
-      <c r="J4" s="11" t="inlineStr">
-        <is>
-          <t>https://www.waveshare.com/bus-servo-adapter-a.htm</t>
+          <t>estimate</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>STS3250 bus (neck and wrist pitch)</t>
+          <t>the dev kit has 4 USB-A and 2 USB-C ports; the robot uses 3 CAN adapters, 3 servo adapters, the camera, the IMU and the gamepad receiver</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>can-usb-dual</t>
+          <t>servo-adapter</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Isolated USB-CAN adapter, dual channel (InnoMaker USB2CAN-X2 class; SocketCAN)</t>
+          <t>Feetech serial-bus USB adapter (Waveshare Bus Servo Adapter (A) class)</t>
         </is>
       </c>
       <c r="E5" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F5" s="9" t="n">
         <v>0</v>
       </c>
       <c r="G5" s="16" t="n">
-        <v>130</v>
+        <v>5</v>
       </c>
       <c r="H5" s="16">
         <f>(E5+F5)*G5</f>
-        <v>260</v>
+        <v>5</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>unconfirmed 2026-10-29: no live US listing found; ~$126 (AED 462) at a UAE marketplace</t>
+          <t>Waveshare 2026-10-29: $4.99 (SKU 25514)</t>
         </is>
       </c>
       <c r="J5" s="11" t="inlineStr">
         <is>
-          <t>https://github.com/INNO-MAKER/usb2can</t>
+          <t>https://www.waveshare.com/bus-servo-adapter-a.htm</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>one per leg (hip and shank buses), 3 kV isolation per its manual; with can-usb-batt and the Orin's two on-board ports (arm buses) this covers all 7 CAN buses in robot.yaml in the 3 adapter outlines of the electronics bay</t>
+          <t>STS3250 bus (neck and wrist pitch)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>can-usb-single</t>
+          <t>can-usb-dual</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Isolated USB-CAN adapter, single channel (CANable Pro class; candleLight / gs_usb)</t>
+          <t>Isolated USB-CAN adapter, dual channel (InnoMaker USB2CAN-X2 class; SocketCAN)</t>
         </is>
       </c>
       <c r="E6" s="9" t="n">
@@ -9690,112 +9685,112 @@
         <v>0</v>
       </c>
       <c r="G6" s="16" t="n">
-        <v>60</v>
+        <v>130</v>
       </c>
       <c r="H6" s="16">
         <f>(E6+F6)*G6</f>
-        <v>120</v>
+        <v>260</v>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>reseller listing 2026-10-29, unverified: CANable Pro $60, Pro 1.1 (5 kV) $70</t>
+          <t>unconfirmed 2026-10-29: no live US listing found; ~$126 (AED 462) at a UAE marketplace</t>
         </is>
       </c>
       <c r="J6" s="11" t="inlineStr">
         <is>
-          <t>https://reach.dog/shop/openlight-labs/products/canable-pro-isolated-usb-to-can-adapter</t>
+          <t>https://github.com/INNO-MAKER/usb2can</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>one for the battery (BMS) bus, one for the actuator bench rig</t>
+          <t>one per leg (hip and shank buses), 3 kV isolation per its manual; with can-usb-batt and the Orin's two on-board ports (arm buses) this covers all 7 CAN buses in robot.yaml in the 3 adapter outlines of the electronics bay</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>limb-conn</t>
+          <t>can-usb-single</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Limb-root connectors: XT60-class power pair and latching signal pair, per limb</t>
+          <t>Isolated USB-CAN adapter, single channel (CANable Pro class; candleLight / gs_usb)</t>
         </is>
       </c>
       <c r="E7" s="9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F7" s="9" t="n">
         <v>0</v>
       </c>
       <c r="G7" s="16" t="n">
-        <v>12</v>
+        <v>60</v>
       </c>
       <c r="H7" s="16">
         <f>(E7+F7)*G7</f>
-        <v>48</v>
+        <v>120</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>estimate</t>
+          <t>reseller listing 2026-10-29, unverified: CANable Pro $60, Pro 1.1 (5 kV) $70</t>
+        </is>
+      </c>
+      <c r="J7" s="11" t="inlineStr">
+        <is>
+          <t>https://reach.dog/shop/openlight-labs/products/canable-pro-isolated-usb-to-can-adapter</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>on the bulkheads beside each limb's first flange</t>
+          <t>one for the battery (BMS) bus, one for the actuator bench rig</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>can-robstride-dbg</t>
+          <t>limb-conn</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>RobStride USB-to-CAN debug adapter (official GUI tool)</t>
+          <t>Limb-root connectors: XT60-class power pair and latching signal pair, per limb</t>
         </is>
       </c>
       <c r="E8" s="9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F8" s="9" t="n">
         <v>0</v>
       </c>
       <c r="G8" s="16" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="H8" s="16">
         <f>(E8+F8)*G8</f>
-        <v>15</v>
+        <v>48</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Seeed listing 2026-10, unverified: $15 each, $14 at 10+</t>
-        </is>
-      </c>
-      <c r="J8" s="11" t="inlineStr">
-        <is>
-          <t>https://www.seeedstudio.com/Robostride-CAN-USB-Driver-Board-p-6708.html</t>
+          <t>estimate</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>for RobStride's configuration GUI (IDs, firmware); check whether it works as a SocketCAN bus before using it on the robot</t>
+          <t>on the bulkheads beside each limb's first flange</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>harness</t>
+          <t>can-robstride-dbg</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Silicone wire; connectors; strain relief; sleeving</t>
+          <t>RobStride USB-to-CAN debug adapter (official GUI tool)</t>
         </is>
       </c>
       <c r="E9" s="9" t="n">
@@ -9805,59 +9800,72 @@
         <v>0</v>
       </c>
       <c r="G9" s="16" t="n">
-        <v>200</v>
+        <v>15</v>
       </c>
       <c r="H9" s="16">
         <f>(E9+F9)*G9</f>
-        <v>200</v>
+        <v>15</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>estimate</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="n"/>
+          <t>Seeed listing 2026-10, unverified: $15 each, $14 at 10+</t>
+        </is>
+      </c>
+      <c r="J9" s="11" t="inlineStr">
+        <is>
+          <t>https://www.seeedstudio.com/Robostride-CAN-USB-Driver-Board-p-6708.html</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>for RobStride's configuration GUI (IDs, firmware); check whether it works as a SocketCAN bus before using it on the robot</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>can-cable</t>
+          <t>cable-grommets</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Twisted-pair CAN cable, connectors and 120 Ω terminations</t>
+          <t>Rubber grommets for the motor cable holes (20-30 mm holes in 2-4 mm plate)</t>
         </is>
       </c>
       <c r="E10" s="9" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F10" s="9" t="n">
         <v>0</v>
       </c>
       <c r="G10" s="16" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="H10" s="16">
         <f>(E10+F10)*G10</f>
-        <v>50</v>
+        <v>8</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
-      <c r="K10" s="2" t="n"/>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>where a motor's cable passes a plate: the thigh floors and pelvis top plate (hip yaw and waist RS03 caps), the shoulder roll top plates (shoulder yaw RS06 caps) and the wrist brackets (RS00 rear faces); 7 used, 1 spare</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>gamepad</t>
+          <t>harness</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Wireless gamepad</t>
+          <t>Silicone wire; connectors; strain relief; sleeving</t>
         </is>
       </c>
       <c r="E11" s="9" t="n">
@@ -9867,51 +9875,113 @@
         <v>0</v>
       </c>
       <c r="G11" s="16" t="n">
-        <v>60</v>
+        <v>200</v>
       </c>
       <c r="H11" s="16">
         <f>(E11+F11)*G11</f>
+        <v>200</v>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>estimate</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>can-cable</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Twisted-pair CAN cable, connectors and 120 Ω terminations</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="16" t="n">
+        <v>50</v>
+      </c>
+      <c r="H12" s="16">
+        <f>(E12+F12)*G12</f>
+        <v>50</v>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>estimate</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>gamepad</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Wireless gamepad</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="16" t="n">
         <v>60</v>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="H13" s="16">
+        <f>(E13+F13)*G13</f>
+        <v>60</v>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
-      <c r="K11" s="2" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="n"/>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="K13" s="2" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n"/>
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Total electronics &amp; wiring</t>
         </is>
       </c>
-      <c r="C13" s="5" t="n"/>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="5" t="n"/>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="14">
-        <f>SUM(H2:H11)</f>
-        <v>808</v>
-      </c>
-      <c r="I13" s="5" t="n"/>
-      <c r="J13" s="5" t="n"/>
-      <c r="K13" s="5" t="n"/>
+      <c r="C15" s="5" t="n"/>
+      <c r="D15" s="5" t="n"/>
+      <c r="E15" s="5" t="n"/>
+      <c r="F15" s="5" t="n"/>
+      <c r="G15" s="5" t="n"/>
+      <c r="H15" s="14">
+        <f>SUM(H2:H13)</f>
+        <v>836</v>
+      </c>
+      <c r="I15" s="5" t="n"/>
+      <c r="J15" s="5" t="n"/>
+      <c r="K15" s="5" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K11"/>
+  <autoFilter ref="A1:K13"/>
   <dataValidations count="1">
-    <dataValidation sqref="D2:D11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose one of: to buy, ordered, owned" type="list">
+    <dataValidation sqref="D2:D13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose one of: to buy, ordered, owned" type="list">
       <formula1>"to buy,ordered,owned"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J4" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J6" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Harness clip points, faceted torso shell, shells refined to the new frame; docs synced
- Harness clips in the parts: push-in mount holes on solid pads (clip_spot), printed
  TPU edge clips for thick plates (cad/clips.py), a P-clip at the shoulder flange;
  CLIPS checked against cad_model.yaml.
- Torso shell faceted (alternating octagon sections, hulled), shoulder chamfers and a
  front bevel that clears the shoulder roll bracket; flat-shaded in renders.
- Grilles over the arm motors; room for each harness loop over the arc between its
  clip holes, on the rear arc at the knee (it had notched the thigh shell).
- 41.17 kg bare, 41.99 kg with shells; cad.covers --check finds no contacts.
- README, decisions, roadmap, wiring doc, the site's home page and guide pages 00 and
  08 updated (build123d frame, front rings, bearings, clips, shells); README render.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bom/bom.xlsx
+++ b/bom/bom.xlsx
@@ -26,13 +26,13 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Hands'!$A$1:$K$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Compute &amp; sensors'!$A$1:$K$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Power'!$A$1:$K$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Electronics &amp; wiring'!$A$1:$K$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Electronics &amp; wiring'!$A$1:$K$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Structure &amp; materials'!$A$1:$K$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Fasteners'!$A$1:$K$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Tooling'!$A$1:$K$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Safety'!$A$1:$K$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Sourcing'!$A$1:$J$29</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Made parts (CAD)'!$A$1:$K$142</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Made parts (CAD)'!$A$1:$K$146</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Actuator bolts (CAD)'!$A$1:$F$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -662,24 +662,24 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTA('Electronics &amp; wiring'!A2:A13)</f>
-        <v>12</v>
+        <f>COUNTA('Electronics &amp; wiring'!A2:A14)</f>
+        <v>13</v>
       </c>
       <c r="C9" s="13">
-        <f>'Electronics &amp; wiring'!H15</f>
-        <v>836</v>
+        <f>'Electronics &amp; wiring'!H16</f>
+        <v>845.9</v>
       </c>
       <c r="D9" s="13">
-        <f>SUMIFS('Electronics &amp; wiring'!$H$2:$H$13,'Electronics &amp; wiring'!$D$2:$D$13,"owned")</f>
+        <f>SUMIFS('Electronics &amp; wiring'!$H$2:$H$14,'Electronics &amp; wiring'!$D$2:$D$14,"owned")</f>
         <v>0</v>
       </c>
       <c r="E9" s="13">
-        <f>SUMIFS('Electronics &amp; wiring'!$H$2:$H$13,'Electronics &amp; wiring'!$D$2:$D$13,"ordered")</f>
+        <f>SUMIFS('Electronics &amp; wiring'!$H$2:$H$14,'Electronics &amp; wiring'!$D$2:$D$14,"ordered")</f>
         <v>0</v>
       </c>
       <c r="F9" s="13">
         <f>C9-D9-E9</f>
-        <v>836</v>
+        <v>845.9</v>
       </c>
     </row>
     <row r="10">
@@ -798,11 +798,11 @@
       </c>
       <c r="B14" s="5">
         <f>SUM(B5:B13)</f>
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C14" s="14">
         <f>SUM(C5:C13)</f>
-        <v>17559.03</v>
+        <v>17568.93</v>
       </c>
       <c r="D14" s="14">
         <f>SUM(D5:D13)</f>
@@ -814,7 +814,7 @@
       </c>
       <c r="F14" s="14">
         <f>SUM(F5:F13)</f>
-        <v>17559.03</v>
+        <v>17568.93</v>
       </c>
     </row>
     <row r="16" ht="48" customHeight="1">
@@ -2451,7 +2451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K142"/>
+  <dimension ref="A1:K146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4420,7 +4420,7 @@
         <v>3</v>
       </c>
       <c r="G54" s="12" t="n">
-        <v>14</v>
+        <v>13.8</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
@@ -4686,7 +4686,7 @@
         <v>4</v>
       </c>
       <c r="G61" s="12" t="n">
-        <v>197.5</v>
+        <v>197.1</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
@@ -4800,7 +4800,7 @@
         <v>3</v>
       </c>
       <c r="G64" s="12" t="n">
-        <v>112.9</v>
+        <v>112.7</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
@@ -4990,7 +4990,7 @@
         <v>6</v>
       </c>
       <c r="G69" s="12" t="n">
-        <v>107.7</v>
+        <v>114.5</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
@@ -5408,7 +5408,7 @@
         <v>5</v>
       </c>
       <c r="G80" s="12" t="n">
-        <v>71.7</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="H80" t="inlineStr">
         <is>
@@ -5446,11 +5446,11 @@
         <v>5</v>
       </c>
       <c r="G81" s="12" t="n">
-        <v>26.9</v>
+        <v>20.4</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>52 x 52 x 5</t>
+          <t>46 x 46 x 5</t>
         </is>
       </c>
       <c r="I81" s="2" t="n"/>
@@ -5598,7 +5598,7 @@
         <v>3</v>
       </c>
       <c r="G85" s="12" t="n">
-        <v>27.3</v>
+        <v>27.9</v>
       </c>
       <c r="H85" t="inlineStr">
         <is>
@@ -5864,7 +5864,7 @@
         <v>6</v>
       </c>
       <c r="G92" s="12" t="n">
-        <v>182</v>
+        <v>188.9</v>
       </c>
       <c r="H92" t="inlineStr">
         <is>
@@ -6054,7 +6054,7 @@
         <v>10</v>
       </c>
       <c r="G97" s="12" t="n">
-        <v>190</v>
+        <v>187.8</v>
       </c>
       <c r="H97" t="inlineStr">
         <is>
@@ -6092,11 +6092,11 @@
         <v>4</v>
       </c>
       <c r="G98" s="12" t="n">
-        <v>40.8</v>
+        <v>27.3</v>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>70 x 70 x 4</t>
+          <t>58 x 58 x 4</t>
         </is>
       </c>
       <c r="I98" s="2" t="n"/>
@@ -6320,7 +6320,7 @@
         <v>6</v>
       </c>
       <c r="G104" s="12" t="n">
-        <v>127.2</v>
+        <v>132.4</v>
       </c>
       <c r="H104" t="inlineStr">
         <is>
@@ -6358,7 +6358,7 @@
         <v>5</v>
       </c>
       <c r="G105" s="12" t="n">
-        <v>156.2</v>
+        <v>159.2</v>
       </c>
       <c r="H105" t="inlineStr">
         <is>
@@ -6510,11 +6510,11 @@
         <v>4</v>
       </c>
       <c r="G109" s="12" t="n">
-        <v>21.5</v>
+        <v>16.3</v>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>52 x 52 x 4</t>
+          <t>46 x 46 x 4</t>
         </is>
       </c>
       <c r="I109" s="2" t="n"/>
@@ -6548,7 +6548,7 @@
         <v>4</v>
       </c>
       <c r="G110" s="12" t="n">
-        <v>46.4</v>
+        <v>45</v>
       </c>
       <c r="H110" t="inlineStr">
         <is>
@@ -6586,7 +6586,7 @@
         <v>6</v>
       </c>
       <c r="G111" s="12" t="n">
-        <v>95.59999999999999</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="H111" t="inlineStr">
         <is>
@@ -6700,7 +6700,7 @@
         <v>3</v>
       </c>
       <c r="G114" s="12" t="n">
-        <v>11.4</v>
+        <v>11.1</v>
       </c>
       <c r="H114" t="inlineStr">
         <is>
@@ -6812,7 +6812,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>200 x 90 x 56</t>
+          <t>200 x 92 x 56</t>
         </is>
       </c>
       <c r="I117" s="2" t="n"/>
@@ -6878,11 +6878,11 @@
         </is>
       </c>
       <c r="G119" s="12" t="n">
-        <v>41.5</v>
+        <v>44.2</v>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>174 x 93 x 87</t>
+          <t>174 x 107 x 98</t>
         </is>
       </c>
       <c r="I119" s="2" t="n"/>
@@ -6913,11 +6913,11 @@
         </is>
       </c>
       <c r="G120" s="12" t="n">
-        <v>41.5</v>
+        <v>44.2</v>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>174 x 93 x 87</t>
+          <t>174 x 107 x 98</t>
         </is>
       </c>
       <c r="I120" s="2" t="n"/>
@@ -6948,11 +6948,11 @@
         </is>
       </c>
       <c r="G121" s="12" t="n">
-        <v>49.7</v>
+        <v>60.4</v>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>215 x 98 x 84</t>
+          <t>219 x 106 x 98</t>
         </is>
       </c>
       <c r="I121" s="2" t="n"/>
@@ -6983,11 +6983,11 @@
         </is>
       </c>
       <c r="G122" s="12" t="n">
-        <v>41.4</v>
+        <v>45.1</v>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>174 x 93 x 89</t>
+          <t>174 x 112 x 98</t>
         </is>
       </c>
       <c r="I122" s="2" t="n"/>
@@ -7018,11 +7018,11 @@
         </is>
       </c>
       <c r="G123" s="12" t="n">
-        <v>41.4</v>
+        <v>45.1</v>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>174 x 93 x 89</t>
+          <t>174 x 112 x 98</t>
         </is>
       </c>
       <c r="I123" s="2" t="n"/>
@@ -7053,11 +7053,11 @@
         </is>
       </c>
       <c r="G124" s="12" t="n">
-        <v>54.4</v>
+        <v>56.4</v>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>215 x 98 x 91</t>
+          <t>219 x 113 x 98</t>
         </is>
       </c>
       <c r="I124" s="2" t="n"/>
@@ -7088,11 +7088,11 @@
         </is>
       </c>
       <c r="G125" s="12" t="n">
-        <v>20.2</v>
+        <v>17.8</v>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>80 x 77 x 76</t>
+          <t>80 x 76 x 76</t>
         </is>
       </c>
       <c r="I125" s="2" t="n"/>
@@ -7263,11 +7263,11 @@
         </is>
       </c>
       <c r="G130" s="12" t="n">
-        <v>16.1</v>
+        <v>14.7</v>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>103 x 94 x 82</t>
+          <t>103 x 93 x 82</t>
         </is>
       </c>
       <c r="I130" s="2" t="n"/>
@@ -7486,7 +7486,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>{side}_foot_sole</t>
+          <t>pelvis_back_clip_{side}</t>
         </is>
       </c>
       <c r="B137" s="9" t="n">
@@ -7508,20 +7508,24 @@
         </is>
       </c>
       <c r="G137" s="12" t="n">
-        <v>78.59999999999999</v>
+        <v>1.6</v>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>240 x 110 x 3</t>
-        </is>
-      </c>
-      <c r="I137" s="2" t="n"/>
+          <t>26 x 15 x 14</t>
+        </is>
+      </c>
+      <c r="I137" s="2" t="inlineStr">
+        <is>
+          <t>harness edge clip for a 10 mm plate (cad/clips.py)</t>
+        </is>
+      </c>
       <c r="K137" s="2" t="n"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>pelvis_back</t>
+          <t>torso_bridge_clip</t>
         </is>
       </c>
       <c r="B138" s="9" t="n">
@@ -7529,37 +7533,38 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>service</t>
+          <t>print</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>al7075</t>
+          <t>tpu</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>flat 10.0 mm</t>
-        </is>
-      </c>
-      <c r="F138" t="n">
-        <v>10</v>
+          <t>3D</t>
+        </is>
       </c>
       <c r="G138" s="12" t="n">
-        <v>632.9</v>
+        <v>1.6</v>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>324 x 135 x 10</t>
-        </is>
-      </c>
-      <c r="I138" s="2" t="n"/>
+          <t>24 x 12 x 10</t>
+        </is>
+      </c>
+      <c r="I138" s="2" t="inlineStr">
+        <is>
+          <t>harness edge clip for a 8 mm plate (cad/clips.py)</t>
+        </is>
+      </c>
       <c r="K138" s="2" t="n"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>torso_upright_{side}</t>
+          <t>{side}_foot_sole</t>
         </is>
       </c>
       <c r="B139" s="9" t="n">
@@ -7567,28 +7572,25 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>service</t>
+          <t>print</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>al7075</t>
+          <t>tpu</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>flat 3.0 mm</t>
-        </is>
-      </c>
-      <c r="F139" t="n">
-        <v>3</v>
+          <t>3D</t>
+        </is>
       </c>
       <c r="G139" s="12" t="n">
-        <v>116.8</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>314 x 149 x 3</t>
+          <t>240 x 110 x 3</t>
         </is>
       </c>
       <c r="I139" s="2" t="n"/>
@@ -7597,7 +7599,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>{side}_foot_base</t>
+          <t>{side}_hip_pitch_outer_clip</t>
         </is>
       </c>
       <c r="B140" s="9" t="n">
@@ -7605,37 +7607,38 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>service</t>
+          <t>print</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>al7075</t>
+          <t>tpu</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>flat 4.0 mm</t>
-        </is>
-      </c>
-      <c r="F140" t="n">
-        <v>4</v>
+          <t>3D</t>
+        </is>
       </c>
       <c r="G140" s="12" t="n">
-        <v>96.90000000000001</v>
+        <v>1.6</v>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>230 x 100 x 4</t>
-        </is>
-      </c>
-      <c r="I140" s="2" t="n"/>
+          <t>24 x 12 x 10</t>
+        </is>
+      </c>
+      <c r="I140" s="2" t="inlineStr">
+        <is>
+          <t>harness edge clip for a 8 mm plate (cad/clips.py)</t>
+        </is>
+      </c>
       <c r="K140" s="2" t="n"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>{side}_shin_inner</t>
+          <t>{side}_shoulder_roll_front_clip</t>
         </is>
       </c>
       <c r="B141" s="9" t="n">
@@ -7643,41 +7646,42 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>service</t>
+          <t>print</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>al7075</t>
+          <t>tpu</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>flat 4.0 mm</t>
-        </is>
-      </c>
-      <c r="F141" t="n">
-        <v>4</v>
+          <t>3D</t>
+        </is>
       </c>
       <c r="G141" s="12" t="n">
-        <v>194.8</v>
+        <v>1.6</v>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>379 x 140 x 4</t>
-        </is>
-      </c>
-      <c r="I141" s="2" t="n"/>
+          <t>26 x 20 x 14</t>
+        </is>
+      </c>
+      <c r="I141" s="2" t="inlineStr">
+        <is>
+          <t>harness edge clip for a 10 mm plate (cad/clips.py)</t>
+        </is>
+      </c>
       <c r="K141" s="2" t="n"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>{side}_shin_outer</t>
+          <t>pelvis_back</t>
         </is>
       </c>
       <c r="B142" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C142" t="inlineStr">
         <is>
@@ -7691,27 +7695,179 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>flat 5.0 mm</t>
+          <t>flat 10.0 mm</t>
         </is>
       </c>
       <c r="F142" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G142" s="12" t="n">
-        <v>186.7</v>
+        <v>632.9</v>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>310 x 160 x 5</t>
+          <t>324 x 135 x 10</t>
         </is>
       </c>
       <c r="I142" s="2" t="n"/>
       <c r="K142" s="2" t="n"/>
     </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>torso_upright_{side}</t>
+        </is>
+      </c>
+      <c r="B143" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>service</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>al7075</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>flat 3.0 mm</t>
+        </is>
+      </c>
+      <c r="F143" t="n">
+        <v>3</v>
+      </c>
+      <c r="G143" s="12" t="n">
+        <v>116.8</v>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>314 x 149 x 3</t>
+        </is>
+      </c>
+      <c r="I143" s="2" t="n"/>
+      <c r="K143" s="2" t="n"/>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>{side}_foot_base</t>
+        </is>
+      </c>
+      <c r="B144" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>service</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>al7075</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>flat 4.0 mm</t>
+        </is>
+      </c>
+      <c r="F144" t="n">
+        <v>4</v>
+      </c>
+      <c r="G144" s="12" t="n">
+        <v>96.90000000000001</v>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>230 x 100 x 4</t>
+        </is>
+      </c>
+      <c r="I144" s="2" t="n"/>
+      <c r="K144" s="2" t="n"/>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>{side}_shin_inner</t>
+        </is>
+      </c>
+      <c r="B145" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>service</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>al7075</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>flat 4.0 mm</t>
+        </is>
+      </c>
+      <c r="F145" t="n">
+        <v>4</v>
+      </c>
+      <c r="G145" s="12" t="n">
+        <v>198.5</v>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>379 x 140 x 4</t>
+        </is>
+      </c>
+      <c r="I145" s="2" t="n"/>
+      <c r="K145" s="2" t="n"/>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>{side}_shin_outer</t>
+        </is>
+      </c>
+      <c r="B146" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>service</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>al7075</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>flat 5.0 mm</t>
+        </is>
+      </c>
+      <c r="F146" t="n">
+        <v>5</v>
+      </c>
+      <c r="G146" s="12" t="n">
+        <v>186.7</v>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>310 x 160 x 5</t>
+        </is>
+      </c>
+      <c r="I146" s="2" t="n"/>
+      <c r="K146" s="2" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K142"/>
+  <autoFilter ref="A1:K146"/>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J142" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose one of: to make, ordered, made" type="list">
+    <dataValidation sqref="J2:J146" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose one of: to make, ordered, made" type="list">
       <formula1>"to make,ordered,made"</formula1>
     </dataValidation>
   </dataValidations>
@@ -9449,7 +9605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -9785,118 +9941,122 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>can-robstride-dbg</t>
+          <t>clip-mounts</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>RobStride USB-to-CAN debug adapter (official GUI tool)</t>
+          <t>Push-in cable-tie mounts (fir-tree stem for a 6.5 mm hole in a 1-6 mm panel)</t>
         </is>
       </c>
       <c r="E9" s="9" t="n">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G9" s="16" t="n">
-        <v>15</v>
+        <v>0.3</v>
       </c>
       <c r="H9" s="16">
         <f>(E9+F9)*G9</f>
-        <v>15</v>
+        <v>9.9</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Seeed listing 2026-10, unverified: $15 each, $14 at 10+</t>
-        </is>
-      </c>
-      <c r="J9" s="11" t="inlineStr">
-        <is>
-          <t>https://www.seeedstudio.com/Robostride-CAN-USB-Driver-Board-p-6708.html</t>
+          <t>estimate</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>for RobStride's configuration GUI (IDs, firmware); check whether it works as a SocketCAN bus before using it on the robot</t>
+          <t>one in each 6.5 mm harness clip hole on a solid pad (cad/mounts.py: CLIP_HOLE), at the service loops electrical/harness.yaml lists; the thicker plates take the printed TPU edge clips (cad/clips.py) instead</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>cable-grommets</t>
+          <t>can-robstride-dbg</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Rubber grommets for the motor cable holes (20-30 mm holes in 2-4 mm plate)</t>
+          <t>RobStride USB-to-CAN debug adapter (official GUI tool)</t>
         </is>
       </c>
       <c r="E10" s="9" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F10" s="9" t="n">
         <v>0</v>
       </c>
       <c r="G10" s="16" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="H10" s="16">
         <f>(E10+F10)*G10</f>
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>estimate</t>
+          <t>Seeed listing 2026-10, unverified: $15 each, $14 at 10+</t>
+        </is>
+      </c>
+      <c r="J10" s="11" t="inlineStr">
+        <is>
+          <t>https://www.seeedstudio.com/Robostride-CAN-USB-Driver-Board-p-6708.html</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>where a motor's cable passes a plate: the thigh floors and pelvis top plate (hip yaw and waist RS03 caps), the shoulder roll top plates (shoulder yaw RS06 caps) and the wrist brackets (RS00 rear faces); 7 used, 1 spare</t>
+          <t>for RobStride's configuration GUI (IDs, firmware); check whether it works as a SocketCAN bus before using it on the robot</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>harness</t>
+          <t>cable-grommets</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Silicone wire; connectors; strain relief; sleeving</t>
+          <t>Rubber grommets for the motor cable holes (20-30 mm holes in 2-4 mm plate)</t>
         </is>
       </c>
       <c r="E11" s="9" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F11" s="9" t="n">
         <v>0</v>
       </c>
       <c r="G11" s="16" t="n">
-        <v>200</v>
+        <v>1</v>
       </c>
       <c r="H11" s="16">
         <f>(E11+F11)*G11</f>
-        <v>200</v>
+        <v>8</v>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
-      <c r="K11" s="2" t="n"/>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>where a motor's cable passes a plate: the thigh floors and pelvis top plate (hip yaw and waist RS03 caps), the shoulder roll top plates (shoulder yaw RS06 caps) and the wrist brackets (RS00 rear faces); 7 used, 1 spare</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>can-cable</t>
+          <t>harness</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Twisted-pair CAN cable, connectors and 120 Ω terminations</t>
+          <t>Silicone wire; connectors; strain relief; sleeving</t>
         </is>
       </c>
       <c r="E12" s="9" t="n">
@@ -9906,11 +10066,11 @@
         <v>0</v>
       </c>
       <c r="G12" s="16" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="H12" s="16">
         <f>(E12+F12)*G12</f>
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
@@ -9922,12 +10082,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>gamepad</t>
+          <t>can-cable</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Wireless gamepad</t>
+          <t>Twisted-pair CAN cable, connectors and 120 Ω terminations</t>
         </is>
       </c>
       <c r="E13" s="9" t="n">
@@ -9937,43 +10097,74 @@
         <v>0</v>
       </c>
       <c r="G13" s="16" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H13" s="16">
         <f>(E13+F13)*G13</f>
+        <v>50</v>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>estimate</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>gamepad</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Wireless gamepad</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="16" t="n">
         <v>60</v>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="H14" s="16">
+        <f>(E14+F14)*G14</f>
+        <v>60</v>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
-      <c r="K13" s="2" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="n"/>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="K14" s="2" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n"/>
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Total electronics &amp; wiring</t>
         </is>
       </c>
-      <c r="C15" s="5" t="n"/>
-      <c r="D15" s="5" t="n"/>
-      <c r="E15" s="5" t="n"/>
-      <c r="F15" s="5" t="n"/>
-      <c r="G15" s="5" t="n"/>
-      <c r="H15" s="14">
-        <f>SUM(H2:H13)</f>
-        <v>836</v>
-      </c>
-      <c r="I15" s="5" t="n"/>
-      <c r="J15" s="5" t="n"/>
-      <c r="K15" s="5" t="n"/>
+      <c r="C16" s="5" t="n"/>
+      <c r="D16" s="5" t="n"/>
+      <c r="E16" s="5" t="n"/>
+      <c r="F16" s="5" t="n"/>
+      <c r="G16" s="5" t="n"/>
+      <c r="H16" s="14">
+        <f>SUM(H2:H14)</f>
+        <v>845.9</v>
+      </c>
+      <c r="I16" s="5" t="n"/>
+      <c r="J16" s="5" t="n"/>
+      <c r="K16" s="5" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K13"/>
+  <autoFilter ref="A1:K14"/>
   <dataValidations count="1">
-    <dataValidation sqref="D2:D13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose one of: to buy, ordered, owned" type="list">
+    <dataValidation sqref="D2:D14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose one of: to buy, ordered, owned" type="list">
       <formula1>"to buy,ordered,owned"</formula1>
     </dataValidation>
   </dataValidations>
@@ -9981,7 +10172,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J6" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>